<commit_message>
chore: checkpoint current state before JOBS UI review
</commit_message>
<xml_diff>
--- a/MAIN_SERVER/templates/불량대책서_샘플_종결본_v2.xlsx
+++ b/MAIN_SERVER/templates/불량대책서_샘플_종결본_v2.xlsx
@@ -12,21 +12,21 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="부품 검토자료" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="reply_containment_scope">'대책서'!$B$21</definedName>
-    <definedName name="reply_containment">'대책서'!$B$22</definedName>
-    <definedName name="reply_root_cause_label">'대책서'!$B$25</definedName>
-    <definedName name="reply_root_cause">'대책서'!$B$26</definedName>
-    <definedName name="reply_escape_cause">'대책서'!$B$28</definedName>
-    <definedName name="reply_prevention">'대책서'!$B$31</definedName>
-    <definedName name="reply_verify_period">'검증'!$B$5</definedName>
-    <definedName name="reply_verify_recipe">'검증'!$D$5</definedName>
-    <definedName name="reply_verify_inspected">'검증'!$E$5</definedName>
-    <definedName name="reply_verify_defective">'검증'!$F$5</definedName>
-    <definedName name="reply_verify_status">'검증'!$H$5</definedName>
-    <definedName name="reply_verify_note">'검증'!$B$6</definedName>
-    <definedName name="reply_closed_at">'검증'!$F$8</definedName>
-    <definedName name="reply_closure_note">'검증'!$B$9</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'대책서'!$A$1:$L$42</definedName>
+    <definedName name="reply_containment_scope">'대책서'!$C$18</definedName>
+    <definedName name="reply_containment">'대책서'!$C$19</definedName>
+    <definedName name="reply_root_cause_label">'대책서'!$C$20</definedName>
+    <definedName name="reply_root_cause">'대책서'!$C$21</definedName>
+    <definedName name="reply_escape_cause">'대책서'!$C$22</definedName>
+    <definedName name="reply_prevention">'대책서'!$C$23</definedName>
+    <definedName name="reply_verify_period">'대책서'!$C$25</definedName>
+    <definedName name="reply_verify_recipe">'대책서'!$E$25</definedName>
+    <definedName name="reply_verify_inspected">'대책서'!$G$25</definedName>
+    <definedName name="reply_verify_defective">'대책서'!$I$25</definedName>
+    <definedName name="reply_verify_status">'대책서'!$K$25</definedName>
+    <definedName name="reply_verify_note">'대책서'!$C$27</definedName>
+    <definedName name="reply_closed_at">'대책서'!$E$28</definedName>
+    <definedName name="reply_closure_note">'대책서'!$C$29</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'대책서'!$A$1:$L$30</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'불량 근거'!$A$1:$E$26</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'부품 검토자료'!$A$1:$F$21</definedName>
   </definedNames>
@@ -40,7 +40,7 @@
     <numFmt numFmtId="164" formatCode="0.0&quot;배&quot;"/>
     <numFmt numFmtId="165" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="41">
+  <fonts count="54">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -273,8 +273,80 @@
       <color rgb="0080601B"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00243D5B"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="00262626"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00243D5B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00262626"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00243D5B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="00262626"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00262626"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="0069727D"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="0069727D"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="00516276"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="0069727D"/>
+      <sz val="7.5"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00243D5B"/>
+      <sz val="17"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00243D5B"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -346,8 +418,13 @@
         <fgColor rgb="00F5F7FA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F3F5"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="14">
+  <borders count="32">
     <border>
       <left/>
       <right/>
@@ -487,11 +564,199 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BCC3CC"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="00BCC3CC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BCC3CC"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BCC3CC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BCC3CC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BCC3CC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BCC3CC"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="00BCC3CC"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BCC3CC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BCC3CC"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BCC3CC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BCC3CC"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BCC3CC"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BCC3CC"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BCC3CC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BCC3CC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BCC3CC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BCC3CC"/>
+      </right>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BCC3CC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BCC3CC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BCC3CC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BCC3CC"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BCC3CC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BCC3CC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BCC3CC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BCC3CC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BCC3CC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BCC3CC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BCC3CC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BCC3CC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BCC3CC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BCC3CC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BCC3CC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BCC3CC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BCC3CC"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BCC3CC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="156">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -689,7 +954,7 @@
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="37" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -736,11 +1001,176 @@
     <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="41" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="42" fillId="10" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="42" fillId="10" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="15" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="44" fillId="10" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="15" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="10" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="47" fillId="10" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="10" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="42" fillId="8" borderId="23" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="25" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="30" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="31" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="10" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="8" borderId="23" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="26" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="27" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="23" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="8" borderId="23" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="44" fillId="10" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="44" fillId="7" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="45" fillId="15" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="8" borderId="23" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="23" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="23" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="8" borderId="23" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="47" fillId="7" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="10" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="6">
     <dxf>
       <font>
         <b val="1"/>
@@ -771,6 +1201,39 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFF4D7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00216348"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00EEF5F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C2A2A"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F9EEEE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="0080601B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF9EB"/>
         </patternFill>
       </fill>
     </dxf>
@@ -853,14 +1316,154 @@
     <author>User</author>
   </authors>
   <commentList>
-    <comment ref="C16" authorId="0" shapeId="0">
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>부품 식별자: CAP</t>
+      </text>
+    </comment>
+    <comment ref="C6" authorId="0" shapeId="0">
+      <text>
+        <t>제조사 P/N·정격·공급사 (이전 v2)
+일치 · Contoso CX-0603X7R104K100
+정격 0.10µF ±10% 100V X7R 0603 · 공급사 Northwind Traders
+자세한 비교는 「부품 검토자료」 참조.</t>
+      </text>
+    </comment>
+    <comment ref="C7" authorId="0" shapeId="0">
+      <text>
+        <t>시스템은 배정 대기만 초기 기입합니다. 실제 주관 담당자는 관리자가 작성합니다.</t>
+      </text>
+    </comment>
+    <comment ref="J7" authorId="0" shapeId="0">
+      <text>
+        <t>시스템은 담당자 입력만 초기 기입합니다. 실제 협조 부서는 관리자가 작성합니다.</t>
+      </text>
+    </comment>
+    <comment ref="A9" authorId="0" shapeId="0">
+      <text>
+        <t>문서 상태와 회신 기한은 시스템이 ISSUED / 담당자 입력으로 초기화하며 이후 관리자가 갱신합니다. Job 상태 또는 DB의 메일 전송 상태와 별개입니다.</t>
+      </text>
+    </comment>
+    <comment ref="A12" authorId="0" shapeId="0">
+      <text>
+        <t>시스템 자동 기입. 발행 검사 시각까지 동일 Job의 검사 완료 Unit 수 × 해당 부품 슬롯 수입니다. requested_quantity(목표 PASS 수량)가 아닙니다.</t>
+      </text>
+    </comment>
+    <comment ref="D12" authorId="0" shapeId="0">
+      <text>
+        <t>시스템 자동 기입. 동일 Job·부품·불량 유형의 production.unit_defects 기록 수입니다. 불량 Unit 수와 다를 수 있습니다.</t>
+      </text>
+    </comment>
+    <comment ref="J12" authorId="0" shapeId="0">
+      <text>
+        <t>자동 계산. 관리자가 아래 검증 검사 수량·불량 수량을 입력하면 PPM을 계산합니다. 검사 시스템에서 재집계해 자동 채우는 값은 아닙니다.</t>
+      </text>
+    </comment>
+    <comment ref="C14" authorId="0" shapeId="0">
+      <text>
+        <t>발행 시점 전체 슬롯 분포: CAP-02 8건 · CAP-04 5건
+전체 분포는 불량 근거 시트에 자동 기입됩니다.</t>
+      </text>
+    </comment>
+    <comment ref="C15" authorId="0" shapeId="0">
+      <text>
+        <t>상세 원문 (이전 v2)
+확정 불량 1건을 기준으로 즉시 발행했다. 발행 시점까지 동일 Job·부품·유형은 16건이며 CAP-02·CAP-04에 13건이 기록됐다. 원인은 자동 추정하지 않으며 담당자가 검사 이미지와 데이터시트 품질 기준을 확인한다.</t>
+      </text>
+    </comment>
+    <comment ref="C19" authorId="0" shapeId="0">
+      <text>
+        <t>상세 원문 (이전 v2)
+08-19 10:20  CAP-02·CAP-04 슬롯 정지, 생산팀장 승인(구두 10:15 · 결재 10:40).
+08-16 이후 생산분 전량 출하 보류 — job 7112~7139 / unit 10388~10604 (2,500대).
+전수 AOI 재검에서 9건 추가 검출, 누적 25건 / 24대 격리. 고객 통보 대상 아님(출하 전).
+배치 하강속도만 mock-v2 값으로 되돌린 임시 레시피 mock-v3h 적용 후 10:50 생산 재개. 08-19 18:00 기준 재발 없음.</t>
+      </text>
+    </comment>
+    <comment ref="C20" authorId="0" shapeId="0">
       <text>
         <t>② 발생 원인의 핵심을 한 줄로 요약합니다.</t>
       </text>
     </comment>
     <comment ref="C21" authorId="0" shapeId="0">
       <text>
-        <t>④의 상세 대책을 한두 문장으로 요약합니다. 상세 내용 변경 시 함께 갱신하세요.</t>
+        <t>상세 원문 (이전 v2)
+mock-v3 에서 배치 하강속도(18 → 32 mm/s)와 그리퍼 파지력(3.0 → 4.0 N)을 함께 올렸다.
+CAP-02·CAP-04 는 보드 지지 핀에서 가장 먼 위치라 착지 충격 시 국부 굽힘이 가장 크다. 설비팀 로그에서 두 슬롯 피크력이 다른 CAP 슬롯의 1.7배(6.8N vs 4.0N).
+mock-v3h 로 되돌린 뒤 재발이 멈춘 것으로 검증했다(가설 아님). 불량 25건이 입고 Lot 4개에 고르게 분포해 부품 Lot 요인은 배제한다.</t>
+      </text>
+    </comment>
+    <comment ref="C22" authorId="0" shapeId="0">
+      <text>
+        <t>상세 원문 (이전 v2)
+인라인 AOI 판정 기준이 단자 들뜸과 외관 결손만 보고 있어 미세 굽힘 크랙을 걸러내지 못했다.
+「부품 검토자료」의 MLCC 항목은 '크랙 의심 Lot 단면 또는 비파괴 검사'를 요구하지만, 현재 인라인에는 해당 항목이 없고 단면 검사는 주 1회 샘플로만 돌고 있었다.
+그 결과 08-16 생산분에 이미 크랙이 있었으나 08-18 16:30 임계 초과 시점까지 검출되지 않았다.</t>
+      </text>
+    </comment>
+    <comment ref="C23" authorId="0" shapeId="0">
+      <text>
+        <t>상세 원문 (이전 v2)
+영구대책 ① 레시피 — 하강속도 20 mm/s, 파지력 3.2 N 으로 확정한 mock-v4 적용. 변경관리 ECN-2608-114 승인 08-21, 적용 08-29.
+영구대책 ② 설비 — CAP-02·CAP-04 에 보드 지지 핀 2개 추가(설비팀, 08-28 완료). 수평전개로 IND-01·IND-02 에도 함께 적용했다.
+부품 교체는 하지 않는다. 「부품 검토자료」 후보 2종 모두 표준 단자라 굽힘 크랙 개선 근거가 없다.
+기존 대책 요약
+하강속도·파지력 조정, 보드 지지 핀 추가. 부품 교체 없음.</t>
+      </text>
+    </comment>
+    <comment ref="F26" authorId="0" shapeId="0">
+      <text>
+        <t>자동 계산. 검증 불량 수량 ÷ 검증 검사 수량. 검증 수량은 부품 검사 건수 기준입니다.</t>
+      </text>
+    </comment>
+    <comment ref="C27" authorId="0" shapeId="0">
+      <text>
+        <t>상세 원문 (이전 v2)
+CRACK 3건 / 24,500건 = 122 PPM. 기준 400 PPM 의 0.31배이고 최소 검사 건수를 충족한다. 대책 전 1,280 PPM 대비 10.5배 개선, CAP-02·CAP-04 집중도도 해소됐다.</t>
+      </text>
+    </comment>
+    <comment ref="C29" authorId="0" shapeId="0">
+      <text>
+        <t>상세 원문 (이전 v2)
+영구대책 적용과 효과가 확인되어 종결한다. 잔여 위험 — 지지 핀은 현재 보드 리비전 기준이라 레이아웃 변경 시 재검토가 필요하다. AOI 기준 보완은 별건 QA-PROC-2609-003 으로 이관.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>User</author>
+  </authors>
+  <commentList>
+    <comment ref="B9" authorId="0" shapeId="0">
+      <text>
+        <t>현행 데이터시트 대조로 공통 기준을 포함했습니다.
+이전 샘플 문구:
+외관/단자, 0603·100V·X7R 확인, LCR·절연저항 샘플</t>
+      </text>
+    </comment>
+    <comment ref="E9" authorId="0" shapeId="0">
+      <text>
+        <t>현행 데이터시트 대조로 공통 기준을 포함했습니다.
+이전 샘플 문구:
+크랙/IR 저하는 Lot·패널 위치별 격리, 보드 굴곡·분리·프로브 지지 조건을 재현하고 공정 조건 수정</t>
+      </text>
+    </comment>
+    <comment ref="B10" authorId="0" shapeId="0">
+      <text>
+        <t>현행 데이터시트 대조로 공통 기준을 포함했습니다.
+이전 샘플 문구:
+land/reflow 준수; panel depanel·ICT probe·connector 체결 시 board support로 보드 굽힘 억제</t>
+      </text>
+    </comment>
+    <comment ref="B11" authorId="0" shapeId="0">
+      <text>
+        <t>현행 데이터시트 대조로 공통 기준을 포함했습니다.
+이전 샘플 문구:
+AOI, LCR/IR; crack 의심 Lot 단면 또는 비파괴 검사</t>
       </text>
     </comment>
   </commentList>
@@ -1214,984 +1817,785 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001F3864"/>
+    <tabColor rgb="00243D5B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7.3" customWidth="1" min="1" max="1"/>
-    <col width="7.3" customWidth="1" min="2" max="2"/>
-    <col width="7.3" customWidth="1" min="3" max="3"/>
-    <col width="7.3" customWidth="1" min="4" max="4"/>
-    <col width="7.3" customWidth="1" min="5" max="5"/>
-    <col width="7.3" customWidth="1" min="6" max="6"/>
-    <col width="7.3" customWidth="1" min="7" max="7"/>
-    <col width="7.3" customWidth="1" min="8" max="8"/>
-    <col width="7.3" customWidth="1" min="9" max="9"/>
-    <col width="7.3" customWidth="1" min="10" max="10"/>
-    <col width="7.3" customWidth="1" min="11" max="11"/>
-    <col width="7.3" customWidth="1" min="12" max="12"/>
+    <col width="6.4" customWidth="1" min="1" max="1"/>
+    <col width="6.4" customWidth="1" min="2" max="2"/>
+    <col width="6.4" customWidth="1" min="3" max="3"/>
+    <col width="6.4" customWidth="1" min="4" max="4"/>
+    <col width="6.4" customWidth="1" min="5" max="5"/>
+    <col width="6.4" customWidth="1" min="6" max="6"/>
+    <col width="6.4" customWidth="1" min="7" max="7"/>
+    <col width="6.4" customWidth="1" min="8" max="8"/>
+    <col width="6.4" customWidth="1" min="9" max="9"/>
+    <col width="6.4" customWidth="1" min="10" max="10"/>
+    <col width="6.4" customWidth="1" min="11" max="11"/>
+    <col width="6.4" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="44" t="inlineStr">
-        <is>
-          <t>불량 대책서</t>
-        </is>
-      </c>
-      <c r="J1" s="45" t="inlineStr">
-        <is>
-          <t>v2  /  검토용</t>
-        </is>
-      </c>
-      <c r="K1" s="46" t="n"/>
-      <c r="L1" s="46" t="n"/>
-    </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="47" t="inlineStr">
-        <is>
-          <t>01  현황 · 초동 조치     /     02  원인 · 대책 · 검증 · 종결</t>
-        </is>
-      </c>
-      <c r="J2" s="48" t="inlineStr">
-        <is>
-          <t>CAP</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="49" t="inlineStr">
+    <row r="1" ht="17" customHeight="1">
+      <c r="A1" s="89" t="inlineStr">
+        <is>
+          <t>불 량 대 책 서</t>
+        </is>
+      </c>
+      <c r="G1" s="118" t="inlineStr">
+        <is>
+          <t>작성</t>
+        </is>
+      </c>
+      <c r="H1" s="119" t="n"/>
+      <c r="I1" s="118" t="inlineStr">
+        <is>
+          <t>검토</t>
+        </is>
+      </c>
+      <c r="J1" s="119" t="n"/>
+      <c r="K1" s="118" t="inlineStr">
+        <is>
+          <t>승인</t>
+        </is>
+      </c>
+      <c r="L1" s="119" t="n"/>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="G2" s="120" t="n"/>
+      <c r="H2" s="121" t="n"/>
+      <c r="I2" s="120" t="n"/>
+      <c r="J2" s="121" t="n"/>
+      <c r="K2" s="120" t="n"/>
+      <c r="L2" s="121" t="n"/>
+    </row>
+    <row r="3" ht="15" customHeight="1">
+      <c r="G3" s="122" t="n"/>
+      <c r="H3" s="123" t="n"/>
+      <c r="I3" s="122" t="n"/>
+      <c r="J3" s="123" t="n"/>
+      <c r="K3" s="122" t="n"/>
+      <c r="L3" s="123" t="n"/>
+    </row>
+    <row r="4" ht="12" customHeight="1">
+      <c r="A4" s="124" t="inlineStr">
+        <is>
+          <t>시스템 자동 기입 · 발행 시점 고정  |  담당·기한·문서 상태는 관리자 갱신</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="118" t="inlineStr">
         <is>
           <t>문서번호</t>
         </is>
       </c>
-      <c r="B3" s="46" t="n"/>
-      <c r="C3" s="50" t="inlineStr">
+      <c r="B5" s="119" t="n"/>
+      <c r="C5" s="125" t="inlineStr">
         <is>
           <t>QA-CAP-CRACK-20260819-001</t>
         </is>
       </c>
-      <c r="H3" s="49" t="inlineStr">
+      <c r="D5" s="126" t="n"/>
+      <c r="E5" s="126" t="n"/>
+      <c r="F5" s="126" t="n"/>
+      <c r="G5" s="119" t="n"/>
+      <c r="H5" s="118" t="inlineStr">
         <is>
           <t>발행일시</t>
         </is>
       </c>
-      <c r="I3" s="46" t="n"/>
-      <c r="J3" s="51" t="inlineStr">
+      <c r="I5" s="119" t="n"/>
+      <c r="J5" s="127" t="inlineStr">
         <is>
           <t>2026-08-19 09:00:00</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="49" t="inlineStr">
+      <c r="K5" s="126" t="n"/>
+      <c r="L5" s="119" t="n"/>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="118" t="inlineStr">
         <is>
           <t>대상 부품</t>
         </is>
       </c>
-      <c r="B4" s="46" t="n"/>
-      <c r="C4" s="50" t="inlineStr">
+      <c r="B6" s="119" t="n"/>
+      <c r="C6" s="125" t="inlineStr">
         <is>
           <t>CAP  (MLCC)</t>
         </is>
       </c>
-      <c r="H4" s="49" t="inlineStr">
+      <c r="D6" s="126" t="n"/>
+      <c r="E6" s="126" t="n"/>
+      <c r="F6" s="126" t="n"/>
+      <c r="G6" s="119" t="n"/>
+      <c r="H6" s="118" t="inlineStr">
         <is>
           <t>불량 유형</t>
         </is>
       </c>
-      <c r="I4" s="46" t="n"/>
-      <c r="J4" s="51" t="inlineStr">
+      <c r="I6" s="119" t="n"/>
+      <c r="J6" s="127" t="inlineStr">
         <is>
           <t>CRACK</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="49" t="inlineStr">
+      <c r="K6" s="126" t="n"/>
+      <c r="L6" s="119" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="118" t="inlineStr">
         <is>
           <t>주관 담당</t>
         </is>
       </c>
-      <c r="B5" s="46" t="n"/>
-      <c r="C5" s="50" t="inlineStr">
+      <c r="B7" s="119" t="n"/>
+      <c r="C7" s="128" t="inlineStr">
         <is>
           <t>품질보증팀 김OO</t>
         </is>
       </c>
-      <c r="H5" s="49" t="inlineStr">
+      <c r="D7" s="129" t="n"/>
+      <c r="E7" s="129" t="n"/>
+      <c r="F7" s="129" t="n"/>
+      <c r="G7" s="130" t="n"/>
+      <c r="H7" s="118" t="inlineStr">
         <is>
           <t>협조 부서</t>
         </is>
       </c>
-      <c r="I5" s="46" t="n"/>
-      <c r="J5" s="51" t="inlineStr">
+      <c r="I7" s="119" t="n"/>
+      <c r="J7" s="131" t="inlineStr">
         <is>
           <t>설비팀 · 생산팀 · 구매</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="49" t="inlineStr">
+      <c r="K7" s="129" t="n"/>
+      <c r="L7" s="130" t="n"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="118" t="inlineStr">
         <is>
           <t>발행 대상</t>
         </is>
       </c>
-      <c r="B6" s="46" t="n"/>
-      <c r="C6" s="50" t="inlineStr">
+      <c r="B8" s="119" t="n"/>
+      <c r="C8" s="125" t="inlineStr">
         <is>
           <t>Job 7112 · Unit 10412 · CAP-02</t>
         </is>
       </c>
-      <c r="H6" s="49" t="inlineStr">
+      <c r="D8" s="126" t="n"/>
+      <c r="E8" s="126" t="n"/>
+      <c r="F8" s="126" t="n"/>
+      <c r="G8" s="119" t="n"/>
+      <c r="H8" s="118" t="inlineStr">
         <is>
           <t>검사 시각</t>
         </is>
       </c>
-      <c r="I6" s="46" t="n"/>
-      <c r="J6" s="51" t="inlineStr">
+      <c r="I8" s="119" t="n"/>
+      <c r="J8" s="127" t="inlineStr">
         <is>
           <t>2026-08-18 16:30:12</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CLOSED     ①~④ 작성 완료   ⑤ 효과 검증 · ⑥ 종결은 「대책서」 2쪽</t>
-        </is>
-      </c>
-      <c r="B7" s="46" t="n"/>
-      <c r="C7" s="46" t="n"/>
-      <c r="D7" s="46" t="n"/>
-      <c r="E7" s="46" t="n"/>
-      <c r="F7" s="46" t="n"/>
-      <c r="G7" s="46" t="n"/>
-      <c r="H7" s="46" t="n"/>
-      <c r="I7" s="46" t="n"/>
-      <c r="J7" s="46" t="n"/>
-      <c r="K7" s="46" t="n"/>
-      <c r="L7" s="46" t="n"/>
-    </row>
-    <row r="8" ht="8" customHeight="1">
-      <c r="A8" s="52" t="n"/>
-      <c r="B8" s="52" t="n"/>
-      <c r="C8" s="52" t="n"/>
-      <c r="D8" s="52" t="n"/>
-      <c r="E8" s="52" t="n"/>
-      <c r="F8" s="52" t="n"/>
-      <c r="G8" s="52" t="n"/>
-      <c r="H8" s="52" t="n"/>
-      <c r="I8" s="52" t="n"/>
-      <c r="J8" s="52" t="n"/>
-      <c r="K8" s="52" t="n"/>
-      <c r="L8" s="52" t="n"/>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="53" t="inlineStr">
-        <is>
-          <t>불량 현황  |  발행 시점과 대책 적용 후 비교</t>
-        </is>
-      </c>
-      <c r="B9" s="54" t="n"/>
-      <c r="C9" s="54" t="n"/>
-      <c r="D9" s="54" t="n"/>
-      <c r="E9" s="54" t="n"/>
-      <c r="F9" s="54" t="n"/>
-      <c r="G9" s="54" t="n"/>
-      <c r="H9" s="54" t="n"/>
-      <c r="I9" s="54" t="n"/>
-      <c r="J9" s="54" t="n"/>
-      <c r="K9" s="54" t="n"/>
-      <c r="L9" s="54" t="n"/>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="49" t="inlineStr">
+      <c r="K8" s="126" t="n"/>
+      <c r="L8" s="119" t="n"/>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="132" t="inlineStr">
+        <is>
+          <t>상태  CLOSED  ·  ①~⑥ 작성 완료  ·  발행 기준: 확정 불량 1건</t>
+        </is>
+      </c>
+      <c r="B9" s="129" t="n"/>
+      <c r="C9" s="129" t="n"/>
+      <c r="D9" s="129" t="n"/>
+      <c r="E9" s="129" t="n"/>
+      <c r="F9" s="129" t="n"/>
+      <c r="G9" s="129" t="n"/>
+      <c r="H9" s="129" t="n"/>
+      <c r="I9" s="129" t="n"/>
+      <c r="J9" s="129" t="n"/>
+      <c r="K9" s="129" t="n"/>
+      <c r="L9" s="130" t="n"/>
+    </row>
+    <row r="10" ht="6" customHeight="1"/>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="118" t="inlineStr">
+        <is>
+          <t>부품 검사 수량</t>
+        </is>
+      </c>
+      <c r="B11" s="126" t="n"/>
+      <c r="C11" s="119" t="n"/>
+      <c r="D11" s="118" t="inlineStr">
+        <is>
+          <t>불량 건수</t>
+        </is>
+      </c>
+      <c r="E11" s="126" t="n"/>
+      <c r="F11" s="119" t="n"/>
+      <c r="G11" s="118" t="inlineStr">
+        <is>
+          <t>발행 PPM</t>
+        </is>
+      </c>
+      <c r="H11" s="126" t="n"/>
+      <c r="I11" s="119" t="n"/>
+      <c r="J11" s="118" t="inlineStr">
+        <is>
+          <t>검증 PPM(계산)</t>
+        </is>
+      </c>
+      <c r="K11" s="126" t="n"/>
+      <c r="L11" s="119" t="n"/>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="133" t="n">
+        <v>12500</v>
+      </c>
+      <c r="B12" s="126" t="n"/>
+      <c r="C12" s="119" t="n"/>
+      <c r="D12" s="133" t="n">
+        <v>16</v>
+      </c>
+      <c r="E12" s="126" t="n"/>
+      <c r="F12" s="119" t="n"/>
+      <c r="G12" s="133" t="n">
+        <v>1280</v>
+      </c>
+      <c r="H12" s="126" t="n"/>
+      <c r="I12" s="119" t="n"/>
+      <c r="J12" s="134">
+        <f>IF(AND(ISNUMBER(G25),ISNUMBER(I25),G25&gt;0),I25/G25*1000000,"")</f>
+        <v/>
+      </c>
+      <c r="K12" s="135" t="n"/>
+      <c r="L12" s="136" t="n"/>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="118" t="inlineStr">
+        <is>
+          <t>집계 기간</t>
+        </is>
+      </c>
+      <c r="B13" s="119" t="n"/>
+      <c r="C13" s="127" t="inlineStr">
+        <is>
+          <t>2026-08-12 ~ 08-19  (7일 / ROLLING)</t>
+        </is>
+      </c>
+      <c r="D13" s="126" t="n"/>
+      <c r="E13" s="126" t="n"/>
+      <c r="F13" s="126" t="n"/>
+      <c r="G13" s="119" t="n"/>
+      <c r="H13" s="118" t="inlineStr">
+        <is>
+          <t>레시피</t>
+        </is>
+      </c>
+      <c r="I13" s="119" t="n"/>
+      <c r="J13" s="127" t="inlineStr">
+        <is>
+          <t>mock-v3</t>
+        </is>
+      </c>
+      <c r="K13" s="126" t="n"/>
+      <c r="L13" s="119" t="n"/>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="118" t="inlineStr">
+        <is>
+          <t>발생 위치</t>
+        </is>
+      </c>
+      <c r="B14" s="119" t="n"/>
+      <c r="C14" s="127" t="inlineStr">
+        <is>
+          <t>CAP-02 (발행 대상)
+전체 분포: 불량 근거</t>
+        </is>
+      </c>
+      <c r="D14" s="126" t="n"/>
+      <c r="E14" s="126" t="n"/>
+      <c r="F14" s="119" t="n"/>
+      <c r="G14" s="118" t="inlineStr">
+        <is>
+          <t>완제품 영향</t>
+        </is>
+      </c>
+      <c r="H14" s="119" t="n"/>
+      <c r="I14" s="127" t="inlineStr">
+        <is>
+          <t>2,500대 중 15대 (0.60%)</t>
+        </is>
+      </c>
+      <c r="J14" s="126" t="n"/>
+      <c r="K14" s="126" t="n"/>
+      <c r="L14" s="119" t="n"/>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="118" t="inlineStr">
+        <is>
+          <t>자동 분석</t>
+        </is>
+      </c>
+      <c r="B15" s="119" t="n"/>
+      <c r="C15" s="127" t="inlineStr">
+        <is>
+          <t>확정 불량 1건으로 발행. 동일 Job·부품·유형 누적 16건 중 CAP-02·CAP-04에 13건 집중. 원인은 자동 추정하지 않으며 담당자가 이미지·품질 기준을 확인.</t>
+        </is>
+      </c>
+      <c r="D15" s="126" t="n"/>
+      <c r="E15" s="126" t="n"/>
+      <c r="F15" s="126" t="n"/>
+      <c r="G15" s="126" t="n"/>
+      <c r="H15" s="126" t="n"/>
+      <c r="I15" s="126" t="n"/>
+      <c r="J15" s="126" t="n"/>
+      <c r="K15" s="126" t="n"/>
+      <c r="L15" s="119" t="n"/>
+    </row>
+    <row r="16" ht="6" customHeight="1"/>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="137" t="inlineStr">
+        <is>
+          <t>관리자 직접 작성  |  ①~⑥ 조치·원인·대책·검증·종결 (예시)</t>
+        </is>
+      </c>
+      <c r="B17" s="126" t="n"/>
+      <c r="C17" s="126" t="n"/>
+      <c r="D17" s="126" t="n"/>
+      <c r="E17" s="126" t="n"/>
+      <c r="F17" s="126" t="n"/>
+      <c r="G17" s="126" t="n"/>
+      <c r="H17" s="126" t="n"/>
+      <c r="I17" s="126" t="n"/>
+      <c r="J17" s="126" t="n"/>
+      <c r="K17" s="126" t="n"/>
+      <c r="L17" s="119" t="n"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="118" t="inlineStr">
+        <is>
+          <t>① 초동 조치</t>
+        </is>
+      </c>
+      <c r="B18" s="138" t="n"/>
+      <c r="C18" s="139" t="inlineStr">
+        <is>
+          <t>■ 생산 중단    ■ 출하 보류    ■ 재고 선별    □ 고객 통보    □ 설비 정지</t>
+        </is>
+      </c>
+      <c r="D18" s="129" t="n"/>
+      <c r="E18" s="129" t="n"/>
+      <c r="F18" s="129" t="n"/>
+      <c r="G18" s="129" t="n"/>
+      <c r="H18" s="129" t="n"/>
+      <c r="I18" s="129" t="n"/>
+      <c r="J18" s="129" t="n"/>
+      <c r="K18" s="129" t="n"/>
+      <c r="L18" s="130" t="n"/>
+    </row>
+    <row r="19" ht="58" customHeight="1">
+      <c r="A19" s="140" t="n"/>
+      <c r="B19" s="141" t="n"/>
+      <c r="C19" s="128" t="inlineStr">
+        <is>
+          <t>08-19 10:20 CAP-02·CAP-04 정지(생산팀장 승인). 08-16 이후 Job 7112~7139 / Unit 10388~10604, 2,500대 출하 보류.
+전수 재검 9건 추가, 누적 25건 / 24대 격리. mock-v3h 적용 후 10:50 생산 재개, 당일 18:00 재발 없음. 출하 전으로 고객 통보 제외.</t>
+        </is>
+      </c>
+      <c r="D19" s="129" t="n"/>
+      <c r="E19" s="129" t="n"/>
+      <c r="F19" s="129" t="n"/>
+      <c r="G19" s="129" t="n"/>
+      <c r="H19" s="129" t="n"/>
+      <c r="I19" s="129" t="n"/>
+      <c r="J19" s="129" t="n"/>
+      <c r="K19" s="129" t="n"/>
+      <c r="L19" s="130" t="n"/>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="118" t="inlineStr">
+        <is>
+          <t>② 발생 원인</t>
+        </is>
+      </c>
+      <c r="B20" s="138" t="n"/>
+      <c r="C20" s="142" t="inlineStr">
+        <is>
+          <t>배치 하강속도 상향 + 지지 핀 최원거리 슬롯</t>
+        </is>
+      </c>
+      <c r="D20" s="129" t="n"/>
+      <c r="E20" s="129" t="n"/>
+      <c r="F20" s="129" t="n"/>
+      <c r="G20" s="129" t="n"/>
+      <c r="H20" s="129" t="n"/>
+      <c r="I20" s="129" t="n"/>
+      <c r="J20" s="129" t="n"/>
+      <c r="K20" s="129" t="n"/>
+      <c r="L20" s="130" t="n"/>
+    </row>
+    <row r="21" ht="56" customHeight="1">
+      <c r="A21" s="140" t="n"/>
+      <c r="B21" s="141" t="n"/>
+      <c r="C21" s="128" t="inlineStr">
+        <is>
+          <t>mock-v3 하강속도 18→32 mm/s·파지력 3.0→4.0 N 상향과 지지 핀에서 먼 슬롯의 보드 굽힘이 원인.
+CAP-02·CAP-04 피크력 6.8 N(타 슬롯 4.0 N, 1.7배). mock-v3h 복귀 후 재발 중단. 입고 Lot 4개에 고르게 발생해 Lot 요인 배제.</t>
+        </is>
+      </c>
+      <c r="D21" s="129" t="n"/>
+      <c r="E21" s="129" t="n"/>
+      <c r="F21" s="129" t="n"/>
+      <c r="G21" s="129" t="n"/>
+      <c r="H21" s="129" t="n"/>
+      <c r="I21" s="129" t="n"/>
+      <c r="J21" s="129" t="n"/>
+      <c r="K21" s="129" t="n"/>
+      <c r="L21" s="130" t="n"/>
+    </row>
+    <row r="22" ht="53" customHeight="1">
+      <c r="A22" s="118" t="inlineStr">
+        <is>
+          <t>③ 유출 원인</t>
+        </is>
+      </c>
+      <c r="B22" s="119" t="n"/>
+      <c r="C22" s="128" t="inlineStr">
+        <is>
+          <t>인라인 AOI는 단자 들뜸·외관 결손만 판정해 미세 굽힘 크랙을 검출하지 못함. 품질 기준의 단면·비파괴 검사는 인라인에 없고 주 1회 샘플 검사만 시행.
+08-16 생산분의 크랙을 08-18 16:30에 검출.</t>
+        </is>
+      </c>
+      <c r="D22" s="129" t="n"/>
+      <c r="E22" s="129" t="n"/>
+      <c r="F22" s="129" t="n"/>
+      <c r="G22" s="129" t="n"/>
+      <c r="H22" s="129" t="n"/>
+      <c r="I22" s="129" t="n"/>
+      <c r="J22" s="129" t="n"/>
+      <c r="K22" s="129" t="n"/>
+      <c r="L22" s="130" t="n"/>
+    </row>
+    <row r="23" ht="55" customHeight="1">
+      <c r="A23" s="118" t="inlineStr">
+        <is>
+          <t>④ 재발방지
+대책</t>
+        </is>
+      </c>
+      <c r="B23" s="119" t="n"/>
+      <c r="C23" s="128" t="inlineStr">
+        <is>
+          <t>mock-v4: 하강속도 20 mm/s·파지력 3.2 N 적용(ECN-2608-114 승인 08-21, 적용 08-29).
+CAP-02·CAP-04 지지 핀 2개 추가(설비팀, 08-28), IND-01·IND-02 수평전개. 후보 2종은 표준 단자로 크랙 개선 근거가 없어 부품 교체 제외.</t>
+        </is>
+      </c>
+      <c r="D23" s="129" t="n"/>
+      <c r="E23" s="129" t="n"/>
+      <c r="F23" s="129" t="n"/>
+      <c r="G23" s="129" t="n"/>
+      <c r="H23" s="129" t="n"/>
+      <c r="I23" s="129" t="n"/>
+      <c r="J23" s="129" t="n"/>
+      <c r="K23" s="129" t="n"/>
+      <c r="L23" s="130" t="n"/>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="118" t="inlineStr">
+        <is>
+          <t>⑤ 효과 검증</t>
+        </is>
+      </c>
+      <c r="B24" s="138" t="n"/>
+      <c r="C24" s="118" t="inlineStr">
+        <is>
+          <t>검증 기간</t>
+        </is>
+      </c>
+      <c r="D24" s="119" t="n"/>
+      <c r="E24" s="118" t="inlineStr">
+        <is>
+          <t>적용 레시피</t>
+        </is>
+      </c>
+      <c r="F24" s="119" t="n"/>
+      <c r="G24" s="118" t="inlineStr">
         <is>
           <t>검사 수량</t>
         </is>
       </c>
-      <c r="B10" s="46" t="n"/>
-      <c r="C10" s="46" t="n"/>
-      <c r="D10" s="49" t="inlineStr">
+      <c r="H24" s="119" t="n"/>
+      <c r="I24" s="118" t="inlineStr">
         <is>
           <t>불량 수량</t>
         </is>
       </c>
-      <c r="E10" s="46" t="n"/>
-      <c r="F10" s="46" t="n"/>
-      <c r="G10" s="49" t="inlineStr">
-        <is>
-          <t>발행 시점 PPM</t>
-        </is>
-      </c>
-      <c r="H10" s="46" t="n"/>
-      <c r="I10" s="46" t="n"/>
-      <c r="J10" s="49" t="inlineStr">
-        <is>
-          <t>검증 PPM</t>
-        </is>
-      </c>
-      <c r="K10" s="46" t="n"/>
-      <c r="L10" s="46" t="n"/>
-    </row>
-    <row r="11" ht="36" customHeight="1">
-      <c r="A11" s="55" t="n">
-        <v>12500</v>
-      </c>
-      <c r="B11" s="46" t="n"/>
-      <c r="C11" s="46" t="n"/>
-      <c r="D11" s="55" t="n">
-        <v>16</v>
-      </c>
-      <c r="E11" s="46" t="n"/>
-      <c r="F11" s="46" t="n"/>
-      <c r="G11" s="55" t="n">
-        <v>1280</v>
-      </c>
-      <c r="H11" s="46" t="n"/>
-      <c r="I11" s="46" t="n"/>
-      <c r="J11" s="55">
-        <f>IF(AND(ISNUMBER(F34),ISNUMBER(H34),F34&gt;0),H34/F34*1000000,"")</f>
+      <c r="J24" s="119" t="n"/>
+      <c r="K24" s="118" t="inlineStr">
+        <is>
+          <t>판정</t>
+        </is>
+      </c>
+      <c r="L24" s="119" t="n"/>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="143" t="n"/>
+      <c r="B25" s="144" t="n"/>
+      <c r="C25" s="145" t="inlineStr">
+        <is>
+          <t>08-29 ~ 09-12</t>
+        </is>
+      </c>
+      <c r="D25" s="130" t="n"/>
+      <c r="E25" s="145" t="inlineStr">
+        <is>
+          <t>mock-v4</t>
+        </is>
+      </c>
+      <c r="F25" s="130" t="n"/>
+      <c r="G25" s="146" t="n">
+        <v>24500</v>
+      </c>
+      <c r="H25" s="130" t="n"/>
+      <c r="I25" s="146" t="n">
+        <v>3</v>
+      </c>
+      <c r="J25" s="130" t="n"/>
+      <c r="K25" s="145" t="inlineStr">
+        <is>
+          <t>EFFECTIVE</t>
+        </is>
+      </c>
+      <c r="L25" s="130" t="n"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="143" t="n"/>
+      <c r="B26" s="144" t="n"/>
+      <c r="C26" s="118" t="inlineStr">
+        <is>
+          <t>불량률(자동 계산)</t>
+        </is>
+      </c>
+      <c r="D26" s="126" t="n"/>
+      <c r="E26" s="119" t="n"/>
+      <c r="F26" s="147">
+        <f>IF(AND(ISNUMBER(G25),ISNUMBER(I25),G25&gt;0),I25/G25,"")</f>
         <v/>
       </c>
-      <c r="K11" s="46" t="n"/>
-      <c r="L11" s="46" t="n"/>
-    </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="49" t="inlineStr">
-        <is>
-          <t>집계 기간</t>
-        </is>
-      </c>
-      <c r="B12" s="46" t="n"/>
-      <c r="C12" s="51" t="inlineStr">
-        <is>
-          <t>2026-08-12 ~ 08-19  (7일 / ROLLING)</t>
-        </is>
-      </c>
-      <c r="H12" s="49" t="inlineStr">
-        <is>
-          <t>레시피</t>
-        </is>
-      </c>
-      <c r="I12" s="46" t="n"/>
-      <c r="J12" s="51" t="inlineStr">
-        <is>
-          <t>mock-v3</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="49" t="inlineStr">
-        <is>
-          <t>발생 위치</t>
-        </is>
-      </c>
-      <c r="B13" s="46" t="n"/>
-      <c r="C13" s="51" t="inlineStr">
-        <is>
-          <t>CAP-02 8건 · CAP-04 5건</t>
-        </is>
-      </c>
-      <c r="H13" s="49" t="inlineStr">
-        <is>
-          <t>발행 기준</t>
-        </is>
-      </c>
-      <c r="I13" s="46" t="n"/>
-      <c r="J13" s="51" t="inlineStr">
-        <is>
-          <t>확정 불량 1건</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="49" t="inlineStr">
-        <is>
-          <t>완제품 영향</t>
-        </is>
-      </c>
-      <c r="B14" s="46" t="n"/>
-      <c r="C14" s="51" t="inlineStr">
-        <is>
-          <t>2,500대 중 15대 (0.60%)</t>
-        </is>
-      </c>
-      <c r="F14" s="49" t="inlineStr">
-        <is>
-          <t>제조사 P/N</t>
-        </is>
-      </c>
-      <c r="G14" s="46" t="n"/>
-      <c r="H14" s="56" t="inlineStr">
-        <is>
-          <t>일치 · Contoso CX-0603X7R104K100
-정격 0.10µF ±10% 100V X7R 0603 · 공급사 Northwind Traders</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="56" customHeight="1">
-      <c r="A15" s="49" t="inlineStr">
-        <is>
-          <t>자동 분석</t>
-        </is>
-      </c>
-      <c r="B15" s="46" t="n"/>
-      <c r="C15" s="57" t="inlineStr">
-        <is>
-          <t>확정 불량 1건을 기준으로 즉시 발행했다. 발행 시점까지 동일 Job·부품·유형은 16건이며 CAP-02·CAP-04에 13건이 기록됐다. 원인은 자동 추정하지 않으며 담당자가 검사 이미지와 데이터시트 품질 기준을 확인한다.</t>
-        </is>
-      </c>
-      <c r="D15" s="46" t="n"/>
-      <c r="E15" s="46" t="n"/>
-      <c r="F15" s="46" t="n"/>
-      <c r="G15" s="46" t="n"/>
-      <c r="H15" s="46" t="n"/>
-      <c r="I15" s="46" t="n"/>
-      <c r="J15" s="46" t="n"/>
-      <c r="K15" s="46" t="n"/>
-      <c r="L15" s="46" t="n"/>
-    </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="49" t="inlineStr">
-        <is>
-          <t>핵심 원인</t>
-        </is>
-      </c>
-      <c r="B16" s="46" t="n"/>
-      <c r="C16" s="58" t="inlineStr">
-        <is>
-          <t>배치 하강속도 상향 + 지지 핀 최원거리 슬롯</t>
-        </is>
-      </c>
-      <c r="D16" s="59" t="n"/>
-      <c r="E16" s="59" t="n"/>
-      <c r="F16" s="59" t="n"/>
-      <c r="G16" s="59" t="n"/>
-      <c r="H16" s="59" t="n"/>
-      <c r="I16" s="59" t="n"/>
-      <c r="J16" s="59" t="n"/>
-      <c r="K16" s="59" t="n"/>
-      <c r="L16" s="59" t="n"/>
-    </row>
-    <row r="17" ht="8" customHeight="1">
-      <c r="A17" s="52" t="n"/>
-      <c r="B17" s="52" t="n"/>
-      <c r="C17" s="52" t="n"/>
-      <c r="D17" s="52" t="n"/>
-      <c r="E17" s="52" t="n"/>
-      <c r="F17" s="52" t="n"/>
-      <c r="G17" s="52" t="n"/>
-      <c r="H17" s="52" t="n"/>
-      <c r="I17" s="52" t="n"/>
-      <c r="J17" s="52" t="n"/>
-      <c r="K17" s="52" t="n"/>
-      <c r="L17" s="52" t="n"/>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="53" t="inlineStr">
-        <is>
-          <t>① 초동 조치  |  확산 방지와 영향 범위</t>
-        </is>
-      </c>
-      <c r="B18" s="54" t="n"/>
-      <c r="C18" s="54" t="n"/>
-      <c r="D18" s="54" t="n"/>
-      <c r="E18" s="54" t="n"/>
-      <c r="F18" s="54" t="n"/>
-      <c r="G18" s="54" t="n"/>
-      <c r="H18" s="54" t="n"/>
-      <c r="I18" s="54" t="n"/>
-      <c r="J18" s="54" t="n"/>
-      <c r="K18" s="54" t="n"/>
-      <c r="L18" s="54" t="n"/>
-    </row>
-    <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="60" t="inlineStr">
-        <is>
-          <t>협조 필요    ☑ 생산 중단    ☑ 출하 보류    ☑ 재고 선별    ☐ 고객 통보    ☐ 설비 정지</t>
-        </is>
-      </c>
-      <c r="B19" s="59" t="n"/>
-      <c r="C19" s="59" t="n"/>
-      <c r="D19" s="59" t="n"/>
-      <c r="E19" s="59" t="n"/>
-      <c r="F19" s="59" t="n"/>
-      <c r="G19" s="59" t="n"/>
-      <c r="H19" s="59" t="n"/>
-      <c r="I19" s="59" t="n"/>
-      <c r="J19" s="59" t="n"/>
-      <c r="K19" s="59" t="n"/>
-      <c r="L19" s="59" t="n"/>
-    </row>
-    <row r="20" ht="100" customHeight="1">
-      <c r="A20" s="61" t="inlineStr">
-        <is>
-          <t>08-19 10:20  CAP-02·CAP-04 슬롯 정지, 생산팀장 승인(구두 10:15 · 결재 10:40).
-08-16 이후 생산분 전량 출하 보류 — job 7112~7139 / unit 10388~10604 (2,500대).
-전수 AOI 재검에서 9건 추가 검출, 누적 25건 / 24대 격리. 고객 통보 대상 아님(출하 전).
-배치 하강속도만 mock-v2 값으로 되돌린 임시 레시피 mock-v3h 적용 후 10:50 생산 재개. 08-19 18:00 기준 재발 없음.</t>
-        </is>
-      </c>
-      <c r="B20" s="59" t="n"/>
-      <c r="C20" s="59" t="n"/>
-      <c r="D20" s="59" t="n"/>
-      <c r="E20" s="59" t="n"/>
-      <c r="F20" s="59" t="n"/>
-      <c r="G20" s="59" t="n"/>
-      <c r="H20" s="59" t="n"/>
-      <c r="I20" s="59" t="n"/>
-      <c r="J20" s="59" t="n"/>
-      <c r="K20" s="59" t="n"/>
-      <c r="L20" s="59" t="n"/>
-    </row>
-    <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="49" t="inlineStr">
-        <is>
-          <t>대책 요약</t>
-        </is>
-      </c>
-      <c r="B21" s="46" t="n"/>
-      <c r="C21" s="62" t="inlineStr">
-        <is>
-          <t>하강속도·파지력 조정, 보드 지지 핀 추가. 부품 교체 없음.</t>
-        </is>
-      </c>
-      <c r="D21" s="59" t="n"/>
-      <c r="E21" s="59" t="n"/>
-      <c r="F21" s="59" t="n"/>
-      <c r="G21" s="59" t="n"/>
-      <c r="H21" s="59" t="n"/>
-      <c r="I21" s="59" t="n"/>
-      <c r="J21" s="59" t="n"/>
-      <c r="K21" s="59" t="n"/>
-      <c r="L21" s="59" t="n"/>
-    </row>
-    <row r="22" ht="50" customHeight="1">
-      <c r="A22" s="46" t="n"/>
-      <c r="B22" s="46" t="n"/>
-      <c r="C22" s="59" t="n"/>
-      <c r="D22" s="59" t="n"/>
-      <c r="E22" s="59" t="n"/>
-      <c r="F22" s="59" t="n"/>
-      <c r="G22" s="59" t="n"/>
-      <c r="H22" s="59" t="n"/>
-      <c r="I22" s="59" t="n"/>
-      <c r="J22" s="59" t="n"/>
-      <c r="K22" s="59" t="n"/>
-      <c r="L22" s="59" t="n"/>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="63" t="inlineStr">
-        <is>
-          <t>작성 안내: 연노랑은 담당자 입력 · 파랑은 현황/계산 · 상세 원인부터 종결까지 다음 페이지에 이어집니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="53" t="inlineStr">
-        <is>
-          <t>불량 대책서  |  원인 · 대책 · 검증 · 종결</t>
-        </is>
-      </c>
-      <c r="B24" s="54" t="n"/>
-      <c r="C24" s="54" t="n"/>
-      <c r="D24" s="54" t="n"/>
-      <c r="E24" s="54" t="n"/>
-      <c r="F24" s="54" t="n"/>
-      <c r="G24" s="54" t="n"/>
-      <c r="H24" s="54" t="n"/>
-      <c r="I24" s="54" t="n"/>
-      <c r="J24" s="54" t="n"/>
-      <c r="K24" s="54" t="n"/>
-      <c r="L24" s="54" t="n"/>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="47">
-        <f>C3&amp;"  ·  "&amp;C4&amp;"  /  "&amp;J4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="53" t="inlineStr">
-        <is>
-          <t>② 발생 원인  |  재현·실물 확인 근거</t>
-        </is>
-      </c>
-      <c r="B26" s="54" t="n"/>
-      <c r="C26" s="54" t="n"/>
-      <c r="D26" s="54" t="n"/>
-      <c r="E26" s="54" t="n"/>
-      <c r="F26" s="54" t="n"/>
-      <c r="G26" s="54" t="n"/>
-      <c r="H26" s="54" t="n"/>
-      <c r="I26" s="54" t="n"/>
-      <c r="J26" s="54" t="n"/>
-      <c r="K26" s="54" t="n"/>
-      <c r="L26" s="54" t="n"/>
-    </row>
-    <row r="27" ht="84" customHeight="1">
-      <c r="A27" s="61" t="inlineStr">
-        <is>
-          <t>mock-v3 에서 배치 하강속도(18 → 32 mm/s)와 그리퍼 파지력(3.0 → 4.0 N)을 함께 올렸다.
-CAP-02·CAP-04 는 보드 지지 핀에서 가장 먼 위치라 착지 충격 시 국부 굽힘이 가장 크다. 설비팀 로그에서 두 슬롯 피크력이 다른 CAP 슬롯의 1.7배(6.8N vs 4.0N).
-mock-v3h 로 되돌린 뒤 재발이 멈춘 것으로 검증했다(가설 아님). 불량 25건이 입고 Lot 4개에 고르게 분포해 부품 Lot 요인은 배제한다.</t>
-        </is>
-      </c>
-      <c r="B27" s="59" t="n"/>
-      <c r="C27" s="59" t="n"/>
-      <c r="D27" s="59" t="n"/>
-      <c r="E27" s="59" t="n"/>
-      <c r="F27" s="59" t="n"/>
-      <c r="G27" s="59" t="n"/>
-      <c r="H27" s="59" t="n"/>
-      <c r="I27" s="59" t="n"/>
-      <c r="J27" s="59" t="n"/>
-      <c r="K27" s="59" t="n"/>
-      <c r="L27" s="59" t="n"/>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="53" t="inlineStr">
-        <is>
-          <t>③ 유출 원인  |  검사·판정 기준의 한계</t>
-        </is>
-      </c>
-      <c r="B28" s="54" t="n"/>
-      <c r="C28" s="54" t="n"/>
-      <c r="D28" s="54" t="n"/>
-      <c r="E28" s="54" t="n"/>
-      <c r="F28" s="54" t="n"/>
-      <c r="G28" s="54" t="n"/>
-      <c r="H28" s="54" t="n"/>
-      <c r="I28" s="54" t="n"/>
-      <c r="J28" s="54" t="n"/>
-      <c r="K28" s="54" t="n"/>
-      <c r="L28" s="54" t="n"/>
-    </row>
-    <row r="29" ht="70" customHeight="1">
-      <c r="A29" s="61" t="inlineStr">
-        <is>
-          <t>인라인 AOI 판정 기준이 단자 들뜸과 외관 결손만 보고 있어 미세 굽힘 크랙을 걸러내지 못했다.
-「부품 검토자료」의 MLCC 항목은 '크랙 의심 Lot 단면 또는 비파괴 검사'를 요구하지만, 현재 인라인에는 해당 항목이 없고 단면 검사는 주 1회 샘플로만 돌고 있었다.
-그 결과 08-16 생산분에 이미 크랙이 있었으나 08-18 16:30 임계 초과 시점까지 검출되지 않았다.</t>
-        </is>
-      </c>
-      <c r="B29" s="59" t="n"/>
-      <c r="C29" s="59" t="n"/>
-      <c r="D29" s="59" t="n"/>
-      <c r="E29" s="59" t="n"/>
-      <c r="F29" s="59" t="n"/>
-      <c r="G29" s="59" t="n"/>
-      <c r="H29" s="59" t="n"/>
-      <c r="I29" s="59" t="n"/>
-      <c r="J29" s="59" t="n"/>
-      <c r="K29" s="59" t="n"/>
-      <c r="L29" s="59" t="n"/>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="53" t="inlineStr">
-        <is>
-          <t>④ 재발방지 대책  |  적용 내용 · 담당 · 일정 · 수평전개</t>
-        </is>
-      </c>
-      <c r="B30" s="54" t="n"/>
-      <c r="C30" s="54" t="n"/>
-      <c r="D30" s="54" t="n"/>
-      <c r="E30" s="54" t="n"/>
-      <c r="F30" s="54" t="n"/>
-      <c r="G30" s="54" t="n"/>
-      <c r="H30" s="54" t="n"/>
-      <c r="I30" s="54" t="n"/>
-      <c r="J30" s="54" t="n"/>
-      <c r="K30" s="54" t="n"/>
-      <c r="L30" s="54" t="n"/>
-    </row>
-    <row r="31" ht="84" customHeight="1">
-      <c r="A31" s="61" t="inlineStr">
-        <is>
-          <t>영구대책 ① 레시피 — 하강속도 20 mm/s, 파지력 3.2 N 으로 확정한 mock-v4 적용. 변경관리 ECN-2608-114 승인 08-21, 적용 08-29.
-영구대책 ② 설비 — CAP-02·CAP-04 에 보드 지지 핀 2개 추가(설비팀, 08-28 완료). 수평전개로 IND-01·IND-02 에도 함께 적용했다.
-부품 교체는 하지 않는다. 「부품 검토자료」 후보 2종 모두 표준 단자라 굽힘 크랙 개선 근거가 없다.</t>
-        </is>
-      </c>
-      <c r="B31" s="59" t="n"/>
-      <c r="C31" s="59" t="n"/>
-      <c r="D31" s="59" t="n"/>
-      <c r="E31" s="59" t="n"/>
-      <c r="F31" s="59" t="n"/>
-      <c r="G31" s="59" t="n"/>
-      <c r="H31" s="59" t="n"/>
-      <c r="I31" s="59" t="n"/>
-      <c r="J31" s="59" t="n"/>
-      <c r="K31" s="59" t="n"/>
-      <c r="L31" s="59" t="n"/>
-    </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="53" t="inlineStr">
-        <is>
-          <t>⑤ 효과 검증  |  적용 후 2~4주</t>
-        </is>
-      </c>
-      <c r="B32" s="54" t="n"/>
-      <c r="C32" s="54" t="n"/>
-      <c r="D32" s="54" t="n"/>
-      <c r="E32" s="54" t="n"/>
-      <c r="F32" s="54" t="n"/>
-      <c r="G32" s="54" t="n"/>
-      <c r="H32" s="54" t="n"/>
-      <c r="I32" s="54" t="n"/>
-      <c r="J32" s="54" t="n"/>
-      <c r="K32" s="54" t="n"/>
-      <c r="L32" s="54" t="n"/>
-    </row>
-    <row r="33" ht="26" customHeight="1">
-      <c r="A33" s="49" t="inlineStr">
-        <is>
-          <t>검증 기간</t>
-        </is>
-      </c>
-      <c r="B33" s="46" t="n"/>
-      <c r="C33" s="46" t="n"/>
-      <c r="D33" s="49" t="inlineStr">
-        <is>
-          <t>적용 레시피</t>
-        </is>
-      </c>
-      <c r="E33" s="46" t="n"/>
-      <c r="F33" s="49" t="inlineStr">
-        <is>
-          <t>검사 수량</t>
-        </is>
-      </c>
-      <c r="G33" s="46" t="n"/>
-      <c r="H33" s="49" t="inlineStr">
-        <is>
-          <t>불량 수량</t>
-        </is>
-      </c>
-      <c r="I33" s="46" t="n"/>
-      <c r="J33" s="49" t="inlineStr">
-        <is>
-          <t>판정</t>
-        </is>
-      </c>
-      <c r="K33" s="46" t="n"/>
-      <c r="L33" s="46" t="n"/>
-    </row>
-    <row r="34" ht="32" customHeight="1">
-      <c r="A34" s="64" t="inlineStr">
-        <is>
-          <t>08-29 ~ 09-12</t>
-        </is>
-      </c>
-      <c r="B34" s="59" t="n"/>
-      <c r="C34" s="59" t="n"/>
-      <c r="D34" s="64" t="inlineStr">
-        <is>
-          <t>mock-v4</t>
-        </is>
-      </c>
-      <c r="E34" s="59" t="n"/>
-      <c r="F34" s="65" t="n">
-        <v>24500</v>
-      </c>
-      <c r="G34" s="59" t="n"/>
-      <c r="H34" s="65" t="n">
-        <v>3</v>
-      </c>
-      <c r="I34" s="59" t="n"/>
-      <c r="J34" s="64" t="inlineStr">
-        <is>
-          <t>EFFECTIVE</t>
-        </is>
-      </c>
-      <c r="K34" s="59" t="n"/>
-      <c r="L34" s="59" t="n"/>
-    </row>
-    <row r="35" ht="24" customHeight="1">
-      <c r="A35" s="49" t="inlineStr">
-        <is>
-          <t>검증 불량률</t>
-        </is>
-      </c>
-      <c r="B35" s="46" t="n"/>
-      <c r="C35" s="46" t="n"/>
-      <c r="D35" s="66">
-        <f>IF(AND(ISNUMBER(F34),ISNUMBER(H34),F34&gt;0),H34/F34,"")</f>
-        <v/>
-      </c>
-      <c r="E35" s="46" t="n"/>
-      <c r="F35" s="47" t="inlineStr">
-        <is>
-          <t>판정 근거는 아래에 작성합니다. 수량은 부품 검사 건수 기준입니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="48" customHeight="1">
-      <c r="A36" s="61" t="inlineStr">
-        <is>
-          <t>CRACK 3건 / 24,500건 = 122 PPM. 기준 400 PPM 의 0.31배이고 최소 검사 건수를 충족한다. 대책 전 1,280 PPM 대비 10.5배 개선, CAP-02·CAP-04 집중도도 해소됐다.</t>
-        </is>
-      </c>
-      <c r="B36" s="59" t="n"/>
-      <c r="C36" s="59" t="n"/>
-      <c r="D36" s="59" t="n"/>
-      <c r="E36" s="59" t="n"/>
-      <c r="F36" s="59" t="n"/>
-      <c r="G36" s="59" t="n"/>
-      <c r="H36" s="59" t="n"/>
-      <c r="I36" s="59" t="n"/>
-      <c r="J36" s="59" t="n"/>
-      <c r="K36" s="59" t="n"/>
-      <c r="L36" s="59" t="n"/>
-    </row>
-    <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="53" t="inlineStr">
-        <is>
-          <t>⑥ 종결 판정</t>
-        </is>
-      </c>
-      <c r="B37" s="54" t="n"/>
-      <c r="C37" s="54" t="n"/>
-      <c r="D37" s="54" t="n"/>
-      <c r="E37" s="54" t="n"/>
-      <c r="F37" s="54" t="n"/>
-      <c r="G37" s="54" t="n"/>
-      <c r="H37" s="54" t="n"/>
-      <c r="I37" s="54" t="n"/>
-      <c r="J37" s="54" t="n"/>
-      <c r="K37" s="54" t="n"/>
-      <c r="L37" s="54" t="n"/>
-    </row>
-    <row r="38" ht="28" customHeight="1">
-      <c r="A38" s="49" t="inlineStr">
+      <c r="G26" s="136" t="n"/>
+      <c r="H26" s="148" t="inlineStr">
+        <is>
+          <t>검증 수량: 부품 검사 건수 기준</t>
+        </is>
+      </c>
+      <c r="I26" s="126" t="n"/>
+      <c r="J26" s="126" t="n"/>
+      <c r="K26" s="126" t="n"/>
+      <c r="L26" s="119" t="n"/>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="140" t="n"/>
+      <c r="B27" s="141" t="n"/>
+      <c r="C27" s="128" t="inlineStr">
+        <is>
+          <t>24,500건 중 3건, 122 PPM으로 기준 400 PPM의 0.31배. 최소 검사 건수 충족, 대책 전 대비 10.5배 개선. CAP-02·CAP-04 집중도 해소.</t>
+        </is>
+      </c>
+      <c r="D27" s="129" t="n"/>
+      <c r="E27" s="129" t="n"/>
+      <c r="F27" s="129" t="n"/>
+      <c r="G27" s="129" t="n"/>
+      <c r="H27" s="129" t="n"/>
+      <c r="I27" s="129" t="n"/>
+      <c r="J27" s="129" t="n"/>
+      <c r="K27" s="129" t="n"/>
+      <c r="L27" s="130" t="n"/>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="118" t="inlineStr">
+        <is>
+          <t>⑥ 종결</t>
+        </is>
+      </c>
+      <c r="B28" s="138" t="n"/>
+      <c r="C28" s="118" t="inlineStr">
         <is>
           <t>종결일</t>
         </is>
       </c>
-      <c r="B38" s="46" t="n"/>
-      <c r="C38" s="62" t="inlineStr">
+      <c r="D28" s="119" t="n"/>
+      <c r="E28" s="128" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D38" s="59" t="n"/>
-      <c r="E38" s="59" t="n"/>
-      <c r="F38" s="59" t="n"/>
-      <c r="G38" s="47" t="inlineStr">
-        <is>
-          <t>잔여 위험과 이관 사항을 종결 의견에 기록</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="56" customHeight="1">
-      <c r="A39" s="61" t="inlineStr">
-        <is>
-          <t>영구대책 적용과 효과가 확인되어 종결한다. 잔여 위험 — 지지 핀은 현재 보드 리비전 기준이라 레이아웃 변경 시 재검토가 필요하다. AOI 기준 보완은 별건 QA-PROC-2609-003 으로 이관.</t>
-        </is>
-      </c>
-      <c r="B39" s="59" t="n"/>
-      <c r="C39" s="59" t="n"/>
-      <c r="D39" s="59" t="n"/>
-      <c r="E39" s="59" t="n"/>
-      <c r="F39" s="59" t="n"/>
-      <c r="G39" s="59" t="n"/>
-      <c r="H39" s="59" t="n"/>
-      <c r="I39" s="59" t="n"/>
-      <c r="J39" s="59" t="n"/>
-      <c r="K39" s="59" t="n"/>
-      <c r="L39" s="59" t="n"/>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="49" t="inlineStr">
-        <is>
-          <t>작성</t>
-        </is>
-      </c>
-      <c r="B40" s="46" t="n"/>
-      <c r="C40" s="46" t="n"/>
-      <c r="D40" s="46" t="n"/>
-      <c r="E40" s="49" t="inlineStr">
-        <is>
-          <t>검토</t>
-        </is>
-      </c>
-      <c r="F40" s="46" t="n"/>
-      <c r="G40" s="46" t="n"/>
-      <c r="H40" s="46" t="n"/>
-      <c r="I40" s="49" t="inlineStr">
-        <is>
-          <t>승인</t>
-        </is>
-      </c>
-      <c r="J40" s="46" t="n"/>
-      <c r="K40" s="46" t="n"/>
-      <c r="L40" s="46" t="n"/>
-    </row>
-    <row r="41" ht="32" customHeight="1">
-      <c r="A41" s="62" t="n"/>
-      <c r="B41" s="59" t="n"/>
-      <c r="C41" s="59" t="n"/>
-      <c r="D41" s="59" t="n"/>
-      <c r="E41" s="62" t="n"/>
-      <c r="F41" s="59" t="n"/>
-      <c r="G41" s="59" t="n"/>
-      <c r="H41" s="59" t="n"/>
-      <c r="I41" s="62" t="n"/>
-      <c r="J41" s="59" t="n"/>
-      <c r="K41" s="59" t="n"/>
-      <c r="L41" s="59" t="n"/>
-    </row>
-    <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="67" t="inlineStr">
-        <is>
-          <t>검토용 v2 · 종결 샘플의 수치·일자는 원본 예시입니다.</t>
+      <c r="F28" s="129" t="n"/>
+      <c r="G28" s="130" t="n"/>
+      <c r="H28" s="149" t="inlineStr">
+        <is>
+          <t>잔여 위험 · 이관 사항 확인</t>
+        </is>
+      </c>
+      <c r="I28" s="126" t="n"/>
+      <c r="J28" s="126" t="n"/>
+      <c r="K28" s="126" t="n"/>
+      <c r="L28" s="119" t="n"/>
+    </row>
+    <row r="29" ht="40" customHeight="1">
+      <c r="A29" s="140" t="n"/>
+      <c r="B29" s="141" t="n"/>
+      <c r="C29" s="128" t="inlineStr">
+        <is>
+          <t>영구대책 효과 확인으로 종결. 보드 리비전 변경 시 지지 핀 재검토 필요. AOI 기준 보완은 QA-PROC-2609-003으로 이관.</t>
+        </is>
+      </c>
+      <c r="D29" s="129" t="n"/>
+      <c r="E29" s="129" t="n"/>
+      <c r="F29" s="129" t="n"/>
+      <c r="G29" s="129" t="n"/>
+      <c r="H29" s="129" t="n"/>
+      <c r="I29" s="129" t="n"/>
+      <c r="J29" s="129" t="n"/>
+      <c r="K29" s="129" t="n"/>
+      <c r="L29" s="130" t="n"/>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="150" t="inlineStr">
+        <is>
+          <t>노랑: 관리자 작성 · 파랑: 자동 계산 · 그 외: 시스템 기입 / 종결 내용은 가상 예시·상세 원문은 메모</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="87">
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
+  <mergeCells count="75">
+    <mergeCell ref="C27:L27"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="I14:L14"/>
     <mergeCell ref="D11:F11"/>
+    <mergeCell ref="K25:L25"/>
     <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A37:L37"/>
+    <mergeCell ref="C23:L23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="H26:L26"/>
+    <mergeCell ref="K2:L3"/>
     <mergeCell ref="C5:G5"/>
-    <mergeCell ref="A21:B22"/>
+    <mergeCell ref="A18:B19"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A6:B6"/>
     <mergeCell ref="J11:L11"/>
-    <mergeCell ref="A26:L26"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="I40:L40"/>
-    <mergeCell ref="A23:L23"/>
-    <mergeCell ref="J3:L3"/>
-    <mergeCell ref="A41:D41"/>
-    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="C19:L19"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="A20:B21"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C18:L18"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="C15:L15"/>
+    <mergeCell ref="A17:L17"/>
+    <mergeCell ref="J12:L12"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A28:B29"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="G2:H3"/>
+    <mergeCell ref="A24:B27"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="I2:J3"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C29:L29"/>
+    <mergeCell ref="J8:L8"/>
+    <mergeCell ref="H28:L28"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="A9:L9"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="C20:L20"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:G8"/>
     <mergeCell ref="H13:I13"/>
-    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="A30:L30"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="C22:L22"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="G1:H1"/>
     <mergeCell ref="J13:L13"/>
-    <mergeCell ref="A36:L36"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="H34:I34"/>
-    <mergeCell ref="A32:L32"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="C15:L15"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="J33:L33"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="A31:L31"/>
-    <mergeCell ref="I41:L41"/>
-    <mergeCell ref="C16:L16"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="A24:L24"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="E40:H40"/>
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="A1:F3"/>
+    <mergeCell ref="A13:B13"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="G38:L38"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="A25:L25"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="A18:L18"/>
-    <mergeCell ref="A42:L42"/>
-    <mergeCell ref="C21:L22"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A20:L20"/>
-    <mergeCell ref="A29:L29"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="J1:L1"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="J10:L10"/>
-    <mergeCell ref="F35:L35"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="J34:L34"/>
+    <mergeCell ref="C21:L21"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="H8:I8"/>
     <mergeCell ref="C13:G13"/>
-    <mergeCell ref="A7:L7"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="C38:F38"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="A27:L27"/>
-    <mergeCell ref="E41:H41"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A40:D40"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="J12:L12"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A19:L19"/>
-    <mergeCell ref="A28:L28"/>
-    <mergeCell ref="A9:L9"/>
-    <mergeCell ref="A39:L39"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="A30:L30"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="H14:L14"/>
-    <mergeCell ref="C3:G3"/>
   </mergeCells>
-  <conditionalFormatting sqref="J34:L34">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+  <conditionalFormatting sqref="K25:L25">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
       <formula>"EFFECTIVE"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
       <formula>"INEFFECTIVE"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
       <formula>"PENDING"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="17">
-    <dataValidation sqref="J4" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="허용되지 않는 값" error="다음 중 하나여야 한다: MISSING,POSITION_ERROR,ORIENTATION_ERROR,CRACK" promptTitle="불량 유형" prompt="참고 시트 2개은 유형과 무관하게 항상 첨부한다.&#10;어느 자료가 이번 건에 쓸모 있는지는 담당자가 판단한다." type="list">
+  <dataValidations count="18">
+    <dataValidation sqref="J6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="허용되지 않는 값" error="다음 중 하나여야 한다: MISSING,POSITION_ERROR,ORIENTATION_ERROR,CRACK" promptTitle="불량 유형" prompt="참고 시트 2개은 유형과 무관하게 항상 첨부한다.&#10;어느 자료가 이번 건에 쓸모 있는지는 담당자가 판단한다." type="list">
       <formula1>"MISSING,POSITION_ERROR,ORIENTATION_ERROR,CRACK"</formula1>
     </dataValidation>
-    <dataValidation sqref="A19" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="① 협조가 필요한 조치" prompt="담당자 혼자 결정할 수 없는 항목이다. 해당하는 것의 ☐ 를 ☑ 로 바꾸고,&#10;아래 칸에 누구에게 언제 요청했는지 적는다.&#10;&#10;생산 중단 → 생산팀장 · 출하 보류 → 영업/물류 · 재고 선별 → 인력 투입 승인&#10;고객 통보 → 품질보증 책임자 · 설비 정지 → 설비팀&#10;"/>
-    <dataValidation sqref="A20" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="① 초동 조치 — 오늘 안에" prompt="격리·선별·출하보류 범위와 완료 시각을 적는다.&#10;영향 받는 job_id / unit_id 범위를 함께 적는다.&#10;&#10;원인이 안 나와도 오늘 회신한다. 여기는 '막았는지'만 쓰는 칸이다.&#10;원인을 없애는 것은 ④ 이고, 이 칸은 확산을 멈추는 칸이다.&#10;"/>
-    <dataValidation sqref="C16" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="② 발생 원인 — 한 줄 요약 (40자)" prompt="아래 본문을 한 줄로 줄인 것. 예: '배치 하강속도 상향 + 지지 핀 최원거리 슬롯'&#10;본문은 길어서 이 칸에 들어가지 않으므로 핵심 원인만 적는다."/>
-    <dataValidation sqref="A27" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="② 발생 원인 — 왜 만들어졌는가" prompt="「불량 근거」의 발생 기록과 검사 이미지를 확인한다.&#10;재현 또는 실물 확인으로 검증한 근거를 적는다.&#10;가설이면 '가설'이라고 표시한다.&#10;"/>
-    <dataValidation sqref="A29" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="③ 유출 원인 — 왜 검사에서 걸리지 않았는가" prompt="「부품 검토자료」의 데이터시트 검사 항목과 대조해 판정 기준의 한계를 적는다.&#10;검사를 안 한 것인지, 했는데 못 걸른 것인지 구분한다.&#10;"/>
-    <dataValidation sqref="A31" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="④ 재발방지 대책 — 원인을 제거하는 영구대책" prompt="레시피·공정조건을 바꾸면 변경 후 recipe_version을 적는다.&#10;부품을 바꾸면 「부품 검토자료」의 대체품 영역의 대체코드를 적는다.&#10;동일 부품을 쓰는 다른 슬롯으로의 수평전개 여부를 포함한다.&#10;&#10;레시피 변경은 변경관리 승인이, 부품 교체는 고객 승인이 필요할 수 있다.&#10;승인 절차가 걸리면 그 일정도 함께 적는다.&#10;"/>
-    <dataValidation sqref="A34" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 검증 기간" prompt="대책을 적용하고 다시 집계한 구간. [시작, 끝) 으로 적는다.&#10;"/>
-    <dataValidation sqref="D34" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 적용 레시피" prompt="대책을 적용한 뒤 실행한 recipe_version.&#10;이 값이 있어야 적용 전후를 같은 제품 안에서 비교할 수 있다.&#10;"/>
-    <dataValidation sqref="F34" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 검증 검사 수량" prompt="부품 기준 검사 건수 (유닛 수 × 해당 부품 슬롯 수).&#10;"/>
-    <dataValidation sqref="H34" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 검증 불량 수량" prompt=""/>
-    <dataValidation sqref="J34" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="허용되지 않는 값" error="다음 중 하나여야 한다: PENDING,EFFECTIVE,INEFFECTIVE" promptTitle="⑤ 판정" prompt="품질 절차에서 정한 판정 기준에 따라 선택한다." type="list">
+    <dataValidation sqref="C18" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="① 협조가 필요한 조치" prompt="담당자 혼자 결정할 수 없는 항목이다. 해당하는 것의 □ 를 ■ 로 바꾸고,&#10;아래 칸에 누구에게 언제 요청했는지 적는다.&#10;&#10;생산 중단 → 생산팀장 · 출하 보류 → 영업/물류 · 재고 선별 → 인력 투입 승인&#10;고객 통보 → 품질보증 책임자 · 설비 정지 → 설비팀&#10;"/>
+    <dataValidation sqref="C19" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="① 초동 조치 — 오늘 안에" prompt="격리·선별·출하보류 범위와 완료 시각을 적는다.&#10;영향 받는 job_id / unit_id 범위를 함께 적는다.&#10;&#10;원인이 안 나와도 오늘 회신한다. 여기는 '막았는지'만 쓰는 칸이다.&#10;원인을 없애는 것은 ④ 이고, 이 칸은 확산을 멈추는 칸이다.&#10;"/>
+    <dataValidation sqref="C20" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="② 발생 원인 — 한 줄 요약 (40자)" prompt="본문을 한 줄로 줄인 것. 예: '배치 하강속도 상향 + 지지 핀 최원거리 슬롯'&#10;본문은 길어서 이 칸에 들어가지 않으므로 핵심 원인만 적는다."/>
+    <dataValidation sqref="C21" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="② 발생 원인 — 왜 만들어졌는가" prompt="「불량 근거」의 발생 기록과 검사 이미지를 확인한다.&#10;재현 또는 실물 확인으로 검증한 근거를 적는다.&#10;가설이면 '가설'이라고 표시한다.&#10;"/>
+    <dataValidation sqref="C22" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="③ 유출 원인 — 왜 검사에서 걸리지 않았는가" prompt="「부품 검토자료」의 데이터시트 검사 항목과 대조해 판정 기준의 한계를 적는다.&#10;검사를 안 한 것인지, 했는데 못 걸른 것인지 구분한다.&#10;"/>
+    <dataValidation sqref="C23" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="④ 재발방지 대책 — 원인을 제거하는 영구대책" prompt="레시피·공정조건을 바꾸면 변경 후 recipe_version을 적는다.&#10;부품을 바꾸면 「부품 검토자료」의 대체품 영역의 대체코드를 적는다.&#10;동일 부품을 쓰는 다른 슬롯으로의 수평전개 여부를 포함한다.&#10;&#10;레시피 변경은 변경관리 승인이, 부품 교체는 고객 승인이 필요할 수 있다.&#10;승인 절차가 걸리면 그 일정도 함께 적는다.&#10;"/>
+    <dataValidation sqref="C25" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 검증 기간" prompt="대책을 적용하고 다시 집계한 구간. [시작, 끝) 으로 적는다.&#10;"/>
+    <dataValidation sqref="E25" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 적용 레시피" prompt="대책을 적용한 뒤 실행한 recipe_version.&#10;이 값이 있어야 적용 전후를 같은 제품 안에서 비교할 수 있다.&#10;"/>
+    <dataValidation sqref="G25" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 검증 검사 수량" prompt="부품 기준 검사 건수 (유닛 수 × 해당 부품 슬롯 수).&#10;"/>
+    <dataValidation sqref="G25" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="수량 확인" error="0 이상의 정수를 입력하세요." type="whole" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="I25" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 검증 불량 수량" prompt=""/>
+    <dataValidation sqref="I25" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="수량 확인" error="0 이상의 정수를 입력하세요." type="whole" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="K25" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="허용되지 않는 값" error="다음 중 하나여야 한다: PENDING,EFFECTIVE,INEFFECTIVE" promptTitle="⑤ 판정" prompt="품질 절차에서 정한 판정 기준에 따라 선택한다." type="list">
       <formula1>"PENDING,EFFECTIVE,INEFFECTIVE"</formula1>
     </dataValidation>
-    <dataValidation sqref="J34" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 판정" prompt="판정 기준과 비교한 결론을 선택한다.&#10;기준은 해당 품질 절차에서 확인한다."/>
-    <dataValidation sqref="A36" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 판정 근거" prompt="재집계 결과를 그렇게 읽은 이유.&#10;"/>
-    <dataValidation sqref="C38" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑥ 종결일" prompt=""/>
-    <dataValidation sqref="A39" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑥ 종결 의견" prompt="잔여 위험과 종결 승인 의견.&#10;"/>
-    <dataValidation sqref="F34 H34" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="수량 확인" error="0 이상의 정수를 입력하세요." type="whole" operator="greaterThanOrEqual">
-      <formula1>0</formula1>
-    </dataValidation>
+    <dataValidation sqref="K25" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 판정" prompt="판정 기준과 비교한 결론을 선택한다.&#10;기준은 해당 품질 절차에서 확인한다."/>
+    <dataValidation sqref="C27" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 판정 근거" prompt="재집계 결과를 그렇게 읽은 이유.&#10;"/>
+    <dataValidation sqref="E28" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑥ 종결일" prompt=""/>
+    <dataValidation sqref="C29" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑥ 종결 의견" prompt="잔여 위험과 종결 승인 의견.&#10;"/>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.32" right="0.32" top="0.35" bottom="0.38" header="0.15" footer="0.17"/>
+  <pageMargins left="0.32" right="0.32" top="0.32" bottom="0.32" header="0.1" footer="0.1"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;L&amp;8 &amp;K627083v2 · 검토용&amp;R&amp;8 &amp;K627083&amp;P / &amp;N</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-  <rowBreaks count="1" manualBreakCount="1">
-    <brk id="23" min="0" max="16383" man="1"/>
-  </rowBreaks>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
@@ -2214,9 +2618,9 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="68" t="inlineStr">
-        <is>
-          <t>불량 근거  |  발행 시점 고정</t>
+      <c r="A1" s="151" t="inlineStr">
+        <is>
+          <t>불량 근거 · 시스템 자동 기입 / 발행 시점 고정</t>
         </is>
       </c>
     </row>
@@ -2609,25 +3013,25 @@
   <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="84" t="inlineStr">
-        <is>
-          <t>부품 검토자료</t>
+      <c r="A1" s="152" t="inlineStr">
+        <is>
+          <t>부품 검토자료 · 시스템 자동 기입</t>
         </is>
       </c>
     </row>
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="85" t="inlineStr">
         <is>
-          <t>부품 범주 MLCC · 데이터시트 대조 일치 · 기준일 2026-08-18 · 조회 2026-08-19 09:00:00</t>
+          <t>부품 범주 MLCC · 대조 일치 · 기준일 2026-08-18 · 현행 자료 조회 2026-09-07 14:00:58</t>
         </is>
       </c>
     </row>
@@ -2637,11 +3041,6 @@
           <t>현재 부품  |  데이터시트 대조</t>
         </is>
       </c>
-      <c r="B3" s="54" t="n"/>
-      <c r="C3" s="54" t="n"/>
-      <c r="D3" s="54" t="n"/>
-      <c r="E3" s="54" t="n"/>
-      <c r="F3" s="54" t="n"/>
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="49" t="inlineStr">
@@ -2659,9 +3058,9 @@
           <t>공급사</t>
         </is>
       </c>
-      <c r="D4" s="49" t="inlineStr">
-        <is>
-          <t>단가</t>
+      <c r="D4" s="153" t="inlineStr">
+        <is>
+          <t>단가(USD)</t>
         </is>
       </c>
       <c r="E4" s="49" t="inlineStr">
@@ -2675,7 +3074,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="52" customHeight="1">
+    <row r="5" ht="44" customHeight="1">
       <c r="A5" s="50" t="inlineStr">
         <is>
           <t>Contoso CX-0603X7R104K100</t>
@@ -2718,14 +3117,9 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="53" t="inlineStr">
         <is>
-          <t>품질 체크리스트  |  검사 항목과 이상 시 조치</t>
-        </is>
-      </c>
-      <c r="B7" s="54" t="n"/>
-      <c r="C7" s="54" t="n"/>
-      <c r="D7" s="54" t="n"/>
-      <c r="E7" s="54" t="n"/>
-      <c r="F7" s="54" t="n"/>
+          <t>품질 체크리스트  |  공통 기준 + 부품별 기준</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="49" t="inlineStr">
@@ -2738,65 +3132,61 @@
           <t>확인 항목</t>
         </is>
       </c>
-      <c r="C8" s="46" t="n"/>
-      <c r="D8" s="46" t="n"/>
       <c r="E8" s="49" t="inlineStr">
         <is>
           <t>이상 시 조치</t>
         </is>
       </c>
-      <c r="F8" s="46" t="n"/>
-    </row>
-    <row r="9" ht="48" customHeight="1">
+    </row>
+    <row r="9" ht="72" customHeight="1">
       <c r="A9" s="49" t="inlineStr">
         <is>
           <t>입고 검사</t>
         </is>
       </c>
-      <c r="B9" s="50" t="inlineStr">
-        <is>
-          <t>외관/단자, 0603·100V·X7R 확인, LCR·절연저항 샘플</t>
-        </is>
-      </c>
-      <c r="E9" s="61" t="inlineStr">
-        <is>
-          <t>크랙/IR 저하는 Lot·패널 위치별 격리, 보드 굴곡·분리·프로브 지지 조건을 재현하고 공정 조건 수정</t>
-        </is>
-      </c>
-      <c r="F9" s="59" t="n"/>
-    </row>
-    <row r="10" ht="48" customHeight="1">
+      <c r="B9" s="154" t="inlineStr">
+        <is>
+          <t>승인 공급처, PO/BOM-MPN-revision, 수량, CoC, Lot/date code, 포장·라벨·봉인 대조
+외관/단자, 0603·100V·X7R 확인, LCR·절연저항 샘플</t>
+        </is>
+      </c>
+      <c r="E9" s="154" t="inlineStr">
+        <is>
+          <t>Line stop → 의심 Lot 전량 격리 → 영향 범위/재공품 추적 → NCR·공급사 FA/8D·CAPA → 변경 승인 후 재검
+크랙/IR 저하는 Lot·패널 위치별 격리, 보드 굴곡·분리·프로브 지지 조건을 재현하고 공정 조건 수정</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="78" customHeight="1">
       <c r="A10" s="49" t="inlineStr">
         <is>
           <t>조립·보관</t>
         </is>
       </c>
-      <c r="B10" s="50" t="inlineStr">
-        <is>
-          <t>land/reflow 준수; panel depanel·ICT probe·connector 체결 시 board support로 보드 굽힘 억제</t>
-        </is>
-      </c>
-      <c r="E10" s="59" t="n"/>
-      <c r="F10" s="59" t="n"/>
-    </row>
-    <row r="11" ht="48" customHeight="1">
+      <c r="B10" s="154" t="inlineStr">
+        <is>
+          <t>격리 상태 표시, ESD/MSL/극성·온습도·노출시간 관리, FIFO, Lot 혼합 금지
+land/reflow 준수; panel depanel·ICT probe·connector 체결 시 board support로 굽힘 억제</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="64" customHeight="1">
       <c r="A11" s="49" t="inlineStr">
         <is>
           <t>기능·신뢰성</t>
         </is>
       </c>
-      <c r="B11" s="50" t="inlineStr">
-        <is>
-          <t>AOI, LCR/IR; crack 의심 Lot 단면 또는 비파괴 검사</t>
-        </is>
-      </c>
-      <c r="E11" s="59" t="n"/>
-      <c r="F11" s="59" t="n"/>
+      <c r="B11" s="154" t="inlineStr">
+        <is>
+          <t>초도품 승인 후 Lot별 샘플링; 검사결과와 serial/Lot 추적
+AOI, LCR/IR; crack 의심 Lot 단면 또는 비파괴 검사</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="47" t="inlineStr">
         <is>
-          <t>부품 데이터시트 Checklist 시트에서 조회 · 원인 자동 추정 자료가 아님</t>
+          <t>Checklist 공통·부품별 항목을 함께 조회 · 원인·적합성 판단은 관리자 작성</t>
         </is>
       </c>
     </row>
@@ -2814,11 +3204,6 @@
           <t>대체품 후보  |  적합성 검증·변경 승인 후 적용</t>
         </is>
       </c>
-      <c r="B14" s="54" t="n"/>
-      <c r="C14" s="54" t="n"/>
-      <c r="D14" s="54" t="n"/>
-      <c r="E14" s="54" t="n"/>
-      <c r="F14" s="54" t="n"/>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="86" t="inlineStr">
@@ -2826,16 +3211,11 @@
           <t>같은 부품 타입이라는 것 외에 검증된 것은 없다 · 동일 정격만으로 drop-in 판단 금지 · 핀/패키지/정격/열/수명 재검증과 변경 승인을 거친 뒤에만 적용한다.</t>
         </is>
       </c>
-      <c r="B15" s="87" t="n"/>
-      <c r="C15" s="87" t="n"/>
-      <c r="D15" s="87" t="n"/>
-      <c r="E15" s="87" t="n"/>
-      <c r="F15" s="87" t="n"/>
-    </row>
-    <row r="16" ht="44" customHeight="1">
+    </row>
+    <row r="16" ht="26" customHeight="1">
       <c r="A16" s="85" t="inlineStr">
         <is>
-          <t>조회 시각 2026-08-19 09:00:00   ·   데이터시트 semiconductor_assembly_quality_datasheet_2026-08-18.xlsx (기준일 2026-08-18)   ·   부품 타입 MLCC   ·   후보 2종   ·   단가 $0.09 ~ $0.15   ·   현재 선정 $0.15</t>
+          <t>같은 타입 후보 2종 · 단가 $0.09 ~ $0.15 · 현재 선정 $0.15 · 호환성 미승인</t>
         </is>
       </c>
     </row>
@@ -2855,9 +3235,9 @@
           <t>공급사</t>
         </is>
       </c>
-      <c r="D17" s="49" t="inlineStr">
-        <is>
-          <t>단가</t>
+      <c r="D17" s="153" t="inlineStr">
+        <is>
+          <t>단가(USD)</t>
         </is>
       </c>
       <c r="E17" s="49" t="inlineStr">
@@ -2871,7 +3251,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="54" customHeight="1">
+    <row r="18" ht="50" customHeight="1">
       <c r="A18" s="88" t="inlineStr">
         <is>
           <t>Litware LW-C0603-104K-100</t>
@@ -2903,7 +3283,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="54" customHeight="1">
+    <row r="19" ht="50" customHeight="1">
       <c r="A19" s="50" t="inlineStr">
         <is>
           <t>Tailspin TS-0603-104M-100</t>
@@ -2938,23 +3318,25 @@
     <row r="20" ht="42" customHeight="1">
       <c r="A20" s="85" t="inlineStr">
         <is>
-          <t>단가는 데이터시트 기준일의 값이고 발주 근거가 아니다. MOQ·재고·리드타임과 상호호환 판정은 이 문서에 없다 → GET /parts/CAP 또는 구매·품질 담당</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="47" t="inlineStr">
-        <is>
-          <t>원본 semiconductor_assembly_quality_datasheet_2026-08-18.xlsx · DB parts: CAP / Contoso CX-0603X7R104K100 / MLCC · 데이터시트 MPN 대조: 일치</t>
+          <t>단가는 데이터시트 기준일의 값이고 발주 근거가 아니다. MOQ·재고·리드타임과 상호호환 판정은 이 문서에 없다 → GET /api/v1/parts/CAP 또는 구매·품질 담당</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="38" customHeight="1">
+      <c r="A21" s="155" t="inlineStr">
+        <is>
+          <t>원본 semiconductor_assembly_quality_datasheet_2026-08-18.xlsx
+SHA-256: e35dacdde1e02dfdc620c1026147d525927b9ca22e4c5ec25c978766c806ad66</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <mergeCells count="16">
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:F16"/>
     <mergeCell ref="B11:D11"/>
-    <mergeCell ref="A16:F16"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="A1:F1"/>
@@ -2979,5 +3361,6 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: snapshot current workspace before mode isolation changes
</commit_message>
<xml_diff>
--- a/MAIN_SERVER/templates/불량대책서_샘플_종결본_v2.xlsx
+++ b/MAIN_SERVER/templates/불량대책서_샘플_종결본_v2.xlsx
@@ -27,7 +27,7 @@
     <definedName name="reply_closed_at">'대책서'!$E$28</definedName>
     <definedName name="reply_closure_note">'대책서'!$C$29</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'대책서'!$A$1:$L$30</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'불량 근거'!$A$1:$E$26</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'불량 근거'!$A$1:$E$23</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'부품 검토자료'!$A$1:$F$21</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -40,7 +40,7 @@
     <numFmt numFmtId="164" formatCode="0.0&quot;배&quot;"/>
     <numFmt numFmtId="165" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="54">
+  <fonts count="66">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -345,8 +345,73 @@
       <color rgb="00243D5B"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00233D59"/>
+      <sz val="23"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00263442"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="00263442"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="00263442"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="00263442"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00263442"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="00657385"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="00263442"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="00263442"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00233D59"/>
+      <sz val="17"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="00263442"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00233D59"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -423,8 +488,28 @@
         <fgColor rgb="00F2F3F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDF3F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F2F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF5F0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="32">
+  <borders count="42">
     <border>
       <left/>
       <right/>
@@ -752,11 +837,118 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BCC6D1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BCC6D1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BCC6D1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BCC6D1"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BCC6D1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BCC6D1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BCC6D1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BCC6D1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BCC6D1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BCC6D1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BCC6D1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BCC6D1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BCC6D1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BCC6D1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BCC6D1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BCC6D1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BCC6D1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BCC6D1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BCC6D1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="156">
+  <cellXfs count="245">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1166,6 +1358,250 @@
     <xf numFmtId="0" fontId="48" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="54" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="10" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="17" borderId="23" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="17" borderId="26" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="17" borderId="27" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="18" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="57" fillId="17" borderId="32" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="17" borderId="32" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="16" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="16" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="16" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="16" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="19" borderId="23" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="19" borderId="26" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="19" borderId="27" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="16" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="16" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="16" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="10" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="10" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="16" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="10" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="18" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="10" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="64" fillId="10" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="17" borderId="23" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="25" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="30" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="31" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="19" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="17" borderId="23" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="26" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="27" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="23" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="19" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="35" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="36" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="19" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="59" fillId="18" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="17" borderId="23" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="17" borderId="23" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="23" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="17" borderId="23" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="47" fillId="19" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="19" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="19" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="19" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="37" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="38" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="39" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="64" fillId="19" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="65" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1209,33 +1645,18 @@
         <b val="1"/>
         <color rgb="00216348"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00EEF5F0"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
         <b val="1"/>
         <color rgb="009C2A2A"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00F9EEEE"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
         <b val="1"/>
         <color rgb="0080601B"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFF9EB"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1321,111 +1742,268 @@
         <t>부품 식별자: CAP</t>
       </text>
     </comment>
+    <comment ref="A4" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+시스템 자동 기입 · 발행 시점 고정  |  담당·기한·문서 상태는 관리자 갱신</t>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+QA-CAP-CRACK-20260819-001</t>
+      </text>
+    </comment>
+    <comment ref="J5" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+2026-08-19 09:00:00</t>
+      </text>
+    </comment>
     <comment ref="C6" authorId="0" shapeId="0">
       <text>
         <t>제조사 P/N·정격·공급사 (이전 v2)
 일치 · Contoso CX-0603X7R104K100
 정격 0.10µF ±10% 100V X7R 0603 · 공급사 Northwind Traders
-자세한 비교는 「부품 검토자료」 참조.</t>
+자세한 비교는 「부품 검토자료」 참조.
+이전 v2 내용(참고):
+CAP  (MLCC)</t>
+      </text>
+    </comment>
+    <comment ref="J6" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+CRACK</t>
       </text>
     </comment>
     <comment ref="C7" authorId="0" shapeId="0">
       <text>
-        <t>시스템은 배정 대기만 초기 기입합니다. 실제 주관 담당자는 관리자가 작성합니다.</t>
+        <t>시스템은 배정 대기만 초기 기입합니다. 실제 주관 담당자는 관리자가 작성합니다.
+이전 v2 내용(참고):
+품질보증팀 김OO</t>
       </text>
     </comment>
     <comment ref="J7" authorId="0" shapeId="0">
       <text>
-        <t>시스템은 담당자 입력만 초기 기입합니다. 실제 협조 부서는 관리자가 작성합니다.</t>
+        <t>시스템은 담당자 입력만 초기 기입합니다. 실제 협조 부서는 관리자가 작성합니다.
+이전 v2 내용(참고):
+설비팀 · 생산팀 · 구매</t>
+      </text>
+    </comment>
+    <comment ref="C8" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+Job 7112 · Unit 10412 · CAP-02</t>
+      </text>
+    </comment>
+    <comment ref="J8" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+2026-08-18 16:30:12</t>
       </text>
     </comment>
     <comment ref="A9" authorId="0" shapeId="0">
       <text>
-        <t>문서 상태와 회신 기한은 시스템이 ISSUED / 담당자 입력으로 초기화하며 이후 관리자가 갱신합니다. Job 상태 또는 DB의 메일 전송 상태와 별개입니다.</t>
+        <t>문서 상태와 회신 기한은 시스템이 ISSUED / 담당자 입력으로 초기화하며 이후 관리자가 갱신합니다. Job 상태 또는 DB의 메일 전송 상태와 별개입니다.
+이전 v2 내용(참고):
+상태  CLOSED  ·  ①~⑥ 작성 완료  ·  발행 기준: 확정 불량 1건</t>
       </text>
     </comment>
     <comment ref="A12" authorId="0" shapeId="0">
       <text>
-        <t>시스템 자동 기입. 발행 검사 시각까지 동일 Job의 검사 완료 Unit 수 × 해당 부품 슬롯 수입니다. requested_quantity(목표 PASS 수량)가 아닙니다.</t>
-      </text>
-    </comment>
-    <comment ref="D12" authorId="0" shapeId="0">
-      <text>
-        <t>시스템 자동 기입. 동일 Job·부품·불량 유형의 production.unit_defects 기록 수입니다. 불량 Unit 수와 다를 수 있습니다.</t>
-      </text>
-    </comment>
-    <comment ref="J12" authorId="0" shapeId="0">
-      <text>
-        <t>자동 계산. 관리자가 아래 검증 검사 수량·불량 수량을 입력하면 PPM을 계산합니다. 검사 시스템에서 재집계해 자동 채우는 값은 아닙니다.</t>
-      </text>
-    </comment>
-    <comment ref="C14" authorId="0" shapeId="0">
-      <text>
-        <t>발행 시점 전체 슬롯 분포: CAP-02 8건 · CAP-04 5건
-전체 분포는 불량 근거 시트에 자동 기입됩니다.</t>
+        <t xml:space="preserve">실제 발주·입고 자료로 확인한 업체명. 데이터시트 공급사를 자동 전사하지 않습니다.
+이전 v2 내용(참고):
+</t>
+      </text>
+    </comment>
+    <comment ref="E12" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">업체 담당자·직책·연락처. 접수 확인은 불량 근거에 기록합니다.
+이전 v2 내용(참고):
+</t>
+      </text>
+    </comment>
+    <comment ref="I12" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">요청 마감 일시와 시간대. 원인·대책 기한은 초동 조치 칸에 기록합니다.
+이전 v2 내용(참고):
+</t>
+      </text>
+    </comment>
+    <comment ref="C13" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+2026-08-12 ~ 08-19  (7일 / ROLLING)</t>
+      </text>
+    </comment>
+    <comment ref="J13" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+mock-v3</t>
+      </text>
+    </comment>
+    <comment ref="A14" authorId="0" shapeId="0">
+      <text>
+        <t>동일 Job·부품·불량 유형, 대상 검사 시점까지 누적. 검사 수량은 검사 Unit 수 × 부품 슬롯 수. 폐기 수량이나 납품 Lot 불량률이 아닙니다.</t>
+      </text>
+    </comment>
+    <comment ref="A15" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+자동 분석</t>
       </text>
     </comment>
     <comment ref="C15" authorId="0" shapeId="0">
       <text>
         <t>상세 원문 (이전 v2)
-확정 불량 1건을 기준으로 즉시 발행했다. 발행 시점까지 동일 Job·부품·유형은 16건이며 CAP-02·CAP-04에 13건이 기록됐다. 원인은 자동 추정하지 않으며 담당자가 검사 이미지와 데이터시트 품질 기준을 확인한다.</t>
+확정 불량 1건을 기준으로 즉시 발행했다. 발행 시점까지 동일 Job·부품·유형은 16건이며 CAP-02·CAP-04에 13건이 기록됐다. 원인은 자동 추정하지 않으며 담당자가 검사 이미지와 데이터시트 품질 기준을 확인한다.
+이전 v2 내용(참고):
+확정 불량 1건으로 발행. 동일 Job·부품·유형 누적 16건 중 CAP-02·CAP-04에 13건 집중. 원인은 자동 추정하지 않으며 담당자가 이미지·품질 기준을 확인.</t>
+      </text>
+    </comment>
+    <comment ref="A17" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+관리자 직접 작성  |  ①~⑥ 조치·원인·대책·검증·종결 (예시)</t>
+      </text>
+    </comment>
+    <comment ref="A18" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+① 초동 조치</t>
+      </text>
+    </comment>
+    <comment ref="C18" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+■ 생산 중단    ■ 출하 보류    ■ 재고 선별    □ 고객 통보    □ 설비 정지</t>
       </text>
     </comment>
     <comment ref="C19" authorId="0" shapeId="0">
       <text>
+        <t>당사 담당자가 작성: 조치 요청 범위 / 실제 실행 시각·확인자 / 확정·의심 수량 구분 / 초기·원인·대책 회신 마감 / 관련 문서번호. 자동 정지 완료로 해석하지 않습니다.</t>
+      </text>
+    </comment>
+    <comment ref="A20" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+② 발생 원인</t>
+      </text>
+    </comment>
+    <comment ref="C20" authorId="0" shapeId="0">
+      <text>
+        <t>② 발생 원인의 핵심을 한 줄로 요약합니다.
+이전 v2 내용(참고):
+배치 하강속도 상향 + 지지 핀 최원거리 슬롯</t>
+      </text>
+    </comment>
+    <comment ref="C21" authorId="0" shapeId="0">
+      <text>
+        <t>거래처 또는 조치부서 회신: 발생 원인 + 재현·비교 시험 근거 + 책임 판단. 추정과 입증을 구분합니다.</t>
+      </text>
+    </comment>
+    <comment ref="A22" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+③ 유출 원인</t>
+      </text>
+    </comment>
+    <comment ref="C22" authorId="0" shapeId="0">
+      <text>
+        <t>왜 기존 검사에서 발견하지 못했는지, 해당 검사 기준·검출 능력과 입증 자료를 적습니다.</t>
+      </text>
+    </comment>
+    <comment ref="A23" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+④ 재발방지
+대책</t>
+      </text>
+    </comment>
+    <comment ref="C23" authorId="0" shapeId="0">
+      <text>
+        <t>변경 내용, 담당자, 완료 예정·실제 일시, 적용 Lot 또는 Unit, 변경 승인·효과 검증 자료 번호.</t>
+      </text>
+    </comment>
+    <comment ref="A24" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+⑤ 효과 검증</t>
+      </text>
+    </comment>
+    <comment ref="C25" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+08-29 ~ 09-12</t>
+      </text>
+    </comment>
+    <comment ref="E25" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+mock-v4</t>
+      </text>
+    </comment>
+    <comment ref="G25" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+24500</t>
+      </text>
+    </comment>
+    <comment ref="I25" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+3</t>
+      </text>
+    </comment>
+    <comment ref="C26" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+불량률(자동 계산)</t>
+      </text>
+    </comment>
+    <comment ref="F26" authorId="0" shapeId="0">
+      <text>
+        <t>자동 계산. 검증 불량 수량 ÷ 검증 검사 수량. 검증 수량은 부품 검사 건수 기준입니다.</t>
+      </text>
+    </comment>
+    <comment ref="H26" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+검증 수량: 부품 검사 건수 기준</t>
+      </text>
+    </comment>
+    <comment ref="C27" authorId="0" shapeId="0">
+      <text>
         <t>상세 원문 (이전 v2)
-08-19 10:20  CAP-02·CAP-04 슬롯 정지, 생산팀장 승인(구두 10:15 · 결재 10:40).
-08-16 이후 생산분 전량 출하 보류 — job 7112~7139 / unit 10388~10604 (2,500대).
-전수 AOI 재검에서 9건 추가 검출, 누적 25건 / 24대 격리. 고객 통보 대상 아님(출하 전).
-배치 하강속도만 mock-v2 값으로 되돌린 임시 레시피 mock-v3h 적용 후 10:50 생산 재개. 08-19 18:00 기준 재발 없음.</t>
-      </text>
-    </comment>
-    <comment ref="C20" authorId="0" shapeId="0">
-      <text>
-        <t>② 발생 원인의 핵심을 한 줄로 요약합니다.</t>
-      </text>
-    </comment>
-    <comment ref="C21" authorId="0" shapeId="0">
+CRACK 3건 / 24,500건 = 122 PPM. 기준 400 PPM 의 0.31배이고 최소 검사 건수를 충족한다. 대책 전 1,280 PPM 대비 10.5배 개선, CAP-02·CAP-04 집중도도 해소됐다.
+이전 v2 내용(참고):
+24,500건 중 3건, 122 PPM으로 기준 400 PPM의 0.31배. 최소 검사 건수 충족, 대책 전 대비 10.5배 개선. CAP-02·CAP-04 집중도 해소.</t>
+      </text>
+    </comment>
+    <comment ref="A28" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+⑥ 종결</t>
+      </text>
+    </comment>
+    <comment ref="H28" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+잔여 위험 · 이관 사항 확인</t>
+      </text>
+    </comment>
+    <comment ref="C29" authorId="0" shapeId="0">
       <text>
         <t>상세 원문 (이전 v2)
-mock-v3 에서 배치 하강속도(18 → 32 mm/s)와 그리퍼 파지력(3.0 → 4.0 N)을 함께 올렸다.
-CAP-02·CAP-04 는 보드 지지 핀에서 가장 먼 위치라 착지 충격 시 국부 굽힘이 가장 크다. 설비팀 로그에서 두 슬롯 피크력이 다른 CAP 슬롯의 1.7배(6.8N vs 4.0N).
-mock-v3h 로 되돌린 뒤 재발이 멈춘 것으로 검증했다(가설 아님). 불량 25건이 입고 Lot 4개에 고르게 분포해 부품 Lot 요인은 배제한다.</t>
-      </text>
-    </comment>
-    <comment ref="C22" authorId="0" shapeId="0">
-      <text>
-        <t>상세 원문 (이전 v2)
-인라인 AOI 판정 기준이 단자 들뜸과 외관 결손만 보고 있어 미세 굽힘 크랙을 걸러내지 못했다.
-「부품 검토자료」의 MLCC 항목은 '크랙 의심 Lot 단면 또는 비파괴 검사'를 요구하지만, 현재 인라인에는 해당 항목이 없고 단면 검사는 주 1회 샘플로만 돌고 있었다.
-그 결과 08-16 생산분에 이미 크랙이 있었으나 08-18 16:30 임계 초과 시점까지 검출되지 않았다.</t>
-      </text>
-    </comment>
-    <comment ref="C23" authorId="0" shapeId="0">
-      <text>
-        <t>상세 원문 (이전 v2)
-영구대책 ① 레시피 — 하강속도 20 mm/s, 파지력 3.2 N 으로 확정한 mock-v4 적용. 변경관리 ECN-2608-114 승인 08-21, 적용 08-29.
-영구대책 ② 설비 — CAP-02·CAP-04 에 보드 지지 핀 2개 추가(설비팀, 08-28 완료). 수평전개로 IND-01·IND-02 에도 함께 적용했다.
-부품 교체는 하지 않는다. 「부품 검토자료」 후보 2종 모두 표준 단자라 굽힘 크랙 개선 근거가 없다.
-기존 대책 요약
-하강속도·파지력 조정, 보드 지지 핀 추가. 부품 교체 없음.</t>
-      </text>
-    </comment>
-    <comment ref="F26" authorId="0" shapeId="0">
-      <text>
-        <t>자동 계산. 검증 불량 수량 ÷ 검증 검사 수량. 검증 수량은 부품 검사 건수 기준입니다.</t>
-      </text>
-    </comment>
-    <comment ref="C27" authorId="0" shapeId="0">
-      <text>
-        <t>상세 원문 (이전 v2)
-CRACK 3건 / 24,500건 = 122 PPM. 기준 400 PPM 의 0.31배이고 최소 검사 건수를 충족한다. 대책 전 1,280 PPM 대비 10.5배 개선, CAP-02·CAP-04 집중도도 해소됐다.</t>
-      </text>
-    </comment>
-    <comment ref="C29" authorId="0" shapeId="0">
-      <text>
-        <t>상세 원문 (이전 v2)
-영구대책 적용과 효과가 확인되어 종결한다. 잔여 위험 — 지지 핀은 현재 보드 리비전 기준이라 레이아웃 변경 시 재검토가 필요하다. AOI 기준 보완은 별건 QA-PROC-2609-003 으로 이관.</t>
+영구대책 적용과 효과가 확인되어 종결한다. 잔여 위험 — 지지 핀은 현재 보드 리비전 기준이라 레이아웃 변경 시 재검토가 필요하다. AOI 기준 보완은 별건 QA-PROC-2609-003 으로 이관.
+이전 v2 내용(참고):
+영구대책 효과 확인으로 종결. 보드 리비전 변경 시 지지 핀 재검토 필요. AOI 기준 보완은 QA-PROC-2609-003으로 이관.</t>
+      </text>
+    </comment>
+    <comment ref="A30" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+노랑: 관리자 작성 · 파랑: 자동 계산 · 그 외: 시스템 기입 / 종결 내용은 가상 예시·상세 원문은 메모</t>
       </text>
     </comment>
   </commentList>
@@ -1438,97 +2016,98 @@
     <author>User</author>
   </authors>
   <commentList>
-    <comment ref="B9" authorId="0" shapeId="0">
-      <text>
-        <t>현행 데이터시트 대조로 공통 기준을 포함했습니다.
-이전 샘플 문구:
-외관/단자, 0603·100V·X7R 확인, LCR·절연저항 샘플</t>
-      </text>
-    </comment>
-    <comment ref="E9" authorId="0" shapeId="0">
-      <text>
-        <t>현행 데이터시트 대조로 공통 기준을 포함했습니다.
-이전 샘플 문구:
-크랙/IR 저하는 Lot·패널 위치별 격리, 보드 굴곡·분리·프로브 지지 조건을 재현하고 공정 조건 수정</t>
-      </text>
-    </comment>
     <comment ref="B10" authorId="0" shapeId="0">
       <text>
-        <t>현행 데이터시트 대조로 공통 기준을 포함했습니다.
-이전 샘플 문구:
-land/reflow 준수; panel depanel·ICT probe·connector 체결 시 board support로 보드 굽힘 억제</t>
+        <t>적용 규격·개정 / 허용 기준 / 실측값 / 시험·사진 번호</t>
       </text>
     </comment>
     <comment ref="B11" authorId="0" shapeId="0">
       <text>
-        <t>현행 데이터시트 대조로 공통 기준을 포함했습니다.
-이전 샘플 문구:
-AOI, LCR/IR; crack 의심 Lot 단면 또는 비파괴 검사</t>
+        <t>실제 납품업체 / PO·납품 번호 / 제조 Lot·Date Code / 입고일</t>
+      </text>
+    </comment>
+    <comment ref="B12" authorId="0" shapeId="0">
+      <text>
+        <t>확정 불량 / 의심 수량 / 재고·공정품·기출하 / 격리 위치</t>
+      </text>
+    </comment>
+    <comment ref="B13" authorId="0" shapeId="0">
+      <text>
+        <t>기판 기능 결과 / 재작업·폐기 판정 / 근거 번호</t>
+      </text>
+    </comment>
+    <comment ref="B14" authorId="0" shapeId="0">
+      <text>
+        <t>통보·접수 확인 일시 / 실제 회신 일시 / 관련 대책서 번호</t>
+      </text>
+    </comment>
+    <comment ref="B15" authorId="0" shapeId="0">
+      <text>
+        <t>정지·재개 확인자와 시각 / 공수·폐기 수량 / 비용 증빙</t>
       </text>
     </comment>
   </commentList>
 </comments>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>20</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5905500" cy="2857500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>20</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5905500" cy="2857500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>User</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+부품 검토자료 · 시스템 자동 기입</t>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0">
+      <text>
+        <t>데이터시트의 공급사 정보입니다. 해당 불량품의 실제 납품업체·귀책과 연결되지 않습니다.</t>
+      </text>
+    </comment>
+    <comment ref="B9" authorId="0" shapeId="0">
+      <text>
+        <t>현행 데이터시트 대조로 공통 기준을 포함했습니다.
+이전 샘플 문구:
+외관/단자, 0603·100V·X7R 확인, LCR·절연저항 샘플</t>
+      </text>
+    </comment>
+    <comment ref="E9" authorId="0" shapeId="0">
+      <text>
+        <t>현행 데이터시트 대조로 공통 기준을 포함했습니다.
+이전 샘플 문구:
+크랙/IR 저하는 Lot·패널 위치별 격리, 보드 굴곡·분리·프로브 지지 조건을 재현하고 공정 조건 수정</t>
+      </text>
+    </comment>
+    <comment ref="B10" authorId="0" shapeId="0">
+      <text>
+        <t>현행 데이터시트 대조로 공통 기준을 포함했습니다.
+이전 샘플 문구:
+land/reflow 준수; panel depanel·ICT probe·connector 체결 시 board support로 보드 굽힘 억제</t>
+      </text>
+    </comment>
+    <comment ref="B11" authorId="0" shapeId="0">
+      <text>
+        <t>현행 데이터시트 대조로 공통 기준을 포함했습니다.
+이전 샘플 문구:
+AOI, LCR/IR; crack 의심 Lot 단면 또는 비파괴 검사</t>
+      </text>
+    </comment>
+    <comment ref="A12" authorId="0" shapeId="0">
+      <text>
+        <t>이전 v2 내용(참고):
+Checklist 공통·부품별 항목을 함께 조회 · 원인·적합성 판단은 관리자 작성</t>
+      </text>
+    </comment>
+    <comment ref="A18" authorId="0" shapeId="0">
+      <text>
+        <t>같은 부품 타입의 후보 목록이며 대체 승인 목록이 아닙니다. 원본 데이터시트에서 MPN별 정격·공급사·가격을 확인합니다.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1817,7 +2396,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00243D5B"/>
+    <tabColor rgb="00233D59"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
@@ -1839,7 +2418,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="17" customHeight="1">
-      <c r="A1" s="89" t="inlineStr">
+      <c r="A1" s="156" t="inlineStr">
         <is>
           <t>불 량 대 책 서</t>
         </is>
@@ -1864,25 +2443,25 @@
       <c r="L1" s="119" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="G2" s="120" t="n"/>
-      <c r="H2" s="121" t="n"/>
-      <c r="I2" s="120" t="n"/>
-      <c r="J2" s="121" t="n"/>
-      <c r="K2" s="120" t="n"/>
-      <c r="L2" s="121" t="n"/>
+      <c r="G2" s="190" t="n"/>
+      <c r="H2" s="157" t="n"/>
+      <c r="I2" s="190" t="n"/>
+      <c r="J2" s="157" t="n"/>
+      <c r="K2" s="190" t="n"/>
+      <c r="L2" s="157" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="G3" s="122" t="n"/>
-      <c r="H3" s="123" t="n"/>
-      <c r="I3" s="122" t="n"/>
-      <c r="J3" s="123" t="n"/>
-      <c r="K3" s="122" t="n"/>
-      <c r="L3" s="123" t="n"/>
-    </row>
-    <row r="4" ht="12" customHeight="1">
-      <c r="A4" s="124" t="inlineStr">
-        <is>
-          <t>시스템 자동 기입 · 발행 시점 고정  |  담당·기한·문서 상태는 관리자 갱신</t>
+      <c r="G3" s="158" t="n"/>
+      <c r="H3" s="159" t="n"/>
+      <c r="I3" s="158" t="n"/>
+      <c r="J3" s="159" t="n"/>
+      <c r="K3" s="158" t="n"/>
+      <c r="L3" s="159" t="n"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="194" t="inlineStr">
+        <is>
+          <t>01  발생 사실 · 시스템 자동 기입  |  확정 불량 개별 건 발행  /  가상 종결 예시</t>
         </is>
       </c>
     </row>
@@ -1893,9 +2472,9 @@
         </is>
       </c>
       <c r="B5" s="119" t="n"/>
-      <c r="C5" s="125" t="inlineStr">
-        <is>
-          <t>QA-CAP-CRACK-20260819-001</t>
+      <c r="C5" s="195" t="inlineStr">
+        <is>
+          <t>QA-D9001-CAP-CRACK</t>
         </is>
       </c>
       <c r="D5" s="126" t="n"/>
@@ -1908,9 +2487,9 @@
         </is>
       </c>
       <c r="I5" s="119" t="n"/>
-      <c r="J5" s="127" t="inlineStr">
-        <is>
-          <t>2026-08-19 09:00:00</t>
+      <c r="J5" s="198" t="inlineStr">
+        <is>
+          <t>2026-09-07 12:05:00</t>
         </is>
       </c>
       <c r="K5" s="126" t="n"/>
@@ -1923,9 +2502,9 @@
         </is>
       </c>
       <c r="B6" s="119" t="n"/>
-      <c r="C6" s="125" t="inlineStr">
-        <is>
-          <t>CAP  (MLCC)</t>
+      <c r="C6" s="195" t="inlineStr">
+        <is>
+          <t>CAP · Contoso CX-0603X7R104K100 (MLCC)</t>
         </is>
       </c>
       <c r="D6" s="126" t="n"/>
@@ -1938,7 +2517,7 @@
         </is>
       </c>
       <c r="I6" s="119" t="n"/>
-      <c r="J6" s="127" t="inlineStr">
+      <c r="J6" s="198" t="inlineStr">
         <is>
           <t>CRACK</t>
         </is>
@@ -1953,28 +2532,28 @@
         </is>
       </c>
       <c r="B7" s="119" t="n"/>
-      <c r="C7" s="128" t="inlineStr">
-        <is>
-          <t>품질보증팀 김OO</t>
-        </is>
-      </c>
-      <c r="D7" s="129" t="n"/>
-      <c r="E7" s="129" t="n"/>
-      <c r="F7" s="129" t="n"/>
-      <c r="G7" s="130" t="n"/>
+      <c r="C7" s="199" t="inlineStr">
+        <is>
+          <t>품질보증 김OO</t>
+        </is>
+      </c>
+      <c r="D7" s="161" t="n"/>
+      <c r="E7" s="161" t="n"/>
+      <c r="F7" s="161" t="n"/>
+      <c r="G7" s="162" t="n"/>
       <c r="H7" s="118" t="inlineStr">
         <is>
           <t>협조 부서</t>
         </is>
       </c>
       <c r="I7" s="119" t="n"/>
-      <c r="J7" s="131" t="inlineStr">
-        <is>
-          <t>설비팀 · 생산팀 · 구매</t>
-        </is>
-      </c>
-      <c r="K7" s="129" t="n"/>
-      <c r="L7" s="130" t="n"/>
+      <c r="J7" s="202" t="inlineStr">
+        <is>
+          <t>생산기술 · 구매</t>
+        </is>
+      </c>
+      <c r="K7" s="161" t="n"/>
+      <c r="L7" s="162" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="118" t="inlineStr">
@@ -1983,9 +2562,10 @@
         </is>
       </c>
       <c r="B8" s="119" t="n"/>
-      <c r="C8" s="125" t="inlineStr">
-        <is>
-          <t>Job 7112 · Unit 10412 · CAP-02</t>
+      <c r="C8" s="203" t="inlineStr">
+        <is>
+          <t>Job 12345678-1234-5678-1234-567812345678
+Unit 103 · CAP-02</t>
         </is>
       </c>
       <c r="D8" s="126" t="n"/>
@@ -1998,85 +2578,84 @@
         </is>
       </c>
       <c r="I8" s="119" t="n"/>
-      <c r="J8" s="127" t="inlineStr">
-        <is>
-          <t>2026-08-18 16:30:12</t>
+      <c r="J8" s="198" t="inlineStr">
+        <is>
+          <t>2026-09-07 12:00:00</t>
         </is>
       </c>
       <c r="K8" s="126" t="n"/>
       <c r="L8" s="119" t="n"/>
     </row>
-    <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="132" t="inlineStr">
-        <is>
-          <t>상태  CLOSED  ·  ①~⑥ 작성 완료  ·  발행 기준: 확정 불량 1건</t>
-        </is>
-      </c>
-      <c r="B9" s="129" t="n"/>
-      <c r="C9" s="129" t="n"/>
-      <c r="D9" s="129" t="n"/>
-      <c r="E9" s="129" t="n"/>
-      <c r="F9" s="129" t="n"/>
-      <c r="G9" s="129" t="n"/>
-      <c r="H9" s="129" t="n"/>
-      <c r="I9" s="129" t="n"/>
-      <c r="J9" s="129" t="n"/>
-      <c r="K9" s="129" t="n"/>
-      <c r="L9" s="130" t="n"/>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="164" t="inlineStr">
+        <is>
+          <t>문서 상태: 종결  |  확정 불량 1건 확인에 따른 통보 · 조치 실행 여부는 담당자 확인</t>
+        </is>
+      </c>
+      <c r="B9" s="161" t="n"/>
+      <c r="C9" s="161" t="n"/>
+      <c r="D9" s="161" t="n"/>
+      <c r="E9" s="161" t="n"/>
+      <c r="F9" s="161" t="n"/>
+      <c r="G9" s="161" t="n"/>
+      <c r="H9" s="161" t="n"/>
+      <c r="I9" s="161" t="n"/>
+      <c r="J9" s="161" t="n"/>
+      <c r="K9" s="161" t="n"/>
+      <c r="L9" s="162" t="n"/>
     </row>
     <row r="10" ht="6" customHeight="1"/>
     <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="118" t="inlineStr">
-        <is>
-          <t>부품 검사 수량</t>
-        </is>
-      </c>
-      <c r="B11" s="126" t="n"/>
-      <c r="C11" s="119" t="n"/>
-      <c r="D11" s="118" t="inlineStr">
-        <is>
-          <t>불량 건수</t>
-        </is>
-      </c>
-      <c r="E11" s="126" t="n"/>
-      <c r="F11" s="119" t="n"/>
-      <c r="G11" s="118" t="inlineStr">
-        <is>
-          <t>발행 PPM</t>
-        </is>
-      </c>
-      <c r="H11" s="126" t="n"/>
-      <c r="I11" s="119" t="n"/>
-      <c r="J11" s="118" t="inlineStr">
-        <is>
-          <t>검증 PPM(계산)</t>
-        </is>
-      </c>
-      <c r="K11" s="126" t="n"/>
-      <c r="L11" s="119" t="n"/>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="133" t="n">
-        <v>12500</v>
-      </c>
-      <c r="B12" s="126" t="n"/>
-      <c r="C12" s="119" t="n"/>
-      <c r="D12" s="133" t="n">
-        <v>16</v>
-      </c>
-      <c r="E12" s="126" t="n"/>
-      <c r="F12" s="119" t="n"/>
-      <c r="G12" s="133" t="n">
-        <v>1280</v>
-      </c>
-      <c r="H12" s="126" t="n"/>
-      <c r="I12" s="119" t="n"/>
-      <c r="J12" s="134">
-        <f>IF(AND(ISNUMBER(G25),ISNUMBER(I25),G25&gt;0),I25/G25*1000000,"")</f>
-        <v/>
-      </c>
-      <c r="K12" s="135" t="n"/>
-      <c r="L12" s="136" t="n"/>
+      <c r="A11" s="167" t="inlineStr">
+        <is>
+          <t>02  실제 납품업체 · 당사 작성</t>
+        </is>
+      </c>
+      <c r="B11" s="204" t="n"/>
+      <c r="C11" s="204" t="n"/>
+      <c r="D11" s="205" t="n"/>
+      <c r="E11" s="167" t="inlineStr">
+        <is>
+          <t>거래처 회신 책임자 · 당사 작성</t>
+        </is>
+      </c>
+      <c r="F11" s="204" t="n"/>
+      <c r="G11" s="204" t="n"/>
+      <c r="H11" s="205" t="n"/>
+      <c r="I11" s="167" t="inlineStr">
+        <is>
+          <t>초기 회신 기한 · 당사 작성</t>
+        </is>
+      </c>
+      <c r="J11" s="204" t="n"/>
+      <c r="K11" s="204" t="n"/>
+      <c r="L11" s="205" t="n"/>
+    </row>
+    <row r="12" ht="25" customHeight="1">
+      <c r="A12" s="168" t="inlineStr">
+        <is>
+          <t>예시 납품업체 A (가상)</t>
+        </is>
+      </c>
+      <c r="B12" s="237" t="n"/>
+      <c r="C12" s="237" t="n"/>
+      <c r="D12" s="238" t="n"/>
+      <c r="E12" s="169" t="inlineStr">
+        <is>
+          <t>이OO / 품질담당</t>
+        </is>
+      </c>
+      <c r="F12" s="237" t="n"/>
+      <c r="G12" s="237" t="n"/>
+      <c r="H12" s="238" t="n"/>
+      <c r="I12" s="169" t="inlineStr">
+        <is>
+          <t>2026-09-08 12:00 KST</t>
+        </is>
+      </c>
+      <c r="J12" s="237" t="n"/>
+      <c r="K12" s="237" t="n"/>
+      <c r="L12" s="238" t="n"/>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="118" t="inlineStr">
@@ -2085,9 +2664,10 @@
         </is>
       </c>
       <c r="B13" s="119" t="n"/>
-      <c r="C13" s="127" t="inlineStr">
-        <is>
-          <t>2026-08-12 ~ 08-19  (7일 / ROLLING)</t>
+      <c r="C13" s="198" t="inlineStr">
+        <is>
+          <t>2026-09-07 10:00:00
+~ 2026-09-07 12:00:00 (발행 시점 누적)</t>
         </is>
       </c>
       <c r="D13" s="126" t="n"/>
@@ -2100,55 +2680,44 @@
         </is>
       </c>
       <c r="I13" s="119" t="n"/>
-      <c r="J13" s="127" t="inlineStr">
-        <is>
-          <t>mock-v3</t>
+      <c r="J13" s="198" t="inlineStr">
+        <is>
+          <t>assembly-r1</t>
         </is>
       </c>
       <c r="K13" s="126" t="n"/>
       <c r="L13" s="119" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="118" t="inlineStr">
-        <is>
-          <t>발생 위치</t>
-        </is>
-      </c>
-      <c r="B14" s="119" t="n"/>
-      <c r="C14" s="127" t="inlineStr">
-        <is>
-          <t>CAP-02 (발행 대상)
-전체 분포: 불량 근거</t>
-        </is>
-      </c>
-      <c r="D14" s="126" t="n"/>
-      <c r="E14" s="126" t="n"/>
-      <c r="F14" s="119" t="n"/>
-      <c r="G14" s="118" t="inlineStr">
-        <is>
-          <t>완제품 영향</t>
-        </is>
-      </c>
-      <c r="H14" s="119" t="n"/>
-      <c r="I14" s="127" t="inlineStr">
-        <is>
-          <t>2,500대 중 15대 (0.60%)</t>
-        </is>
-      </c>
-      <c r="J14" s="126" t="n"/>
-      <c r="K14" s="126" t="n"/>
-      <c r="L14" s="119" t="n"/>
+      <c r="A14" s="208" t="inlineStr">
+        <is>
+          <t>누적 참고 | 부품 검사 500건 · 불량 3건 · 6,000 PPM · 불량 Unit 100대 중 3대</t>
+        </is>
+      </c>
+      <c r="B14" s="204" t="n"/>
+      <c r="C14" s="204" t="n"/>
+      <c r="D14" s="204" t="n"/>
+      <c r="E14" s="204" t="n"/>
+      <c r="F14" s="204" t="n"/>
+      <c r="G14" s="204" t="n"/>
+      <c r="H14" s="204" t="n"/>
+      <c r="I14" s="204" t="n"/>
+      <c r="J14" s="204" t="n"/>
+      <c r="K14" s="204" t="n"/>
+      <c r="L14" s="205" t="n"/>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="118" t="inlineStr">
         <is>
-          <t>자동 분석</t>
+          <t>확인 사실</t>
         </is>
       </c>
       <c r="B15" s="119" t="n"/>
-      <c r="C15" s="127" t="inlineStr">
-        <is>
-          <t>확정 불량 1건으로 발행. 동일 Job·부품·유형 누적 16건 중 CAP-02·CAP-04에 13건 집중. 원인은 자동 추정하지 않으며 담당자가 이미지·품질 기준을 확인.</t>
+      <c r="C15" s="198" t="inlineStr">
+        <is>
+          <t>확정 불량 9001: Unit 103, CAP-02 슬롯에서 CRACK이 확인됐다.
+발행 시점까지 동일 Job·부품·유형 누적 3건이다.
+원인은 자동 추정하지 않으며 담당자가 검사 이미지와 품질기준을 확인한다.</t>
         </is>
       </c>
       <c r="D15" s="126" t="n"/>
@@ -2163,9 +2732,9 @@
     </row>
     <row r="16" ht="6" customHeight="1"/>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="137" t="inlineStr">
-        <is>
-          <t>관리자 직접 작성  |  ①~⑥ 조치·원인·대책·검증·종결 (예시)</t>
+      <c r="A17" s="211" t="inlineStr">
+        <is>
+          <t>03  조치 및 회신  |  당사 작성 → 거래처·조치부서 회신 → 당사 검증</t>
         </is>
       </c>
       <c r="B17" s="126" t="n"/>
@@ -2183,136 +2752,144 @@
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="118" t="inlineStr">
         <is>
-          <t>① 초동 조치</t>
+          <t>① 당사
+초동·요청</t>
         </is>
       </c>
       <c r="B18" s="138" t="n"/>
-      <c r="C18" s="139" t="inlineStr">
-        <is>
-          <t>■ 생산 중단    ■ 출하 보류    ■ 재고 선별    □ 고객 통보    □ 설비 정지</t>
-        </is>
-      </c>
-      <c r="D18" s="129" t="n"/>
-      <c r="E18" s="129" t="n"/>
-      <c r="F18" s="129" t="n"/>
-      <c r="G18" s="129" t="n"/>
-      <c r="H18" s="129" t="n"/>
-      <c r="I18" s="129" t="n"/>
-      <c r="J18" s="129" t="n"/>
-      <c r="K18" s="129" t="n"/>
-      <c r="L18" s="130" t="n"/>
+      <c r="C18" s="212" t="inlineStr">
+        <is>
+          <t>요청  □ 생산 보류  □ 출하 보류  □ 격리·선별  □ 원인 분석  □ 기존 대책 연계</t>
+        </is>
+      </c>
+      <c r="D18" s="161" t="n"/>
+      <c r="E18" s="161" t="n"/>
+      <c r="F18" s="161" t="n"/>
+      <c r="G18" s="161" t="n"/>
+      <c r="H18" s="161" t="n"/>
+      <c r="I18" s="161" t="n"/>
+      <c r="J18" s="161" t="n"/>
+      <c r="K18" s="161" t="n"/>
+      <c r="L18" s="162" t="n"/>
     </row>
     <row r="19" ht="58" customHeight="1">
       <c r="A19" s="140" t="n"/>
       <c r="B19" s="141" t="n"/>
-      <c r="C19" s="128" t="inlineStr">
-        <is>
-          <t>08-19 10:20 CAP-02·CAP-04 정지(생산팀장 승인). 08-16 이후 Job 7112~7139 / Unit 10388~10604, 2,500대 출하 보류.
-전수 재검 9건 추가, 누적 25건 / 24대 격리. mock-v3h 적용 후 10:50 생산 재개, 당일 18:00 재발 없음. 출하 전으로 고객 통보 제외.</t>
-        </is>
-      </c>
-      <c r="D19" s="129" t="n"/>
-      <c r="E19" s="129" t="n"/>
-      <c r="F19" s="129" t="n"/>
-      <c r="G19" s="129" t="n"/>
-      <c r="H19" s="129" t="n"/>
-      <c r="I19" s="129" t="n"/>
-      <c r="J19" s="129" t="n"/>
-      <c r="K19" s="129" t="n"/>
-      <c r="L19" s="130" t="n"/>
+      <c r="C19" s="199" t="inlineStr">
+        <is>
+          <t>CAP-02 공정 보류 요청 09-07 12:10 / 생산팀 정지 확인 12:15.
+Unit 101~103 격리. 공급사 분석 요청, 당사 품질팀이 공정 영향 병행 확인.
+초기 회신 09-08 12:00 / 원인·대책 09-10 17:00. 관련 문서: QA-D8999-CAP-CRACK.</t>
+        </is>
+      </c>
+      <c r="D19" s="161" t="n"/>
+      <c r="E19" s="161" t="n"/>
+      <c r="F19" s="161" t="n"/>
+      <c r="G19" s="161" t="n"/>
+      <c r="H19" s="161" t="n"/>
+      <c r="I19" s="161" t="n"/>
+      <c r="J19" s="161" t="n"/>
+      <c r="K19" s="161" t="n"/>
+      <c r="L19" s="162" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="118" t="inlineStr">
         <is>
-          <t>② 발생 원인</t>
+          <t>② 회신
+발생 원인</t>
         </is>
       </c>
       <c r="B20" s="138" t="n"/>
-      <c r="C20" s="142" t="inlineStr">
-        <is>
-          <t>배치 하강속도 상향 + 지지 핀 최원거리 슬롯</t>
-        </is>
-      </c>
-      <c r="D20" s="129" t="n"/>
-      <c r="E20" s="129" t="n"/>
-      <c r="F20" s="129" t="n"/>
-      <c r="G20" s="129" t="n"/>
-      <c r="H20" s="129" t="n"/>
-      <c r="I20" s="129" t="n"/>
-      <c r="J20" s="129" t="n"/>
-      <c r="K20" s="129" t="n"/>
-      <c r="L20" s="130" t="n"/>
-    </row>
-    <row r="21" ht="56" customHeight="1">
+      <c r="C20" s="213" t="inlineStr">
+        <is>
+          <t>당사 공정 기인 확인 · 공급업체 귀책 미확정 → 근거 없음</t>
+        </is>
+      </c>
+      <c r="D20" s="161" t="n"/>
+      <c r="E20" s="161" t="n"/>
+      <c r="F20" s="161" t="n"/>
+      <c r="G20" s="161" t="n"/>
+      <c r="H20" s="161" t="n"/>
+      <c r="I20" s="161" t="n"/>
+      <c r="J20" s="161" t="n"/>
+      <c r="K20" s="161" t="n"/>
+      <c r="L20" s="162" t="n"/>
+    </row>
+    <row r="21" ht="52" customHeight="1">
       <c r="A21" s="140" t="n"/>
       <c r="B21" s="141" t="n"/>
-      <c r="C21" s="128" t="inlineStr">
-        <is>
-          <t>mock-v3 하강속도 18→32 mm/s·파지력 3.0→4.0 N 상향과 지지 핀에서 먼 슬롯의 보드 굽힘이 원인.
-CAP-02·CAP-04 피크력 6.8 N(타 슬롯 4.0 N, 1.7배). mock-v3h 복귀 후 재발 중단. 입고 Lot 4개에 고르게 발생해 Lot 요인 배제.</t>
-        </is>
-      </c>
-      <c r="D21" s="129" t="n"/>
-      <c r="E21" s="129" t="n"/>
-      <c r="F21" s="129" t="n"/>
-      <c r="G21" s="129" t="n"/>
-      <c r="H21" s="129" t="n"/>
-      <c r="I21" s="129" t="n"/>
-      <c r="J21" s="129" t="n"/>
-      <c r="K21" s="129" t="n"/>
-      <c r="L21" s="130" t="n"/>
-    </row>
-    <row r="22" ht="53" customHeight="1">
+      <c r="C21" s="213" t="inlineStr">
+        <is>
+          <t>생산기술 회신: 보드 지지 조건에 따른 굽힘이 크랙 발생에 기여.
+지지 유무 비교 시험에서 재현하고 조건 복원 시 미발생(FA-01).
+거래처 회신: 보관 시료 검사 이상 없음(FA-02). 납품품 자체 결함은 확인되지 않음.</t>
+        </is>
+      </c>
+      <c r="D21" s="161" t="n"/>
+      <c r="E21" s="161" t="n"/>
+      <c r="F21" s="161" t="n"/>
+      <c r="G21" s="161" t="n"/>
+      <c r="H21" s="161" t="n"/>
+      <c r="I21" s="161" t="n"/>
+      <c r="J21" s="161" t="n"/>
+      <c r="K21" s="161" t="n"/>
+      <c r="L21" s="162" t="n"/>
+    </row>
+    <row r="22" ht="48" customHeight="1">
       <c r="A22" s="118" t="inlineStr">
         <is>
-          <t>③ 유출 원인</t>
+          <t>③ 회신
+유출 원인</t>
         </is>
       </c>
       <c r="B22" s="119" t="n"/>
-      <c r="C22" s="128" t="inlineStr">
-        <is>
-          <t>인라인 AOI는 단자 들뜸·외관 결손만 판정해 미세 굽힘 크랙을 검출하지 못함. 품질 기준의 단면·비파괴 검사는 인라인에 없고 주 1회 샘플 검사만 시행.
-08-16 생산분의 크랙을 08-18 16:30에 검출.</t>
-        </is>
-      </c>
-      <c r="D22" s="129" t="n"/>
-      <c r="E22" s="129" t="n"/>
-      <c r="F22" s="129" t="n"/>
-      <c r="G22" s="129" t="n"/>
-      <c r="H22" s="129" t="n"/>
-      <c r="I22" s="129" t="n"/>
-      <c r="J22" s="129" t="n"/>
-      <c r="K22" s="129" t="n"/>
-      <c r="L22" s="130" t="n"/>
-    </row>
-    <row r="23" ht="55" customHeight="1">
+      <c r="C22" s="213" t="inlineStr">
+        <is>
+          <t>당사 검사 검토: 기존 검사 항목에서 미세 크랙 검출 조건 누락.
+누락 지점과 검출 조건을 비교 검증(FA-03).
+거래처 출하검사 유출 여부는 입증되지 않아 별도 귀책을 확정하지 않음.</t>
+        </is>
+      </c>
+      <c r="D22" s="161" t="n"/>
+      <c r="E22" s="161" t="n"/>
+      <c r="F22" s="161" t="n"/>
+      <c r="G22" s="161" t="n"/>
+      <c r="H22" s="161" t="n"/>
+      <c r="I22" s="161" t="n"/>
+      <c r="J22" s="161" t="n"/>
+      <c r="K22" s="161" t="n"/>
+      <c r="L22" s="162" t="n"/>
+    </row>
+    <row r="23" ht="48" customHeight="1">
       <c r="A23" s="118" t="inlineStr">
         <is>
-          <t>④ 재발방지
-대책</t>
+          <t>④ 회신
+영구 대책</t>
         </is>
       </c>
       <c r="B23" s="119" t="n"/>
-      <c r="C23" s="128" t="inlineStr">
-        <is>
-          <t>mock-v4: 하강속도 20 mm/s·파지력 3.2 N 적용(ECN-2608-114 승인 08-21, 적용 08-29).
-CAP-02·CAP-04 지지 핀 2개 추가(설비팀, 08-28), IND-01·IND-02 수평전개. 후보 2종은 표준 단자로 크랙 개선 근거가 없어 부품 교체 제외.</t>
-        </is>
-      </c>
-      <c r="D23" s="129" t="n"/>
-      <c r="E23" s="129" t="n"/>
-      <c r="F23" s="129" t="n"/>
-      <c r="G23" s="129" t="n"/>
-      <c r="H23" s="129" t="n"/>
-      <c r="I23" s="129" t="n"/>
-      <c r="J23" s="129" t="n"/>
-      <c r="K23" s="129" t="n"/>
-      <c r="L23" s="130" t="n"/>
+      <c r="C23" s="213" t="inlineStr">
+        <is>
+          <t>생산기술: 보드 지지 조건과 검사 기준 보완, 09-10 적용(ECN-01).
+적용 레시피 assembly-r2 / 적용 시작 Unit 104 / 담당 박OO.
+동일 지지 구조 공정 점검 완료. 구매 부품 변경 없음.</t>
+        </is>
+      </c>
+      <c r="D23" s="161" t="n"/>
+      <c r="E23" s="161" t="n"/>
+      <c r="F23" s="161" t="n"/>
+      <c r="G23" s="161" t="n"/>
+      <c r="H23" s="161" t="n"/>
+      <c r="I23" s="161" t="n"/>
+      <c r="J23" s="161" t="n"/>
+      <c r="K23" s="161" t="n"/>
+      <c r="L23" s="162" t="n"/>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="118" t="inlineStr">
         <is>
-          <t>⑤ 효과 검증</t>
+          <t>⑤ 당사
+효과 검증</t>
         </is>
       </c>
       <c r="B24" s="138" t="n"/>
@@ -2350,52 +2927,51 @@
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="143" t="n"/>
       <c r="B25" s="144" t="n"/>
-      <c r="C25" s="145" t="inlineStr">
-        <is>
-          <t>08-29 ~ 09-12</t>
-        </is>
-      </c>
-      <c r="D25" s="130" t="n"/>
-      <c r="E25" s="145" t="inlineStr">
-        <is>
-          <t>mock-v4</t>
-        </is>
-      </c>
-      <c r="F25" s="130" t="n"/>
-      <c r="G25" s="146" t="n">
-        <v>24500</v>
-      </c>
-      <c r="H25" s="130" t="n"/>
-      <c r="I25" s="146" t="n">
-        <v>3</v>
-      </c>
-      <c r="J25" s="130" t="n"/>
-      <c r="K25" s="145" t="inlineStr">
+      <c r="C25" s="214" t="inlineStr">
+        <is>
+          <t>09-10 ~ 09-14</t>
+        </is>
+      </c>
+      <c r="D25" s="162" t="n"/>
+      <c r="E25" s="214" t="inlineStr">
+        <is>
+          <t>assembly-r2</t>
+        </is>
+      </c>
+      <c r="F25" s="162" t="n"/>
+      <c r="G25" s="215" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H25" s="162" t="n"/>
+      <c r="I25" s="215" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="162" t="n"/>
+      <c r="K25" s="214" t="inlineStr">
         <is>
           <t>EFFECTIVE</t>
         </is>
       </c>
-      <c r="L25" s="130" t="n"/>
+      <c r="L25" s="162" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="143" t="n"/>
       <c r="B26" s="144" t="n"/>
       <c r="C26" s="118" t="inlineStr">
         <is>
-          <t>불량률(자동 계산)</t>
+          <t>불량률 · 자동 계산</t>
         </is>
       </c>
       <c r="D26" s="126" t="n"/>
       <c r="E26" s="119" t="n"/>
-      <c r="F26" s="147">
+      <c r="F26" s="216">
         <f>IF(AND(ISNUMBER(G25),ISNUMBER(I25),G25&gt;0),I25/G25,"")</f>
         <v/>
       </c>
-      <c r="G26" s="136" t="n"/>
-      <c r="H26" s="148" t="inlineStr">
-        <is>
-          <t>검증 수량: 부품 검사 건수 기준</t>
-        </is>
+      <c r="G26" s="119" t="n"/>
+      <c r="H26" s="217">
+        <f>IF(AND(ISNUMBER(G25),ISNUMBER(I25),G25&gt;0),"검증 PPM  "&amp;TEXT(I25/G25*1000000,"#,##0"),"검증 PPM  —")</f>
+        <v/>
       </c>
       <c r="I26" s="126" t="n"/>
       <c r="J26" s="126" t="n"/>
@@ -2405,25 +2981,27 @@
     <row r="27" ht="32" customHeight="1">
       <c r="A27" s="140" t="n"/>
       <c r="B27" s="141" t="n"/>
-      <c r="C27" s="128" t="inlineStr">
-        <is>
-          <t>24,500건 중 3건, 122 PPM으로 기준 400 PPM의 0.31배. 최소 검사 건수 충족, 대책 전 대비 10.5배 개선. CAP-02·CAP-04 집중도 해소.</t>
-        </is>
-      </c>
-      <c r="D27" s="129" t="n"/>
-      <c r="E27" s="129" t="n"/>
-      <c r="F27" s="129" t="n"/>
-      <c r="G27" s="129" t="n"/>
-      <c r="H27" s="129" t="n"/>
-      <c r="I27" s="129" t="n"/>
-      <c r="J27" s="129" t="n"/>
-      <c r="K27" s="129" t="n"/>
-      <c r="L27" s="130" t="n"/>
+      <c r="C27" s="199" t="inlineStr">
+        <is>
+          <t>동일 조건 1,000건 검사, 크랙 0건. 합의 검증 기준 충족(검증기록 V-01).
+품질 김OO 확인 / 잔여 위험은 추적 관리.</t>
+        </is>
+      </c>
+      <c r="D27" s="161" t="n"/>
+      <c r="E27" s="161" t="n"/>
+      <c r="F27" s="161" t="n"/>
+      <c r="G27" s="161" t="n"/>
+      <c r="H27" s="161" t="n"/>
+      <c r="I27" s="161" t="n"/>
+      <c r="J27" s="161" t="n"/>
+      <c r="K27" s="161" t="n"/>
+      <c r="L27" s="162" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="118" t="inlineStr">
         <is>
-          <t>⑥ 종결</t>
+          <t>⑥ 당사
+승인·종결</t>
         </is>
       </c>
       <c r="B28" s="138" t="n"/>
@@ -2433,16 +3011,16 @@
         </is>
       </c>
       <c r="D28" s="119" t="n"/>
-      <c r="E28" s="128" t="inlineStr">
+      <c r="E28" s="199" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="F28" s="129" t="n"/>
-      <c r="G28" s="130" t="n"/>
+      <c r="F28" s="161" t="n"/>
+      <c r="G28" s="162" t="n"/>
       <c r="H28" s="149" t="inlineStr">
         <is>
-          <t>잔여 위험 · 이관 사항 확인</t>
+          <t>재개·출하 승인 및 잔여 사항</t>
         </is>
       </c>
       <c r="I28" s="126" t="n"/>
@@ -2453,106 +3031,102 @@
     <row r="29" ht="40" customHeight="1">
       <c r="A29" s="140" t="n"/>
       <c r="B29" s="141" t="n"/>
-      <c r="C29" s="128" t="inlineStr">
-        <is>
-          <t>영구대책 효과 확인으로 종결. 보드 리비전 변경 시 지지 핀 재검토 필요. AOI 기준 보완은 QA-PROC-2609-003으로 이관.</t>
-        </is>
-      </c>
-      <c r="D29" s="129" t="n"/>
-      <c r="E29" s="129" t="n"/>
-      <c r="F29" s="129" t="n"/>
-      <c r="G29" s="129" t="n"/>
-      <c r="H29" s="129" t="n"/>
-      <c r="I29" s="129" t="n"/>
-      <c r="J29" s="129" t="n"/>
-      <c r="K29" s="129" t="n"/>
-      <c r="L29" s="130" t="n"/>
+      <c r="C29" s="199" t="inlineStr">
+        <is>
+          <t>09-10 공정 재개: 생산팀장 승인 / 09-14 출하 보류 해제: 품질팀장 승인.
+격리품 처분은 별도 기록. 공급업체 배상 청구 없음.</t>
+        </is>
+      </c>
+      <c r="D29" s="161" t="n"/>
+      <c r="E29" s="161" t="n"/>
+      <c r="F29" s="161" t="n"/>
+      <c r="G29" s="161" t="n"/>
+      <c r="H29" s="161" t="n"/>
+      <c r="I29" s="161" t="n"/>
+      <c r="J29" s="161" t="n"/>
+      <c r="K29" s="161" t="n"/>
+      <c r="L29" s="162" t="n"/>
     </row>
     <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="150" t="inlineStr">
-        <is>
-          <t>노랑: 관리자 작성 · 파랑: 자동 계산 · 그 외: 시스템 기입 / 종결 내용은 가상 예시·상세 원문은 메모</t>
+      <c r="A30" s="180" t="inlineStr">
+        <is>
+          <t>연녹색: 자동 기입·자동 계산  |  연노랑: 수동 작성(당사·거래처) / 가상 예시</t>
         </is>
       </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
-  <mergeCells count="75">
+  <mergeCells count="70">
     <mergeCell ref="C27:L27"/>
     <mergeCell ref="J6:L6"/>
-    <mergeCell ref="I14:L14"/>
-    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="E28:G28"/>
     <mergeCell ref="K25:L25"/>
+    <mergeCell ref="H26:L26"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="C23:L23"/>
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="C6:G6"/>
+    <mergeCell ref="K24:L24"/>
     <mergeCell ref="E24:F24"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="H26:L26"/>
     <mergeCell ref="K2:L3"/>
     <mergeCell ref="C5:G5"/>
     <mergeCell ref="A18:B19"/>
-    <mergeCell ref="A12:C12"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="J11:L11"/>
     <mergeCell ref="J7:L7"/>
     <mergeCell ref="C19:L19"/>
-    <mergeCell ref="E28:G28"/>
     <mergeCell ref="A20:B21"/>
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C18:L18"/>
     <mergeCell ref="C25:D25"/>
     <mergeCell ref="I25:J25"/>
+    <mergeCell ref="E12:H12"/>
     <mergeCell ref="K1:L1"/>
-    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="A14:L14"/>
     <mergeCell ref="C15:L15"/>
     <mergeCell ref="A17:L17"/>
-    <mergeCell ref="J12:L12"/>
+    <mergeCell ref="A11:D11"/>
     <mergeCell ref="F26:G26"/>
-    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="I11:L11"/>
     <mergeCell ref="A4:L4"/>
     <mergeCell ref="A28:B29"/>
     <mergeCell ref="G24:H24"/>
+    <mergeCell ref="A24:B27"/>
+    <mergeCell ref="G2:H3"/>
+    <mergeCell ref="I24:J24"/>
     <mergeCell ref="H7:I7"/>
-    <mergeCell ref="G2:H3"/>
-    <mergeCell ref="A24:B27"/>
-    <mergeCell ref="I24:J24"/>
     <mergeCell ref="I2:J3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C29:L29"/>
     <mergeCell ref="J8:L8"/>
+    <mergeCell ref="C20:L20"/>
     <mergeCell ref="H28:L28"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="G14:H14"/>
     <mergeCell ref="A9:L9"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="C20:L20"/>
     <mergeCell ref="A23:B23"/>
+    <mergeCell ref="H13:I13"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="C8:G8"/>
-    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="A22:B22"/>
     <mergeCell ref="I1:J1"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="G11:I11"/>
     <mergeCell ref="J5:L5"/>
     <mergeCell ref="A30:L30"/>
     <mergeCell ref="C7:G7"/>
-    <mergeCell ref="A11:C11"/>
     <mergeCell ref="C22:L22"/>
     <mergeCell ref="E25:F25"/>
+    <mergeCell ref="J13:L13"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="G25:H25"/>
     <mergeCell ref="G1:H1"/>
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="I12:L12"/>
     <mergeCell ref="A1:F3"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="C26:E26"/>
     <mergeCell ref="A13:B13"/>
-    <mergeCell ref="H5:I5"/>
     <mergeCell ref="C21:L21"/>
-    <mergeCell ref="C26:E26"/>
-    <mergeCell ref="C28:D28"/>
     <mergeCell ref="H8:I8"/>
-    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="E11:H11"/>
   </mergeCells>
   <conditionalFormatting sqref="K25:L25">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
@@ -2565,7 +3139,7 @@
       <formula>"PENDING"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="18">
+  <dataValidations count="19">
     <dataValidation sqref="J6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="허용되지 않는 값" error="다음 중 하나여야 한다: MISSING,POSITION_ERROR,ORIENTATION_ERROR,CRACK" promptTitle="불량 유형" prompt="참고 시트 2개은 유형과 무관하게 항상 첨부한다.&#10;어느 자료가 이번 건에 쓸모 있는지는 담당자가 판단한다." type="list">
       <formula1>"MISSING,POSITION_ERROR,ORIENTATION_ERROR,CRACK"</formula1>
     </dataValidation>
@@ -2592,6 +3166,9 @@
     <dataValidation sqref="C27" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑤ 판정 근거" prompt="재집계 결과를 그렇게 읽은 이유.&#10;"/>
     <dataValidation sqref="E28" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑥ 종결일" prompt=""/>
     <dataValidation sqref="C29" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="0" promptTitle="⑥ 종결 의견" prompt="잔여 위험과 종결 승인 의견.&#10;"/>
+    <dataValidation sqref="G25 I25" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="수량 확인" error="0 이상의 정수를 입력하세요." type="whole" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.32" right="0.32" top="0.32" bottom="0.32" header="0.1" footer="0.1"/>
@@ -2603,410 +3180,365 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00627083"/>
+    <tabColor rgb="00233D59"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="151" t="inlineStr">
-        <is>
-          <t>불량 근거 · 시스템 자동 기입 / 발행 시점 고정</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="69" t="inlineStr">
-        <is>
-          <t>production.unit_defects 확정 기록 · 문서번호 QA-CAP-CRACK-20260819-001 · 수정 금지</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="70" t="inlineStr">
-        <is>
-          <t>슬롯별 발생 분포        어느 슬롯에 몰려 있는지 · 공정 원인 판단의 1차 근거</t>
-        </is>
-      </c>
-      <c r="B3" s="36" t="n"/>
-      <c r="C3" s="36" t="n"/>
-      <c r="D3" s="36" t="n"/>
-      <c r="E3" s="30" t="n"/>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="71" t="inlineStr">
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="181" t="inlineStr">
+        <is>
+          <t>불량 근거 및 납품 추적</t>
+        </is>
+      </c>
+      <c r="B1" s="239" t="n"/>
+      <c r="C1" s="239" t="n"/>
+      <c r="D1" s="239" t="n"/>
+      <c r="E1" s="240" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="182" t="inlineStr">
+        <is>
+          <t>연녹색: 시스템 자동 기입 · 연노랑: 담당자 수동 작성 / 가상 예시</t>
+        </is>
+      </c>
+      <c r="B2" s="239" t="n"/>
+      <c r="C2" s="239" t="n"/>
+      <c r="D2" s="239" t="n"/>
+      <c r="E2" s="240" t="n"/>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="185" t="inlineStr">
+        <is>
+          <t>01  발행 대상 · 시스템 자동 기입</t>
+        </is>
+      </c>
+      <c r="B3" s="241" t="n"/>
+      <c r="C3" s="241" t="n"/>
+      <c r="D3" s="241" t="n"/>
+      <c r="E3" s="242" t="n"/>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="218" t="inlineStr">
+        <is>
+          <t>문서 QA-D9001-CAP-CRACK · 불량 ID 9001 · Unit 103</t>
+        </is>
+      </c>
+      <c r="B4" s="209" t="n"/>
+      <c r="C4" s="209" t="n"/>
+      <c r="D4" s="209" t="n"/>
+      <c r="E4" s="210" t="n"/>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="218" t="inlineStr">
+        <is>
+          <t>슬롯 CAP-02 · CRACK · 검사 2026-09-07 12:00:00</t>
+        </is>
+      </c>
+      <c r="B5" s="209" t="n"/>
+      <c r="C5" s="209" t="n"/>
+      <c r="D5" s="209" t="n"/>
+      <c r="E5" s="210" t="n"/>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="185" t="inlineStr">
+        <is>
+          <t>02  동일 Job·부품·유형 누적 · 발행 시점 참고</t>
+        </is>
+      </c>
+      <c r="B6" s="241" t="n"/>
+      <c r="C6" s="241" t="n"/>
+      <c r="D6" s="241" t="n"/>
+      <c r="E6" s="242" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="167" t="inlineStr">
         <is>
           <t>슬롯</t>
         </is>
       </c>
-      <c r="B4" s="71" t="inlineStr">
+      <c r="B7" s="167" t="inlineStr">
         <is>
           <t>불량 건수</t>
         </is>
       </c>
-      <c r="C4" s="71" t="inlineStr">
+      <c r="C7" s="167" t="inlineStr">
         <is>
           <t>슬롯 불량률</t>
         </is>
       </c>
-      <c r="D4" s="71" t="inlineStr">
-        <is>
-          <t>비고</t>
-        </is>
-      </c>
-      <c r="E4" s="30" t="n"/>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="72" t="inlineStr">
+      <c r="D7" s="167" t="inlineStr">
+        <is>
+          <t>집계 기준</t>
+        </is>
+      </c>
+      <c r="E7" s="167" t="inlineStr">
+        <is>
+          <t>해석</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="66" customHeight="1">
+      <c r="A8" s="208" t="inlineStr">
         <is>
           <t>CAP-02</t>
         </is>
       </c>
-      <c r="B5" s="73" t="n">
-        <v>8</v>
-      </c>
-      <c r="C5" s="74" t="n">
-        <v>0.0032</v>
-      </c>
-      <c r="D5" s="75" t="inlineStr">
-        <is>
-          <t>상위 2슬롯 81.3% · 공정/설비 우선 의심</t>
-        </is>
-      </c>
-      <c r="E5" s="30" t="n"/>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="72" t="inlineStr">
-        <is>
-          <t>CAP-04</t>
-        </is>
-      </c>
-      <c r="B6" s="73" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" s="74" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="D6" s="32" t="n"/>
-      <c r="E6" s="30" t="n"/>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="72" t="inlineStr">
-        <is>
-          <t>CAP-01</t>
-        </is>
-      </c>
-      <c r="B7" s="73" t="n">
-        <v>2</v>
-      </c>
-      <c r="C7" s="74" t="n">
-        <v>0.0008</v>
-      </c>
-      <c r="D7" s="32" t="n"/>
-      <c r="E7" s="30" t="n"/>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="72" t="inlineStr">
-        <is>
-          <t>CAP-05</t>
-        </is>
-      </c>
-      <c r="B8" s="73" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="74" t="n">
-        <v>0.0004</v>
-      </c>
-      <c r="D8" s="32" t="n"/>
-      <c r="E8" s="30" t="n"/>
-    </row>
-    <row r="9" ht="30" customHeight="1"/>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="70" t="inlineStr">
-        <is>
-          <t>불량 유닛 목록</t>
-        </is>
-      </c>
-      <c r="B10" s="36" t="n"/>
-      <c r="C10" s="36" t="n"/>
-      <c r="D10" s="36" t="n"/>
-      <c r="E10" s="30" t="n"/>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="71" t="inlineStr">
-        <is>
-          <t>unit_id</t>
-        </is>
-      </c>
-      <c r="B11" s="71" t="inlineStr">
-        <is>
-          <t>슬롯</t>
-        </is>
-      </c>
-      <c r="C11" s="71" t="inlineStr">
-        <is>
-          <t>불량 유형</t>
-        </is>
-      </c>
-      <c r="D11" s="71" t="inlineStr">
-        <is>
-          <t>검사 시각</t>
-        </is>
-      </c>
-      <c r="E11" s="71" t="inlineStr">
-        <is>
-          <t>검사 이미지 경로</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="72" t="n">
-        <v>10412</v>
-      </c>
-      <c r="B12" s="72" t="inlineStr">
-        <is>
-          <t>CAP-02</t>
-        </is>
-      </c>
-      <c r="C12" s="72" t="inlineStr">
-        <is>
-          <t>CRACK</t>
-        </is>
-      </c>
-      <c r="D12" s="72" t="inlineStr">
-        <is>
-          <t>2026-08-18 16:30:12</t>
-        </is>
-      </c>
-      <c r="E12" s="75" t="inlineStr">
-        <is>
-          <t>/var/lib/inspect/2026-08-18/u10412.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="72" t="n">
-        <v>10418</v>
-      </c>
-      <c r="B13" s="72" t="inlineStr">
-        <is>
-          <t>CAP-04</t>
-        </is>
-      </c>
-      <c r="C13" s="72" t="inlineStr">
-        <is>
-          <t>CRACK</t>
-        </is>
-      </c>
-      <c r="D13" s="72" t="inlineStr">
-        <is>
-          <t>2026-08-18 16:41:55</t>
-        </is>
-      </c>
-      <c r="E13" s="75" t="inlineStr">
-        <is>
-          <t>/var/lib/inspect/2026-08-18/u10418.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="72" t="n">
-        <v>10425</v>
-      </c>
-      <c r="B14" s="72" t="inlineStr">
-        <is>
-          <t>CAP-02</t>
-        </is>
-      </c>
-      <c r="C14" s="72" t="inlineStr">
-        <is>
-          <t>CRACK</t>
-        </is>
-      </c>
-      <c r="D14" s="72" t="inlineStr">
-        <is>
-          <t>2026-08-18 17:02:30</t>
-        </is>
-      </c>
-      <c r="E14" s="75" t="inlineStr">
-        <is>
-          <t>/var/lib/inspect/2026-08-18/u10425.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="72" t="n">
-        <v>10431</v>
-      </c>
-      <c r="B15" s="72" t="inlineStr">
-        <is>
-          <t>CAP-02</t>
-        </is>
-      </c>
-      <c r="C15" s="72" t="inlineStr">
-        <is>
-          <t>CRACK</t>
-        </is>
-      </c>
-      <c r="D15" s="72" t="inlineStr">
-        <is>
-          <t>2026-08-18 17:19:08</t>
-        </is>
-      </c>
-      <c r="E15" s="75" t="inlineStr">
-        <is>
-          <t>/var/lib/inspect/2026-08-18/u10431.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="72" t="n">
-        <v>10447</v>
-      </c>
-      <c r="B16" s="72" t="inlineStr">
-        <is>
-          <t>CAP-04</t>
-        </is>
-      </c>
-      <c r="C16" s="72" t="inlineStr">
-        <is>
-          <t>CRACK</t>
-        </is>
-      </c>
-      <c r="D16" s="72" t="inlineStr">
-        <is>
-          <t>2026-08-18 18:03:41</t>
-        </is>
-      </c>
-      <c r="E16" s="75" t="inlineStr">
-        <is>
-          <t>/var/lib/inspect/2026-08-18/u10447.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="72" t="inlineStr">
-        <is>
-          <t>…</t>
-        </is>
-      </c>
-      <c r="B17" s="72" t="inlineStr">
-        <is>
-          <t>…</t>
-        </is>
-      </c>
-      <c r="C17" s="72" t="inlineStr">
-        <is>
-          <t>…</t>
-        </is>
-      </c>
-      <c r="D17" s="72" t="inlineStr">
-        <is>
-          <t>…</t>
-        </is>
-      </c>
-      <c r="E17" s="75" t="inlineStr">
-        <is>
-          <t>총 16행 · 발행 시점 스냅샷</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1"/>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="70" t="inlineStr">
-        <is>
-          <t>검사 이미지</t>
-        </is>
-      </c>
-      <c r="B19" s="36" t="n"/>
-      <c r="C19" s="36" t="n"/>
-      <c r="D19" s="36" t="n"/>
-      <c r="E19" s="30" t="n"/>
-    </row>
-    <row r="20" ht="44" customHeight="1">
-      <c r="A20" s="76" t="inlineStr">
-        <is>
-          <t>샘플 이미지 미포함 · InspectionSamples/mock-fail.jpg · SHA-256 —</t>
-        </is>
-      </c>
-      <c r="B20" s="36" t="n"/>
-      <c r="C20" s="36" t="n"/>
-      <c r="D20" s="36" t="n"/>
-      <c r="E20" s="30" t="n"/>
-    </row>
-    <row r="21" ht="40" customHeight="1">
-      <c r="A21" s="34" t="n"/>
-      <c r="B21" s="77" t="n"/>
-      <c r="C21" s="77" t="n"/>
-      <c r="D21" s="77" t="n"/>
-      <c r="E21" s="78" t="n"/>
-    </row>
-    <row r="22" ht="40" customHeight="1">
-      <c r="A22" s="79" t="n"/>
-      <c r="E22" s="80" t="n"/>
-    </row>
-    <row r="23" ht="40" customHeight="1">
-      <c r="A23" s="79" t="n"/>
-      <c r="E23" s="80" t="n"/>
-    </row>
-    <row r="24" ht="40" customHeight="1">
-      <c r="A24" s="79" t="n"/>
-      <c r="E24" s="80" t="n"/>
-    </row>
-    <row r="25" ht="40" customHeight="1">
-      <c r="A25" s="79" t="n"/>
-      <c r="E25" s="80" t="n"/>
-    </row>
-    <row r="26" ht="40" customHeight="1">
-      <c r="A26" s="81" t="n"/>
-      <c r="B26" s="82" t="n"/>
-      <c r="C26" s="82" t="n"/>
-      <c r="D26" s="82" t="n"/>
-      <c r="E26" s="83" t="n"/>
+      <c r="B8" s="208" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C8" s="208" t="inlineStr">
+        <is>
+          <t>3.00%</t>
+        </is>
+      </c>
+      <c r="D8" s="208" t="inlineStr">
+        <is>
+          <t>발행 시점까지 동일 Job·부품·유형 누적</t>
+        </is>
+      </c>
+      <c r="E8" s="182" t="inlineStr">
+        <is>
+          <t>전체 폐기·공급사 귀책을 뜻하지 않음</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="185" t="inlineStr">
+        <is>
+          <t>03  판정·납품 추적 · 당사 담당자 작성</t>
+        </is>
+      </c>
+      <c r="B9" s="241" t="n"/>
+      <c r="C9" s="241" t="n"/>
+      <c r="D9" s="241" t="n"/>
+      <c r="E9" s="242" t="n"/>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="185" t="inlineStr">
+        <is>
+          <t>판정 근거</t>
+        </is>
+      </c>
+      <c r="B10" s="169" t="inlineStr">
+        <is>
+          <t>예시 사내 기준 Q-01 rev.1: 크랙 불허 / 현미경 크랙 확인 / FA-01</t>
+        </is>
+      </c>
+      <c r="C10" s="206" t="n"/>
+      <c r="D10" s="206" t="n"/>
+      <c r="E10" s="207" t="n"/>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="185" t="inlineStr">
+        <is>
+          <t>납품 추적</t>
+        </is>
+      </c>
+      <c r="B11" s="169" t="inlineStr">
+        <is>
+          <t>예시 납품업체 A / PO-DEMO-01 / Lot DEMO-01 / 2026-09-01</t>
+        </is>
+      </c>
+      <c r="C11" s="206" t="n"/>
+      <c r="D11" s="206" t="n"/>
+      <c r="E11" s="207" t="n"/>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="185" t="inlineStr">
+        <is>
+          <t>영향·격리</t>
+        </is>
+      </c>
+      <c r="B12" s="169" t="inlineStr">
+        <is>
+          <t>확정 불량 Unit 3대 / 3대 격리. 그 외 의심 범위는 추적 기록 참조.</t>
+        </is>
+      </c>
+      <c r="C12" s="206" t="n"/>
+      <c r="D12" s="206" t="n"/>
+      <c r="E12" s="207" t="n"/>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="185" t="inlineStr">
+        <is>
+          <t>기능·처분</t>
+        </is>
+      </c>
+      <c r="B13" s="169" t="inlineStr">
+        <is>
+          <t>기판 기능 손실·폐기는 자동 판정하지 않음. 처분 기록 DISP-01 참조.</t>
+        </is>
+      </c>
+      <c r="C13" s="206" t="n"/>
+      <c r="D13" s="206" t="n"/>
+      <c r="E13" s="207" t="n"/>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="185" t="inlineStr">
+        <is>
+          <t>접수·회신</t>
+        </is>
+      </c>
+      <c r="B14" s="169" t="inlineStr">
+        <is>
+          <t>09-07 통보 / 09-08 접수·초기 회신 확인 / 관련 QA-D8999-CAP-CRACK</t>
+        </is>
+      </c>
+      <c r="C14" s="206" t="n"/>
+      <c r="D14" s="206" t="n"/>
+      <c r="E14" s="207" t="n"/>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="185" t="inlineStr">
+        <is>
+          <t>정지·손실</t>
+        </is>
+      </c>
+      <c r="B15" s="169" t="inlineStr">
+        <is>
+          <t>생산팀 09-07 정지 확인 / 09-10 재개 승인. 비용·공수는 증빙 COST-01.</t>
+        </is>
+      </c>
+      <c r="C15" s="206" t="n"/>
+      <c r="D15" s="206" t="n"/>
+      <c r="E15" s="207" t="n"/>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="185" t="inlineStr">
+        <is>
+          <t>04  검사 이미지 · 시스템 첨부</t>
+        </is>
+      </c>
+      <c r="B16" s="241" t="n"/>
+      <c r="C16" s="241" t="n"/>
+      <c r="D16" s="241" t="n"/>
+      <c r="E16" s="242" t="n"/>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="219" t="inlineStr">
+        <is>
+          <t>가상 예시 · 실제 검사 이미지 미첨부 · —
+SHA-256 —</t>
+        </is>
+      </c>
+      <c r="B17" s="209" t="n"/>
+      <c r="C17" s="209" t="n"/>
+      <c r="D17" s="209" t="n"/>
+      <c r="E17" s="210" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="218" t="inlineStr">
+        <is>
+          <t>가상 종결 예시 · 실제 검사 이미지는 포함하지 않았습니다.</t>
+        </is>
+      </c>
+      <c r="B18" s="220" t="n"/>
+      <c r="C18" s="220" t="n"/>
+      <c r="D18" s="220" t="n"/>
+      <c r="E18" s="221" t="n"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="222" t="n"/>
+      <c r="B19" s="223" t="n"/>
+      <c r="C19" s="223" t="n"/>
+      <c r="D19" s="223" t="n"/>
+      <c r="E19" s="224" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="222" t="n"/>
+      <c r="B20" s="223" t="n"/>
+      <c r="C20" s="223" t="n"/>
+      <c r="D20" s="223" t="n"/>
+      <c r="E20" s="224" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="222" t="n"/>
+      <c r="B21" s="223" t="n"/>
+      <c r="C21" s="223" t="n"/>
+      <c r="D21" s="223" t="n"/>
+      <c r="E21" s="224" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="222" t="n"/>
+      <c r="B22" s="223" t="n"/>
+      <c r="C22" s="223" t="n"/>
+      <c r="D22" s="223" t="n"/>
+      <c r="E22" s="224" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="225" t="n"/>
+      <c r="B23" s="226" t="n"/>
+      <c r="C23" s="226" t="n"/>
+      <c r="D23" s="226" t="n"/>
+      <c r="E23" s="227" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0"/>
-  <mergeCells count="12">
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="A20:E20"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
+  <mergeCells count="32">
+    <mergeCell ref="A8"/>
+    <mergeCell ref="C8"/>
+    <mergeCell ref="C7"/>
+    <mergeCell ref="D8"/>
+    <mergeCell ref="E7"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A10"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A13"/>
+    <mergeCell ref="A18:E23"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A15"/>
+    <mergeCell ref="B7"/>
+    <mergeCell ref="A11"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="E8"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="A21:E26"/>
-    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="A7"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B8"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A12"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="D7"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="A14"/>
+    <mergeCell ref="A9:E9"/>
   </mergeCells>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.32" right="0.32" top="0.45" bottom="0.45" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 &amp;K627083v2 · 불량 근거&amp;R&amp;8 &amp;K627083&amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8 &amp;K627083v2 · 불량 근거&amp;C&amp;8 연녹색: 자동 | 연노랑: 수동&amp;R&amp;8 &amp;K627083&amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="008296AD"/>
+    <tabColor rgb="008797A7"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
@@ -3022,85 +3554,95 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="152" t="inlineStr">
-        <is>
-          <t>부품 검토자료 · 시스템 자동 기입</t>
+      <c r="A1" s="187" t="inlineStr">
+        <is>
+          <t>부품 검토자료 · 내부 참고</t>
         </is>
       </c>
     </row>
     <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="85" t="inlineStr">
+      <c r="A2" s="228" t="inlineStr">
         <is>
           <t>부품 범주 MLCC · 대조 일치 · 기준일 2026-08-18 · 현행 자료 조회 2026-09-07 14:00:58</t>
         </is>
       </c>
+      <c r="B2" s="223" t="n"/>
+      <c r="C2" s="223" t="n"/>
+      <c r="D2" s="223" t="n"/>
+      <c r="E2" s="223" t="n"/>
+      <c r="F2" s="223" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="53" t="inlineStr">
+      <c r="A3" s="243" t="inlineStr">
         <is>
           <t>현재 부품  |  데이터시트 대조</t>
         </is>
       </c>
+      <c r="B3" s="244" t="n"/>
+      <c r="C3" s="244" t="n"/>
+      <c r="D3" s="244" t="n"/>
+      <c r="E3" s="244" t="n"/>
+      <c r="F3" s="244" t="n"/>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="49" t="inlineStr">
+      <c r="A4" s="229" t="inlineStr">
         <is>
           <t>현재 MPN</t>
         </is>
       </c>
-      <c r="B4" s="49" t="inlineStr">
+      <c r="B4" s="229" t="inlineStr">
         <is>
           <t>핵심 정격</t>
         </is>
       </c>
-      <c r="C4" s="49" t="inlineStr">
-        <is>
-          <t>공급사</t>
-        </is>
-      </c>
-      <c r="D4" s="153" t="inlineStr">
+      <c r="C4" s="229" t="inlineStr">
+        <is>
+          <t>자료상 공급사</t>
+        </is>
+      </c>
+      <c r="D4" s="230" t="inlineStr">
         <is>
           <t>단가(USD)</t>
         </is>
       </c>
-      <c r="E4" s="49" t="inlineStr">
+      <c r="E4" s="229" t="inlineStr">
         <is>
           <t>가격 기준 수량</t>
         </is>
       </c>
-      <c r="F4" s="49" t="inlineStr">
+      <c r="F4" s="229" t="inlineStr">
         <is>
           <t>가격 확인일</t>
         </is>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1">
-      <c r="A5" s="50" t="inlineStr">
+      <c r="A5" s="231" t="inlineStr">
         <is>
           <t>Contoso CX-0603X7R104K100</t>
         </is>
       </c>
-      <c r="B5" s="50" t="inlineStr">
+      <c r="B5" s="231" t="inlineStr">
         <is>
           <t>0.10µF ±10% 100V X7R 0603</t>
         </is>
       </c>
-      <c r="C5" s="50" t="inlineStr">
+      <c r="C5" s="231" t="inlineStr">
         <is>
           <t>Northwind Traders</t>
         </is>
       </c>
-      <c r="D5" s="50" t="inlineStr">
+      <c r="D5" s="232" t="inlineStr">
         <is>
           <t>$0.15</t>
         </is>
       </c>
-      <c r="E5" s="50" t="inlineStr">
+      <c r="E5" s="231" t="inlineStr">
         <is>
           <t>1개 (Cut Tape)</t>
         </is>
       </c>
-      <c r="F5" s="50" t="inlineStr">
+      <c r="F5" s="231" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
@@ -3115,78 +3657,97 @@
       <c r="F6" s="52" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="53" t="inlineStr">
+      <c r="A7" s="243" t="inlineStr">
         <is>
           <t>품질 체크리스트  |  공통 기준 + 부품별 기준</t>
         </is>
       </c>
+      <c r="B7" s="244" t="n"/>
+      <c r="C7" s="244" t="n"/>
+      <c r="D7" s="244" t="n"/>
+      <c r="E7" s="244" t="n"/>
+      <c r="F7" s="244" t="n"/>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="49" t="inlineStr">
+      <c r="A8" s="229" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="B8" s="49" t="inlineStr">
+      <c r="B8" s="229" t="inlineStr">
         <is>
           <t>확인 항목</t>
         </is>
       </c>
-      <c r="E8" s="49" t="inlineStr">
+      <c r="C8" s="244" t="n"/>
+      <c r="D8" s="244" t="n"/>
+      <c r="E8" s="229" t="inlineStr">
         <is>
           <t>이상 시 조치</t>
         </is>
       </c>
+      <c r="F8" s="244" t="n"/>
     </row>
     <row r="9" ht="72" customHeight="1">
-      <c r="A9" s="49" t="inlineStr">
+      <c r="A9" s="229" t="inlineStr">
         <is>
           <t>입고 검사</t>
         </is>
       </c>
-      <c r="B9" s="154" t="inlineStr">
+      <c r="B9" s="233" t="inlineStr">
         <is>
           <t>승인 공급처, PO/BOM-MPN-revision, 수량, CoC, Lot/date code, 포장·라벨·봉인 대조
 외관/단자, 0603·100V·X7R 확인, LCR·절연저항 샘플</t>
         </is>
       </c>
-      <c r="E9" s="154" t="inlineStr">
+      <c r="C9" s="223" t="n"/>
+      <c r="D9" s="223" t="n"/>
+      <c r="E9" s="233" t="inlineStr">
         <is>
           <t>Line stop → 의심 Lot 전량 격리 → 영향 범위/재공품 추적 → NCR·공급사 FA/8D·CAPA → 변경 승인 후 재검
 크랙/IR 저하는 Lot·패널 위치별 격리, 보드 굴곡·분리·프로브 지지 조건을 재현하고 공정 조건 수정</t>
         </is>
       </c>
+      <c r="F9" s="223" t="n"/>
     </row>
     <row r="10" ht="78" customHeight="1">
-      <c r="A10" s="49" t="inlineStr">
+      <c r="A10" s="229" t="inlineStr">
         <is>
           <t>조립·보관</t>
         </is>
       </c>
-      <c r="B10" s="154" t="inlineStr">
+      <c r="B10" s="233" t="inlineStr">
         <is>
           <t>격리 상태 표시, ESD/MSL/극성·온습도·노출시간 관리, FIFO, Lot 혼합 금지
 land/reflow 준수; panel depanel·ICT probe·connector 체결 시 board support로 굽힘 억제</t>
         </is>
       </c>
+      <c r="C10" s="223" t="n"/>
+      <c r="D10" s="223" t="n"/>
+      <c r="E10" s="223" t="n"/>
+      <c r="F10" s="223" t="n"/>
     </row>
     <row r="11" ht="64" customHeight="1">
-      <c r="A11" s="49" t="inlineStr">
+      <c r="A11" s="229" t="inlineStr">
         <is>
           <t>기능·신뢰성</t>
         </is>
       </c>
-      <c r="B11" s="154" t="inlineStr">
+      <c r="B11" s="233" t="inlineStr">
         <is>
           <t>초도품 승인 후 Lot별 샘플링; 검사결과와 serial/Lot 추적
 AOI, LCR/IR; crack 의심 Lot 단면 또는 비파괴 검사</t>
         </is>
       </c>
+      <c r="C11" s="223" t="n"/>
+      <c r="D11" s="223" t="n"/>
+      <c r="E11" s="223" t="n"/>
+      <c r="F11" s="223" t="n"/>
     </row>
     <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="47" t="inlineStr">
-        <is>
-          <t>Checklist 공통·부품별 항목을 함께 조회 · 원인·적합성 판단은 관리자 작성</t>
+      <c r="A12" s="188" t="inlineStr">
+        <is>
+          <t>연녹색: 데이터시트 자동 조회 · 수동 입력란 없음 · 실제 조치 결과는 담당자 확인</t>
         </is>
       </c>
     </row>
@@ -3199,121 +3760,73 @@
       <c r="F13" s="52" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="53" t="inlineStr">
+      <c r="A14" s="243" t="inlineStr">
         <is>
           <t>대체품 후보  |  적합성 검증·변경 승인 후 적용</t>
         </is>
       </c>
+      <c r="B14" s="244" t="n"/>
+      <c r="C14" s="244" t="n"/>
+      <c r="D14" s="244" t="n"/>
+      <c r="E14" s="244" t="n"/>
+      <c r="F14" s="244" t="n"/>
     </row>
     <row r="15" ht="48" customHeight="1">
-      <c r="A15" s="86" t="inlineStr">
+      <c r="A15" s="234" t="inlineStr">
         <is>
           <t>같은 부품 타입이라는 것 외에 검증된 것은 없다 · 동일 정격만으로 drop-in 판단 금지 · 핀/패키지/정격/열/수명 재검증과 변경 승인을 거친 뒤에만 적용한다.</t>
         </is>
       </c>
+      <c r="B15" s="244" t="n"/>
+      <c r="C15" s="244" t="n"/>
+      <c r="D15" s="244" t="n"/>
+      <c r="E15" s="244" t="n"/>
+      <c r="F15" s="244" t="n"/>
     </row>
     <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="85" t="inlineStr">
+      <c r="A16" s="228" t="inlineStr">
         <is>
           <t>같은 타입 후보 2종 · 단가 $0.09 ~ $0.15 · 현재 선정 $0.15 · 호환성 미승인</t>
         </is>
       </c>
+      <c r="B16" s="223" t="n"/>
+      <c r="C16" s="223" t="n"/>
+      <c r="D16" s="223" t="n"/>
+      <c r="E16" s="223" t="n"/>
+      <c r="F16" s="223" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="49" t="inlineStr">
-        <is>
-          <t>제조사 / P/N</t>
-        </is>
-      </c>
-      <c r="B17" s="49" t="inlineStr">
-        <is>
-          <t>핵심 정격</t>
-        </is>
-      </c>
-      <c r="C17" s="49" t="inlineStr">
-        <is>
-          <t>공급사</t>
-        </is>
-      </c>
-      <c r="D17" s="153" t="inlineStr">
-        <is>
-          <t>단가(USD)</t>
-        </is>
-      </c>
-      <c r="E17" s="49" t="inlineStr">
-        <is>
-          <t>가격 기준 수량</t>
-        </is>
-      </c>
-      <c r="F17" s="49" t="inlineStr">
-        <is>
-          <t>가격 확인일</t>
-        </is>
-      </c>
+      <c r="A17" s="185" t="inlineStr">
+        <is>
+          <t>검토 후보 MPN · 상세 정격·가격은 원본 Components에서 MPN으로 확인</t>
+        </is>
+      </c>
+      <c r="B17" s="241" t="n"/>
+      <c r="C17" s="241" t="n"/>
+      <c r="D17" s="241" t="n"/>
+      <c r="E17" s="241" t="n"/>
+      <c r="F17" s="242" t="n"/>
     </row>
     <row r="18" ht="50" customHeight="1">
-      <c r="A18" s="88" t="inlineStr">
-        <is>
-          <t>Litware LW-C0603-104K-100</t>
-        </is>
-      </c>
-      <c r="B18" s="88" t="inlineStr">
-        <is>
-          <t>0.10µF ±10% 100V X7R 0603</t>
-        </is>
-      </c>
-      <c r="C18" s="88" t="inlineStr">
-        <is>
-          <t>Northwind Traders</t>
-        </is>
-      </c>
-      <c r="D18" s="88" t="inlineStr">
-        <is>
-          <t>$0.12</t>
-        </is>
-      </c>
-      <c r="E18" s="88" t="inlineStr">
-        <is>
-          <t>1개 (Cut Tape)</t>
-        </is>
-      </c>
-      <c r="F18" s="88" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
+      <c r="A18" s="235" t="inlineStr">
+        <is>
+          <t>Litware LW-C0603-104K-100
+Tailspin TS-0603-104M-100</t>
+        </is>
+      </c>
+      <c r="B18" s="220" t="n"/>
+      <c r="C18" s="220" t="n"/>
+      <c r="D18" s="220" t="n"/>
+      <c r="E18" s="220" t="n"/>
+      <c r="F18" s="221" t="n"/>
     </row>
     <row r="19" ht="50" customHeight="1">
-      <c r="A19" s="50" t="inlineStr">
-        <is>
-          <t>Tailspin TS-0603-104M-100</t>
-        </is>
-      </c>
-      <c r="B19" s="50" t="inlineStr">
-        <is>
-          <t>0.10µF ±20% 100V X7R 0603</t>
-        </is>
-      </c>
-      <c r="C19" s="50" t="inlineStr">
-        <is>
-          <t>Wide World Importers</t>
-        </is>
-      </c>
-      <c r="D19" s="50" t="inlineStr">
-        <is>
-          <t>$0.09</t>
-        </is>
-      </c>
-      <c r="E19" s="50" t="inlineStr">
-        <is>
-          <t>1개 (Cut Tape)</t>
-        </is>
-      </c>
-      <c r="F19" s="50" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
+      <c r="A19" s="225" t="n"/>
+      <c r="B19" s="226" t="n"/>
+      <c r="C19" s="226" t="n"/>
+      <c r="D19" s="226" t="n"/>
+      <c r="E19" s="226" t="n"/>
+      <c r="F19" s="227" t="n"/>
     </row>
     <row r="20" ht="42" customHeight="1">
       <c r="A20" s="85" t="inlineStr">
@@ -3323,26 +3836,33 @@
       </c>
     </row>
     <row r="21" ht="38" customHeight="1">
-      <c r="A21" s="155" t="inlineStr">
+      <c r="A21" s="236" t="inlineStr">
         <is>
           <t>원본 semiconductor_assembly_quality_datasheet_2026-08-18.xlsx
 SHA-256: e35dacdde1e02dfdc620c1026147d525927b9ca22e4c5ec25c978766c806ad66</t>
         </is>
       </c>
+      <c r="B21" s="223" t="n"/>
+      <c r="C21" s="223" t="n"/>
+      <c r="D21" s="223" t="n"/>
+      <c r="E21" s="223" t="n"/>
+      <c r="F21" s="223" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
-  <mergeCells count="16">
+  <mergeCells count="18">
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A18:F19"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A15:F15"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="E9:F11"/>
+    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A21:F21"/>
@@ -3355,7 +3875,7 @@
   <pageSetup orientation="portrait" paperSize="9" scale="100"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 &amp;K627083v2 · 검토용&amp;R&amp;8 &amp;K627083&amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8 &amp;K627083v2 · 검토용&amp;C&amp;8 연녹색: 자동 | 연노랑: 수동&amp;R&amp;8 &amp;K627083&amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
chore: checkpoint before Unity visualization recovery
</commit_message>
<xml_diff>
--- a/MAIN_SERVER/templates/불량대책서_샘플_종결본_v2.xlsx
+++ b/MAIN_SERVER/templates/불량대책서_샘플_종결본_v2.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대책서" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대체품" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="reply_containment">'대책서'!$C$23</definedName>
@@ -18,6 +19,7 @@
     <definedName name="reply_closed_at">'대책서'!$I$33</definedName>
     <definedName name="reply_closure_note">'대책서'!$C$34</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'대책서'!$A$1:$L$36</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'대체품'!$A$1:$F$13</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -25,12 +27,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0&quot;배&quot;"/>
     <numFmt numFmtId="165" formatCode="0.000%"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd hh:mm"/>
-    <numFmt numFmtId="168" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd hh:mm"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="73">
     <font>
@@ -540,7 +541,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="43">
+  <borders count="53">
     <border>
       <left/>
       <right/>
@@ -989,11 +990,108 @@
         <color rgb="00A6ADB7"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00A6ADB7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00A6ADB7"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00A6ADB7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00A6ADB7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00A6ADB7"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00A6ADB7"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00A6ADB7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00A6ADB7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00A6ADB7"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00A6ADB7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00A6ADB7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00A6ADB7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00A6ADB7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00A6ADB7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00A6ADB7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <right/>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="271">
+  <cellXfs count="295">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1691,7 +1789,7 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="13" borderId="42" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="4" fillId="13" borderId="42" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -1712,12 +1810,68 @@
     <xf numFmtId="0" fontId="70" fillId="10" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="168" fontId="42" fillId="13" borderId="42" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="42" fillId="13" borderId="42" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="72" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="13" borderId="42" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="42" fillId="13" borderId="42" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="52" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="52" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="72" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2972,4 +3126,228 @@
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>현재 부품과 대체품 후보 · 가상 부품 검토 예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="289" t="inlineStr">
+        <is>
+          <t>현재 부품: CAP / Contoso CX-0603X7R104K100 / MLCC · 데이터시트 대조: 일치</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="29" t="inlineStr">
+        <is>
+          <t>현재 MPN</t>
+        </is>
+      </c>
+      <c r="B3" s="29" t="inlineStr">
+        <is>
+          <t>핵심 정격</t>
+        </is>
+      </c>
+      <c r="C3" s="29" t="inlineStr">
+        <is>
+          <t>공급사</t>
+        </is>
+      </c>
+      <c r="D3" s="29" t="inlineStr">
+        <is>
+          <t>단가 (USD)</t>
+        </is>
+      </c>
+      <c r="E3" s="29" t="inlineStr">
+        <is>
+          <t>가격 기준 수량</t>
+        </is>
+      </c>
+      <c r="F3" s="29" t="inlineStr">
+        <is>
+          <t>가격 확인일</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="50" customHeight="1">
+      <c r="A4" s="39" t="inlineStr">
+        <is>
+          <t>Contoso CX-0603X7R104K100</t>
+        </is>
+      </c>
+      <c r="B4" s="39" t="inlineStr">
+        <is>
+          <t>0.10µF ±10% 100V X7R 0603</t>
+        </is>
+      </c>
+      <c r="C4" s="39" t="inlineStr">
+        <is>
+          <t>Northwind Traders</t>
+        </is>
+      </c>
+      <c r="D4" s="40" t="inlineStr">
+        <is>
+          <t>$0.15</t>
+        </is>
+      </c>
+      <c r="E4" s="39" t="inlineStr">
+        <is>
+          <t>1개 (Cut Tape)</t>
+        </is>
+      </c>
+      <c r="F4" s="39" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="290" t="inlineStr">
+        <is>
+          <t>같은 부품 타입이라는 것 외에 검증된 것은 없다 · 동일 정격만으로 drop-in 판단 금지 · 핀/패키지/정격/열/수명 재검증과 변경 승인을 거친 뒤에만 적용한다.</t>
+        </is>
+      </c>
+      <c r="B6" s="36" t="n"/>
+      <c r="C6" s="36" t="n"/>
+      <c r="D6" s="36" t="n"/>
+      <c r="E6" s="36" t="n"/>
+      <c r="F6" s="30" t="n"/>
+    </row>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="291" t="inlineStr">
+        <is>
+          <t>후보 2종 · 조회 2026-09-09 15:20:33 · 데이터시트 기준일 2026-08-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="292" t="inlineStr">
+        <is>
+          <t>대체품 후보 목록 · 호환성 검증 및 변경 승인 후 적용</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>제조사 / P/N</t>
+        </is>
+      </c>
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>핵심 정격</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>공급사</t>
+        </is>
+      </c>
+      <c r="D9" s="29" t="inlineStr">
+        <is>
+          <t>단가 (USD)</t>
+        </is>
+      </c>
+      <c r="E9" s="29" t="inlineStr">
+        <is>
+          <t>가격 기준 수량</t>
+        </is>
+      </c>
+      <c r="F9" s="29" t="inlineStr">
+        <is>
+          <t>가격 확인일</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="100" customHeight="1">
+      <c r="A10" s="38" t="inlineStr">
+        <is>
+          <t>Litware LW-C0603-104K-100
+Tailspin TS-0603-104M-100</t>
+        </is>
+      </c>
+      <c r="B10" s="38" t="inlineStr">
+        <is>
+          <t>0.10µF ±10% 100V X7R 0603
+0.10µF ±20% 100V X7R 0603</t>
+        </is>
+      </c>
+      <c r="C10" s="38" t="inlineStr">
+        <is>
+          <t>Northwind Traders
+Wide World Importers</t>
+        </is>
+      </c>
+      <c r="D10" s="42" t="inlineStr">
+        <is>
+          <t>$0.12
+$0.09</t>
+        </is>
+      </c>
+      <c r="E10" s="38" t="inlineStr">
+        <is>
+          <t>1개 (Cut Tape)
+1개 (Cut Tape)</t>
+        </is>
+      </c>
+      <c r="F10" s="38" t="inlineStr">
+        <is>
+          <t>2026-08-14
+2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="293" t="inlineStr">
+        <is>
+          <t>단가는 데이터시트 기준일의 참고값입니다. 발주 전 구매·품질 담당자가 최신 가격·재고·납기와 적합성을 확인합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="294" t="inlineStr">
+        <is>
+          <t>원본: semiconductor_assembly_quality_datasheet_2026-08-18.xlsx
+SHA-256: e35dacdde1e02dfdc620c1026147d525927b9ca22e4c5ec25c978766c806ad66</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0"/>
+  <mergeCells count="7">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A7:F7"/>
+  </mergeCells>
+  <pageMargins left="0.35" right="0.35" top="0.45" bottom="0.45" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: snapshot current visualization and reporting changes
</commit_message>
<xml_diff>
--- a/MAIN_SERVER/templates/불량대책서_샘플_종결본_v2.xlsx
+++ b/MAIN_SERVER/templates/불량대책서_샘플_종결본_v2.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대책서" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대체품" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="검사 근거" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대체품" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="reply_containment">'대책서'!$C$23</definedName>
@@ -19,7 +20,8 @@
     <definedName name="reply_closed_at">'대책서'!$I$33</definedName>
     <definedName name="reply_closure_note">'대책서'!$C$34</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'대책서'!$A$1:$L$36</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'대체품'!$A$1:$F$13</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'검사 근거'!$A$1:$L$26</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'대체품'!$A$1:$F$13</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -33,7 +35,7 @@
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd hh:mm"/>
     <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="73">
+  <fonts count="76">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -441,6 +443,23 @@
       <name val="맑은 고딕"/>
       <color rgb="00606060"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="008C5200"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="008C5200"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="20">
@@ -1091,7 +1110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="295">
+  <cellXfs count="303">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1871,6 +1890,28 @@
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="72" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="73" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="75" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -2010,12 +2051,76 @@
   <commentList>
     <comment ref="A19" authorId="0" shapeId="0">
       <text>
-        <t>검사 이미지 경로: —
-SHA-256: —</t>
+        <t>원본: inspection_1e2f3eab-3d28-4e4b-859b-2ff37b5676f7_02_annotated_report.png
+SHA-256: db24b2e4f61367ef5e4ac5397bff03b3e9559d329a346f57db6834360f42f0df
+메인 표시: 원본 오른쪽 EVIDENCE OVERLAY의 보드 영역. 엑셀 이미지 자르기만 적용; 원본 픽셀 유지.</t>
       </text>
     </comment>
   </commentList>
 </comments>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>617634</colOff>
+      <row>14</row>
+      <rowOff>38100</rowOff>
+    </from>
+    <ext cx="2022282" cy="1600200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="의심 위치 보드 오버레이 · 미확정" descr="원본 오른쪽 보드 발췌. FINAL UNKNOWN / UNVERIFIED. 확정 불량 아님."/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" l="66816.81681681682" t="24642.85714285714" r="450.4504504504504" b="13750"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>76200</colOff>
+      <row>5</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <ext cx="9144000" cy="3844324"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2330,79 +2435,56 @@
           <t>불 량 대 책 서</t>
         </is>
       </c>
-      <c r="B1" s="246" t="n"/>
-      <c r="C1" s="246" t="n"/>
-      <c r="D1" s="246" t="n"/>
-      <c r="E1" s="246" t="n"/>
-      <c r="F1" s="246" t="n"/>
-      <c r="G1" s="246" t="n"/>
-      <c r="H1" s="246" t="n"/>
       <c r="I1" s="247" t="inlineStr">
         <is>
           <t>작성</t>
         </is>
       </c>
-      <c r="J1" s="248" t="n"/>
+      <c r="J1" s="271" t="n"/>
       <c r="K1" s="247" t="inlineStr">
         <is>
           <t>승인</t>
         </is>
       </c>
-      <c r="L1" s="248" t="n"/>
+      <c r="L1" s="271" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="246" t="n"/>
-      <c r="B2" s="246" t="n"/>
-      <c r="C2" s="246" t="n"/>
-      <c r="D2" s="246" t="n"/>
-      <c r="E2" s="246" t="n"/>
-      <c r="F2" s="246" t="n"/>
-      <c r="G2" s="246" t="n"/>
-      <c r="H2" s="246" t="n"/>
       <c r="I2" s="249" t="inlineStr">
         <is>
-          <t>김OO (예시)</t>
-        </is>
-      </c>
-      <c r="J2" s="250" t="n"/>
+          <t>작성 예시</t>
+        </is>
+      </c>
+      <c r="J2" s="272" t="n"/>
       <c r="K2" s="249" t="inlineStr">
         <is>
-          <t>최OO (예시)</t>
-        </is>
-      </c>
-      <c r="L2" s="250" t="n"/>
+          <t>승인 전</t>
+        </is>
+      </c>
+      <c r="L2" s="272" t="n"/>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="246" t="n"/>
-      <c r="B3" s="246" t="n"/>
-      <c r="C3" s="246" t="n"/>
-      <c r="D3" s="246" t="n"/>
-      <c r="E3" s="246" t="n"/>
-      <c r="F3" s="246" t="n"/>
-      <c r="G3" s="246" t="n"/>
-      <c r="H3" s="246" t="n"/>
-      <c r="I3" s="250" t="n"/>
-      <c r="J3" s="250" t="n"/>
-      <c r="K3" s="250" t="n"/>
-      <c r="L3" s="250" t="n"/>
+      <c r="I3" s="273" t="n"/>
+      <c r="J3" s="274" t="n"/>
+      <c r="K3" s="273" t="n"/>
+      <c r="L3" s="274" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="251" t="inlineStr">
         <is>
-          <t>01  발생 정보  ·  가상 종결 예시</t>
-        </is>
-      </c>
-      <c r="B4" s="252" t="n"/>
-      <c r="C4" s="252" t="n"/>
-      <c r="D4" s="252" t="n"/>
-      <c r="E4" s="252" t="n"/>
-      <c r="F4" s="252" t="n"/>
-      <c r="G4" s="252" t="n"/>
-      <c r="H4" s="252" t="n"/>
-      <c r="I4" s="252" t="n"/>
-      <c r="J4" s="252" t="n"/>
-      <c r="K4" s="252" t="n"/>
-      <c r="L4" s="252" t="n"/>
+          <t>01  발생 정보 · 판정 미확정 검토 예시</t>
+        </is>
+      </c>
+      <c r="B4" s="275" t="n"/>
+      <c r="C4" s="275" t="n"/>
+      <c r="D4" s="275" t="n"/>
+      <c r="E4" s="275" t="n"/>
+      <c r="F4" s="275" t="n"/>
+      <c r="G4" s="275" t="n"/>
+      <c r="H4" s="275" t="n"/>
+      <c r="I4" s="275" t="n"/>
+      <c r="J4" s="275" t="n"/>
+      <c r="K4" s="275" t="n"/>
+      <c r="L4" s="271" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="253" t="inlineStr">
@@ -2410,29 +2492,29 @@
           <t>문서번호</t>
         </is>
       </c>
-      <c r="B5" s="248" t="n"/>
+      <c r="B5" s="271" t="n"/>
       <c r="C5" s="254" t="inlineStr">
         <is>
-          <t>QA-D9001-CAP-CRACK</t>
-        </is>
-      </c>
-      <c r="D5" s="255" t="n"/>
-      <c r="E5" s="255" t="n"/>
-      <c r="F5" s="255" t="n"/>
-      <c r="G5" s="255" t="n"/>
-      <c r="H5" s="255" t="n"/>
+          <t>검토용 샘플 · 미발행</t>
+        </is>
+      </c>
+      <c r="D5" s="275" t="n"/>
+      <c r="E5" s="275" t="n"/>
+      <c r="F5" s="275" t="n"/>
+      <c r="G5" s="275" t="n"/>
+      <c r="H5" s="271" t="n"/>
       <c r="I5" s="253" t="inlineStr">
         <is>
           <t>문서 상태</t>
         </is>
       </c>
-      <c r="J5" s="248" t="n"/>
+      <c r="J5" s="271" t="n"/>
       <c r="K5" s="256" t="inlineStr">
         <is>
-          <t>종결</t>
-        </is>
-      </c>
-      <c r="L5" s="250" t="n"/>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="L5" s="276" t="n"/>
     </row>
     <row r="6" ht="26" customHeight="1">
       <c r="A6" s="253" t="inlineStr">
@@ -2440,21 +2522,21 @@
           <t>대상 부품</t>
         </is>
       </c>
-      <c r="B6" s="248" t="n"/>
+      <c r="B6" s="271" t="n"/>
       <c r="C6" s="257" t="inlineStr">
         <is>
-          <t>CAP · Contoso CX-0603X7R104K100 (MLCC)</t>
-        </is>
-      </c>
-      <c r="D6" s="255" t="n"/>
-      <c r="E6" s="255" t="n"/>
-      <c r="F6" s="255" t="n"/>
-      <c r="G6" s="255" t="n"/>
-      <c r="H6" s="255" t="n"/>
-      <c r="I6" s="255" t="n"/>
-      <c r="J6" s="255" t="n"/>
-      <c r="K6" s="255" t="n"/>
-      <c r="L6" s="255" t="n"/>
+          <t>SMD 커패시터 · 부품 모델명 / MPN 미확인</t>
+        </is>
+      </c>
+      <c r="D6" s="275" t="n"/>
+      <c r="E6" s="275" t="n"/>
+      <c r="F6" s="275" t="n"/>
+      <c r="G6" s="275" t="n"/>
+      <c r="H6" s="275" t="n"/>
+      <c r="I6" s="275" t="n"/>
+      <c r="J6" s="275" t="n"/>
+      <c r="K6" s="275" t="n"/>
+      <c r="L6" s="271" t="n"/>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="253" t="inlineStr">
@@ -2462,22 +2544,22 @@
           <t>발생 대상</t>
         </is>
       </c>
-      <c r="B7" s="248" t="n"/>
+      <c r="B7" s="271" t="n"/>
       <c r="C7" s="258" t="inlineStr">
         <is>
-          <t>Job 12345678-1234-5678-1234-567812345678
-Unit 103 · 슬롯 CAP-02 · 불량 ID 9001</t>
-        </is>
-      </c>
-      <c r="D7" s="255" t="n"/>
-      <c r="E7" s="255" t="n"/>
-      <c r="F7" s="255" t="n"/>
-      <c r="G7" s="255" t="n"/>
-      <c r="H7" s="255" t="n"/>
-      <c r="I7" s="255" t="n"/>
-      <c r="J7" s="255" t="n"/>
-      <c r="K7" s="255" t="n"/>
-      <c r="L7" s="255" t="n"/>
+          <t>의심 위치: smd_capacitor_01
+Job / Unit / 확정 불량 ID: 제공 자료에서 확인되지 않음</t>
+        </is>
+      </c>
+      <c r="D7" s="275" t="n"/>
+      <c r="E7" s="275" t="n"/>
+      <c r="F7" s="275" t="n"/>
+      <c r="G7" s="275" t="n"/>
+      <c r="H7" s="275" t="n"/>
+      <c r="I7" s="275" t="n"/>
+      <c r="J7" s="275" t="n"/>
+      <c r="K7" s="275" t="n"/>
+      <c r="L7" s="271" t="n"/>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="253" t="inlineStr">
@@ -2485,59 +2567,59 @@
           <t>검사일시</t>
         </is>
       </c>
-      <c r="B8" s="248" t="n"/>
+      <c r="B8" s="271" t="n"/>
       <c r="C8" s="258" t="inlineStr">
         <is>
-          <t>2026-09-07 12:00:00</t>
-        </is>
-      </c>
-      <c r="D8" s="255" t="n"/>
-      <c r="E8" s="255" t="n"/>
-      <c r="F8" s="255" t="n"/>
+          <t>미확인</t>
+        </is>
+      </c>
+      <c r="D8" s="275" t="n"/>
+      <c r="E8" s="275" t="n"/>
+      <c r="F8" s="271" t="n"/>
       <c r="G8" s="253" t="inlineStr">
         <is>
           <t>발행일시</t>
         </is>
       </c>
-      <c r="H8" s="248" t="n"/>
+      <c r="H8" s="271" t="n"/>
       <c r="I8" s="258" t="inlineStr">
         <is>
-          <t>2026-09-07 12:05:00</t>
-        </is>
-      </c>
-      <c r="J8" s="255" t="n"/>
-      <c r="K8" s="255" t="n"/>
-      <c r="L8" s="255" t="n"/>
+          <t>미발행</t>
+        </is>
+      </c>
+      <c r="J8" s="275" t="n"/>
+      <c r="K8" s="275" t="n"/>
+      <c r="L8" s="271" t="n"/>
     </row>
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="253" t="inlineStr">
         <is>
-          <t>불량 유형</t>
-        </is>
-      </c>
-      <c r="B9" s="248" t="n"/>
+          <t>의심 유형</t>
+        </is>
+      </c>
+      <c r="B9" s="271" t="n"/>
       <c r="C9" s="259" t="inlineStr">
         <is>
-          <t>CRACK</t>
-        </is>
-      </c>
-      <c r="D9" s="255" t="n"/>
-      <c r="E9" s="255" t="n"/>
-      <c r="F9" s="255" t="n"/>
+          <t>위치 이상 의심</t>
+        </is>
+      </c>
+      <c r="D9" s="275" t="n"/>
+      <c r="E9" s="275" t="n"/>
+      <c r="F9" s="271" t="n"/>
       <c r="G9" s="253" t="inlineStr">
         <is>
           <t>발행 대상</t>
         </is>
       </c>
-      <c r="H9" s="248" t="n"/>
+      <c r="H9" s="271" t="n"/>
       <c r="I9" s="260" t="inlineStr">
         <is>
-          <t>확정 불량 1건</t>
-        </is>
-      </c>
-      <c r="J9" s="255" t="n"/>
-      <c r="K9" s="255" t="n"/>
-      <c r="L9" s="255" t="n"/>
+          <t>의심 후보 1개 · 미확정</t>
+        </is>
+      </c>
+      <c r="J9" s="275" t="n"/>
+      <c r="K9" s="275" t="n"/>
+      <c r="L9" s="271" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="253" t="inlineStr">
@@ -2545,27 +2627,25 @@
           <t>주관 담당</t>
         </is>
       </c>
-      <c r="B10" s="248" t="n"/>
+      <c r="B10" s="271" t="n"/>
       <c r="C10" s="261" t="inlineStr">
         <is>
-          <t>품질보증 김OO</t>
-        </is>
-      </c>
-      <c r="D10" s="250" t="n"/>
-      <c r="E10" s="250" t="n"/>
-      <c r="F10" s="250" t="n"/>
+          <t>담당자 지정 필요</t>
+        </is>
+      </c>
+      <c r="D10" s="277" t="n"/>
+      <c r="E10" s="277" t="n"/>
+      <c r="F10" s="276" t="n"/>
       <c r="G10" s="253" t="inlineStr">
         <is>
           <t>초기 회신</t>
         </is>
       </c>
-      <c r="H10" s="248" t="n"/>
-      <c r="I10" s="262" t="n">
-        <v>46273.5</v>
-      </c>
-      <c r="J10" s="250" t="n"/>
-      <c r="K10" s="250" t="n"/>
-      <c r="L10" s="250" t="n"/>
+      <c r="H10" s="271" t="n"/>
+      <c r="I10" s="278" t="n"/>
+      <c r="J10" s="277" t="n"/>
+      <c r="K10" s="277" t="n"/>
+      <c r="L10" s="276" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="253" t="inlineStr">
@@ -2573,21 +2653,21 @@
           <t>납품 추적</t>
         </is>
       </c>
-      <c r="B11" s="248" t="n"/>
+      <c r="B11" s="271" t="n"/>
       <c r="C11" s="263" t="inlineStr">
         <is>
-          <t>예시 납품업체 A · PO-DEMO-01 · Lot DEMO-01</t>
-        </is>
-      </c>
-      <c r="D11" s="250" t="n"/>
-      <c r="E11" s="250" t="n"/>
-      <c r="F11" s="250" t="n"/>
-      <c r="G11" s="250" t="n"/>
-      <c r="H11" s="250" t="n"/>
-      <c r="I11" s="250" t="n"/>
-      <c r="J11" s="250" t="n"/>
-      <c r="K11" s="250" t="n"/>
-      <c r="L11" s="250" t="n"/>
+          <t>실제 납품업체 · Lot / PO 미확인</t>
+        </is>
+      </c>
+      <c r="D11" s="277" t="n"/>
+      <c r="E11" s="277" t="n"/>
+      <c r="F11" s="277" t="n"/>
+      <c r="G11" s="277" t="n"/>
+      <c r="H11" s="277" t="n"/>
+      <c r="I11" s="277" t="n"/>
+      <c r="J11" s="277" t="n"/>
+      <c r="K11" s="277" t="n"/>
+      <c r="L11" s="276" t="n"/>
     </row>
     <row r="12" ht="5" customHeight="1">
       <c r="A12" s="264" t="n"/>
@@ -2606,20 +2686,20 @@
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="265" t="inlineStr">
         <is>
-          <t>02  불량 현상 및 판정 근거</t>
-        </is>
-      </c>
-      <c r="B13" s="266" t="n"/>
-      <c r="C13" s="266" t="n"/>
-      <c r="D13" s="266" t="n"/>
-      <c r="E13" s="266" t="n"/>
-      <c r="F13" s="266" t="n"/>
-      <c r="G13" s="266" t="n"/>
-      <c r="H13" s="266" t="n"/>
-      <c r="I13" s="266" t="n"/>
-      <c r="J13" s="266" t="n"/>
-      <c r="K13" s="266" t="n"/>
-      <c r="L13" s="266" t="n"/>
+          <t>02  의심 현상 및 검사 근거</t>
+        </is>
+      </c>
+      <c r="B13" s="275" t="n"/>
+      <c r="C13" s="275" t="n"/>
+      <c r="D13" s="275" t="n"/>
+      <c r="E13" s="275" t="n"/>
+      <c r="F13" s="275" t="n"/>
+      <c r="G13" s="275" t="n"/>
+      <c r="H13" s="275" t="n"/>
+      <c r="I13" s="275" t="n"/>
+      <c r="J13" s="275" t="n"/>
+      <c r="K13" s="275" t="n"/>
+      <c r="L13" s="271" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="247" t="inlineStr">
@@ -2627,59 +2707,50 @@
           <t>확인 사실 · 판정 근거</t>
         </is>
       </c>
-      <c r="B14" s="248" t="n"/>
-      <c r="C14" s="248" t="n"/>
-      <c r="D14" s="248" t="n"/>
-      <c r="E14" s="248" t="n"/>
-      <c r="F14" s="248" t="n"/>
+      <c r="B14" s="275" t="n"/>
+      <c r="C14" s="275" t="n"/>
+      <c r="D14" s="275" t="n"/>
+      <c r="E14" s="275" t="n"/>
+      <c r="F14" s="271" t="n"/>
       <c r="G14" s="247" t="inlineStr">
         <is>
-          <t>해당 검사 이미지</t>
-        </is>
-      </c>
-      <c r="H14" s="248" t="n"/>
-      <c r="I14" s="248" t="n"/>
-      <c r="J14" s="248" t="n"/>
-      <c r="K14" s="248" t="n"/>
-      <c r="L14" s="248" t="n"/>
+          <t>의심 위치 · 판정 미확정</t>
+        </is>
+      </c>
+      <c r="H14" s="275" t="n"/>
+      <c r="I14" s="275" t="n"/>
+      <c r="J14" s="275" t="n"/>
+      <c r="K14" s="275" t="n"/>
+      <c r="L14" s="271" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="257" t="inlineStr">
         <is>
-          <t>Unit 103 / CAP-02에서
-CRACK이 확인됨.</t>
-        </is>
-      </c>
-      <c r="B15" s="255" t="n"/>
-      <c r="C15" s="255" t="n"/>
-      <c r="D15" s="255" t="n"/>
-      <c r="E15" s="255" t="n"/>
-      <c r="F15" s="255" t="n"/>
-      <c r="G15" s="267" t="inlineStr">
-        <is>
-          <t>가상 예시
-실제 검사 이미지 미첨부</t>
-        </is>
-      </c>
-      <c r="H15" s="255" t="n"/>
-      <c r="I15" s="255" t="n"/>
-      <c r="J15" s="255" t="n"/>
-      <c r="K15" s="255" t="n"/>
-      <c r="L15" s="255" t="n"/>
+          <t>smd_capacitor_01에 위치 이상 의심 표시.
+확정 불량 판정은 제공되지 않음.</t>
+        </is>
+      </c>
+      <c r="B15" s="279" t="n"/>
+      <c r="C15" s="279" t="n"/>
+      <c r="D15" s="279" t="n"/>
+      <c r="E15" s="279" t="n"/>
+      <c r="F15" s="280" t="n"/>
+      <c r="G15" s="267" t="n"/>
+      <c r="H15" s="279" t="n"/>
+      <c r="I15" s="279" t="n"/>
+      <c r="J15" s="279" t="n"/>
+      <c r="K15" s="279" t="n"/>
+      <c r="L15" s="280" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="255" t="n"/>
-      <c r="B16" s="255" t="n"/>
-      <c r="C16" s="255" t="n"/>
-      <c r="D16" s="255" t="n"/>
-      <c r="E16" s="255" t="n"/>
-      <c r="F16" s="255" t="n"/>
-      <c r="G16" s="255" t="n"/>
-      <c r="H16" s="255" t="n"/>
-      <c r="I16" s="255" t="n"/>
-      <c r="J16" s="255" t="n"/>
-      <c r="K16" s="255" t="n"/>
-      <c r="L16" s="255" t="n"/>
+      <c r="A16" s="281" t="n"/>
+      <c r="B16" s="282" t="n"/>
+      <c r="C16" s="282" t="n"/>
+      <c r="D16" s="282" t="n"/>
+      <c r="E16" s="282" t="n"/>
+      <c r="F16" s="283" t="n"/>
+      <c r="G16" s="284" t="n"/>
+      <c r="L16" s="285" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="247" t="inlineStr">
@@ -2687,68 +2758,57 @@
           <t>판정 근거</t>
         </is>
       </c>
-      <c r="B17" s="248" t="n"/>
+      <c r="B17" s="280" t="n"/>
       <c r="C17" s="263" t="inlineStr">
         <is>
-          <t>Q-01 rev.1: 크랙 불허
-현미경 확인 (FA-01)</t>
-        </is>
-      </c>
-      <c r="D17" s="250" t="n"/>
-      <c r="E17" s="250" t="n"/>
-      <c r="F17" s="250" t="n"/>
-      <c r="G17" s="255" t="n"/>
-      <c r="H17" s="255" t="n"/>
-      <c r="I17" s="255" t="n"/>
-      <c r="J17" s="255" t="n"/>
-      <c r="K17" s="255" t="n"/>
-      <c r="L17" s="255" t="n"/>
+          <t>UNKNOWN / UNVERIFIED
+확정 판정 근거 미제공</t>
+        </is>
+      </c>
+      <c r="D17" s="286" t="n"/>
+      <c r="E17" s="286" t="n"/>
+      <c r="F17" s="272" t="n"/>
+      <c r="G17" s="284" t="n"/>
+      <c r="L17" s="285" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="248" t="n"/>
-      <c r="B18" s="248" t="n"/>
-      <c r="C18" s="250" t="n"/>
-      <c r="D18" s="250" t="n"/>
-      <c r="E18" s="250" t="n"/>
-      <c r="F18" s="250" t="n"/>
-      <c r="G18" s="255" t="n"/>
-      <c r="H18" s="255" t="n"/>
-      <c r="I18" s="255" t="n"/>
-      <c r="J18" s="255" t="n"/>
-      <c r="K18" s="255" t="n"/>
-      <c r="L18" s="255" t="n"/>
+      <c r="A18" s="281" t="n"/>
+      <c r="B18" s="283" t="n"/>
+      <c r="C18" s="273" t="n"/>
+      <c r="D18" s="287" t="n"/>
+      <c r="E18" s="287" t="n"/>
+      <c r="F18" s="274" t="n"/>
+      <c r="G18" s="284" t="n"/>
+      <c r="L18" s="285" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="268" t="inlineStr">
         <is>
-          <t>가상 예시 · 실제 검사 이미지 미첨부</t>
-        </is>
-      </c>
-      <c r="B19" s="255" t="n"/>
-      <c r="C19" s="255" t="n"/>
-      <c r="D19" s="255" t="n"/>
-      <c r="E19" s="255" t="n"/>
-      <c r="F19" s="255" t="n"/>
-      <c r="G19" s="255" t="n"/>
-      <c r="H19" s="255" t="n"/>
-      <c r="I19" s="255" t="n"/>
-      <c r="J19" s="255" t="n"/>
-      <c r="K19" s="255" t="n"/>
-      <c r="L19" s="255" t="n"/>
+          <t>오른쪽 보드 오버레이 발췌 · 미확정
+전체 진단 화면은 ‘검사 근거’ 시트 참조</t>
+        </is>
+      </c>
+      <c r="B19" s="279" t="n"/>
+      <c r="C19" s="279" t="n"/>
+      <c r="D19" s="279" t="n"/>
+      <c r="E19" s="279" t="n"/>
+      <c r="F19" s="280" t="n"/>
+      <c r="G19" s="284" t="n"/>
+      <c r="L19" s="285" t="n"/>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="255" t="n"/>
-      <c r="B20" s="255" t="n"/>
-      <c r="C20" s="255" t="n"/>
-      <c r="D20" s="255" t="n"/>
-      <c r="E20" s="255" t="n"/>
-      <c r="F20" s="255" t="n"/>
-      <c r="G20" s="255" t="n"/>
-      <c r="H20" s="255" t="n"/>
-      <c r="I20" s="255" t="n"/>
-      <c r="J20" s="255" t="n"/>
-      <c r="K20" s="255" t="n"/>
-      <c r="L20" s="255" t="n"/>
+      <c r="A20" s="281" t="n"/>
+      <c r="B20" s="282" t="n"/>
+      <c r="C20" s="282" t="n"/>
+      <c r="D20" s="282" t="n"/>
+      <c r="E20" s="282" t="n"/>
+      <c r="F20" s="283" t="n"/>
+      <c r="G20" s="281" t="n"/>
+      <c r="H20" s="282" t="n"/>
+      <c r="I20" s="282" t="n"/>
+      <c r="J20" s="282" t="n"/>
+      <c r="K20" s="282" t="n"/>
+      <c r="L20" s="283" t="n"/>
     </row>
     <row r="21" ht="5" customHeight="1">
       <c r="A21" s="264" t="n"/>
@@ -2770,17 +2830,17 @@
           <t>03  조치 · 효과 확인 · 종결</t>
         </is>
       </c>
-      <c r="B22" s="252" t="n"/>
-      <c r="C22" s="252" t="n"/>
-      <c r="D22" s="252" t="n"/>
-      <c r="E22" s="252" t="n"/>
-      <c r="F22" s="252" t="n"/>
-      <c r="G22" s="252" t="n"/>
-      <c r="H22" s="252" t="n"/>
-      <c r="I22" s="252" t="n"/>
-      <c r="J22" s="252" t="n"/>
-      <c r="K22" s="252" t="n"/>
-      <c r="L22" s="252" t="n"/>
+      <c r="B22" s="275" t="n"/>
+      <c r="C22" s="275" t="n"/>
+      <c r="D22" s="275" t="n"/>
+      <c r="E22" s="275" t="n"/>
+      <c r="F22" s="275" t="n"/>
+      <c r="G22" s="275" t="n"/>
+      <c r="H22" s="275" t="n"/>
+      <c r="I22" s="275" t="n"/>
+      <c r="J22" s="275" t="n"/>
+      <c r="K22" s="275" t="n"/>
+      <c r="L22" s="271" t="n"/>
     </row>
     <row r="23" ht="25" customHeight="1">
       <c r="A23" s="253" t="inlineStr">
@@ -2788,36 +2848,36 @@
           <t>초동조치</t>
         </is>
       </c>
-      <c r="B23" s="248" t="n"/>
+      <c r="B23" s="280" t="n"/>
       <c r="C23" s="263" t="inlineStr">
         <is>
-          <t>Unit 103 격리, 동일 조건 재공품 확인 및 공정 보류 완료 (09-07 12:15).
-담당: 생산 이OO / 납품업체 분석 요청, 영향 범위 확인 (격리기록 CT-01).</t>
-        </is>
-      </c>
-      <c r="D23" s="250" t="n"/>
-      <c r="E23" s="250" t="n"/>
-      <c r="F23" s="250" t="n"/>
-      <c r="G23" s="250" t="n"/>
-      <c r="H23" s="250" t="n"/>
-      <c r="I23" s="250" t="n"/>
-      <c r="J23" s="250" t="n"/>
-      <c r="K23" s="250" t="n"/>
-      <c r="L23" s="250" t="n"/>
+          <t>조치 계획 예시: 해당 부위 실물·검사 원본 대조 후 재검 여부 결정.
+격리·보류의 실제 수행 여부와 영향 범위는 확인 대기.</t>
+        </is>
+      </c>
+      <c r="D23" s="286" t="n"/>
+      <c r="E23" s="286" t="n"/>
+      <c r="F23" s="286" t="n"/>
+      <c r="G23" s="286" t="n"/>
+      <c r="H23" s="286" t="n"/>
+      <c r="I23" s="286" t="n"/>
+      <c r="J23" s="286" t="n"/>
+      <c r="K23" s="286" t="n"/>
+      <c r="L23" s="272" t="n"/>
     </row>
     <row r="24" ht="25" customHeight="1">
-      <c r="A24" s="248" t="n"/>
-      <c r="B24" s="248" t="n"/>
-      <c r="C24" s="250" t="n"/>
-      <c r="D24" s="250" t="n"/>
-      <c r="E24" s="250" t="n"/>
-      <c r="F24" s="250" t="n"/>
-      <c r="G24" s="250" t="n"/>
-      <c r="H24" s="250" t="n"/>
-      <c r="I24" s="250" t="n"/>
-      <c r="J24" s="250" t="n"/>
-      <c r="K24" s="250" t="n"/>
-      <c r="L24" s="250" t="n"/>
+      <c r="A24" s="281" t="n"/>
+      <c r="B24" s="283" t="n"/>
+      <c r="C24" s="273" t="n"/>
+      <c r="D24" s="287" t="n"/>
+      <c r="E24" s="287" t="n"/>
+      <c r="F24" s="287" t="n"/>
+      <c r="G24" s="287" t="n"/>
+      <c r="H24" s="287" t="n"/>
+      <c r="I24" s="287" t="n"/>
+      <c r="J24" s="287" t="n"/>
+      <c r="K24" s="287" t="n"/>
+      <c r="L24" s="274" t="n"/>
     </row>
     <row r="25" ht="25" customHeight="1">
       <c r="A25" s="253" t="inlineStr">
@@ -2825,36 +2885,35 @@
           <t>발생 원인</t>
         </is>
       </c>
-      <c r="B25" s="248" t="n"/>
+      <c r="B25" s="280" t="n"/>
       <c r="C25" s="263" t="inlineStr">
         <is>
-          <t>보드 지지 부족에 따른 굽힘으로 크랙 발생. 지지 유무 비교 시험으로 재현 (FA-01).
-당사 공정 원인 확인 / 납품업체 보관 시료 이상 없음 (FA-02).</t>
-        </is>
-      </c>
-      <c r="D25" s="250" t="n"/>
-      <c r="E25" s="250" t="n"/>
-      <c r="F25" s="250" t="n"/>
-      <c r="G25" s="250" t="n"/>
-      <c r="H25" s="250" t="n"/>
-      <c r="I25" s="250" t="n"/>
-      <c r="J25" s="250" t="n"/>
-      <c r="K25" s="250" t="n"/>
-      <c r="L25" s="250" t="n"/>
+          <t>미확정. 위치 이상 의심 표시만으로 발생 원인이나 공급사 귀책을 판단할 수 없음.</t>
+        </is>
+      </c>
+      <c r="D25" s="286" t="n"/>
+      <c r="E25" s="286" t="n"/>
+      <c r="F25" s="286" t="n"/>
+      <c r="G25" s="286" t="n"/>
+      <c r="H25" s="286" t="n"/>
+      <c r="I25" s="286" t="n"/>
+      <c r="J25" s="286" t="n"/>
+      <c r="K25" s="286" t="n"/>
+      <c r="L25" s="272" t="n"/>
     </row>
     <row r="26" ht="25" customHeight="1">
-      <c r="A26" s="248" t="n"/>
-      <c r="B26" s="248" t="n"/>
-      <c r="C26" s="250" t="n"/>
-      <c r="D26" s="250" t="n"/>
-      <c r="E26" s="250" t="n"/>
-      <c r="F26" s="250" t="n"/>
-      <c r="G26" s="250" t="n"/>
-      <c r="H26" s="250" t="n"/>
-      <c r="I26" s="250" t="n"/>
-      <c r="J26" s="250" t="n"/>
-      <c r="K26" s="250" t="n"/>
-      <c r="L26" s="250" t="n"/>
+      <c r="A26" s="281" t="n"/>
+      <c r="B26" s="283" t="n"/>
+      <c r="C26" s="273" t="n"/>
+      <c r="D26" s="287" t="n"/>
+      <c r="E26" s="287" t="n"/>
+      <c r="F26" s="287" t="n"/>
+      <c r="G26" s="287" t="n"/>
+      <c r="H26" s="287" t="n"/>
+      <c r="I26" s="287" t="n"/>
+      <c r="J26" s="287" t="n"/>
+      <c r="K26" s="287" t="n"/>
+      <c r="L26" s="274" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="253" t="inlineStr">
@@ -2862,36 +2921,35 @@
           <t>유출 원인</t>
         </is>
       </c>
-      <c r="B27" s="248" t="n"/>
+      <c r="B27" s="280" t="n"/>
       <c r="C27" s="263" t="inlineStr">
         <is>
-          <t>기존 검사에 미세 크랙 검출 조건 누락. 조건 비교 시험으로 확인 (FA-03).
-납품업체 출하검사 유출 여부는 입증되지 않음.</t>
-        </is>
-      </c>
-      <c r="D27" s="250" t="n"/>
-      <c r="E27" s="250" t="n"/>
-      <c r="F27" s="250" t="n"/>
-      <c r="G27" s="250" t="n"/>
-      <c r="H27" s="250" t="n"/>
-      <c r="I27" s="250" t="n"/>
-      <c r="J27" s="250" t="n"/>
-      <c r="K27" s="250" t="n"/>
-      <c r="L27" s="250" t="n"/>
+          <t>미확정. 보조 pose 플래그 4개와 검사 불가 항목 13개의 세부 결과 확인 필요.</t>
+        </is>
+      </c>
+      <c r="D27" s="286" t="n"/>
+      <c r="E27" s="286" t="n"/>
+      <c r="F27" s="286" t="n"/>
+      <c r="G27" s="286" t="n"/>
+      <c r="H27" s="286" t="n"/>
+      <c r="I27" s="286" t="n"/>
+      <c r="J27" s="286" t="n"/>
+      <c r="K27" s="286" t="n"/>
+      <c r="L27" s="272" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="248" t="n"/>
-      <c r="B28" s="248" t="n"/>
-      <c r="C28" s="250" t="n"/>
-      <c r="D28" s="250" t="n"/>
-      <c r="E28" s="250" t="n"/>
-      <c r="F28" s="250" t="n"/>
-      <c r="G28" s="250" t="n"/>
-      <c r="H28" s="250" t="n"/>
-      <c r="I28" s="250" t="n"/>
-      <c r="J28" s="250" t="n"/>
-      <c r="K28" s="250" t="n"/>
-      <c r="L28" s="250" t="n"/>
+      <c r="A28" s="281" t="n"/>
+      <c r="B28" s="283" t="n"/>
+      <c r="C28" s="273" t="n"/>
+      <c r="D28" s="287" t="n"/>
+      <c r="E28" s="287" t="n"/>
+      <c r="F28" s="287" t="n"/>
+      <c r="G28" s="287" t="n"/>
+      <c r="H28" s="287" t="n"/>
+      <c r="I28" s="287" t="n"/>
+      <c r="J28" s="287" t="n"/>
+      <c r="K28" s="287" t="n"/>
+      <c r="L28" s="274" t="n"/>
     </row>
     <row r="29" ht="25" customHeight="1">
       <c r="A29" s="253" t="inlineStr">
@@ -2899,36 +2957,36 @@
           <t>재발방지</t>
         </is>
       </c>
-      <c r="B29" s="248" t="n"/>
+      <c r="B29" s="280" t="n"/>
       <c r="C29" s="263" t="inlineStr">
         <is>
-          <t>보드 지지 조건 및 검사 기준 보완. 박OO / 09-10 완료 (ECN-01).
-assembly-r2, Unit 104부터 적용. 동일 구조 공정 점검 완료 / 부품 변경 없음.</t>
-        </is>
-      </c>
-      <c r="D29" s="250" t="n"/>
-      <c r="E29" s="250" t="n"/>
-      <c r="F29" s="250" t="n"/>
-      <c r="G29" s="250" t="n"/>
-      <c r="H29" s="250" t="n"/>
-      <c r="I29" s="250" t="n"/>
-      <c r="J29" s="250" t="n"/>
-      <c r="K29" s="250" t="n"/>
-      <c r="L29" s="250" t="n"/>
+          <t>원인 확인 후 담당자·기한·적용 범위를 정해 대책 수립.
+실제 대책 적용 여부는 제공 자료에서 확인되지 않음.</t>
+        </is>
+      </c>
+      <c r="D29" s="286" t="n"/>
+      <c r="E29" s="286" t="n"/>
+      <c r="F29" s="286" t="n"/>
+      <c r="G29" s="286" t="n"/>
+      <c r="H29" s="286" t="n"/>
+      <c r="I29" s="286" t="n"/>
+      <c r="J29" s="286" t="n"/>
+      <c r="K29" s="286" t="n"/>
+      <c r="L29" s="272" t="n"/>
     </row>
     <row r="30" ht="25" customHeight="1">
-      <c r="A30" s="248" t="n"/>
-      <c r="B30" s="248" t="n"/>
-      <c r="C30" s="250" t="n"/>
-      <c r="D30" s="250" t="n"/>
-      <c r="E30" s="250" t="n"/>
-      <c r="F30" s="250" t="n"/>
-      <c r="G30" s="250" t="n"/>
-      <c r="H30" s="250" t="n"/>
-      <c r="I30" s="250" t="n"/>
-      <c r="J30" s="250" t="n"/>
-      <c r="K30" s="250" t="n"/>
-      <c r="L30" s="250" t="n"/>
+      <c r="A30" s="281" t="n"/>
+      <c r="B30" s="283" t="n"/>
+      <c r="C30" s="273" t="n"/>
+      <c r="D30" s="287" t="n"/>
+      <c r="E30" s="287" t="n"/>
+      <c r="F30" s="287" t="n"/>
+      <c r="G30" s="287" t="n"/>
+      <c r="H30" s="287" t="n"/>
+      <c r="I30" s="287" t="n"/>
+      <c r="J30" s="287" t="n"/>
+      <c r="K30" s="287" t="n"/>
+      <c r="L30" s="274" t="n"/>
     </row>
     <row r="31" ht="25" customHeight="1">
       <c r="A31" s="253" t="inlineStr">
@@ -2936,36 +2994,36 @@
           <t>효과 확인</t>
         </is>
       </c>
-      <c r="B31" s="248" t="n"/>
+      <c r="B31" s="280" t="n"/>
       <c r="C31" s="263" t="inlineStr">
         <is>
-          <t>09-10~09-14, 개선 조건에서 1,000건 확인·크랙 0건 (V-01).
-합의 기준 충족: EFFECTIVE / 품질 김OO 확인.</t>
-        </is>
-      </c>
-      <c r="D31" s="250" t="n"/>
-      <c r="E31" s="250" t="n"/>
-      <c r="F31" s="250" t="n"/>
-      <c r="G31" s="250" t="n"/>
-      <c r="H31" s="250" t="n"/>
-      <c r="I31" s="250" t="n"/>
-      <c r="J31" s="250" t="n"/>
-      <c r="K31" s="250" t="n"/>
-      <c r="L31" s="250" t="n"/>
+          <t>미검증. FINAL UNKNOWN이며 빈 히트맵은 PASS를 의미하지 않음.
+ALIGN 0.981은 정렬 지표이며 불량 확률이 아님.</t>
+        </is>
+      </c>
+      <c r="D31" s="286" t="n"/>
+      <c r="E31" s="286" t="n"/>
+      <c r="F31" s="286" t="n"/>
+      <c r="G31" s="286" t="n"/>
+      <c r="H31" s="286" t="n"/>
+      <c r="I31" s="286" t="n"/>
+      <c r="J31" s="286" t="n"/>
+      <c r="K31" s="286" t="n"/>
+      <c r="L31" s="272" t="n"/>
     </row>
     <row r="32" ht="25" customHeight="1">
-      <c r="A32" s="248" t="n"/>
-      <c r="B32" s="248" t="n"/>
-      <c r="C32" s="250" t="n"/>
-      <c r="D32" s="250" t="n"/>
-      <c r="E32" s="250" t="n"/>
-      <c r="F32" s="250" t="n"/>
-      <c r="G32" s="250" t="n"/>
-      <c r="H32" s="250" t="n"/>
-      <c r="I32" s="250" t="n"/>
-      <c r="J32" s="250" t="n"/>
-      <c r="K32" s="250" t="n"/>
-      <c r="L32" s="250" t="n"/>
+      <c r="A32" s="281" t="n"/>
+      <c r="B32" s="283" t="n"/>
+      <c r="C32" s="273" t="n"/>
+      <c r="D32" s="287" t="n"/>
+      <c r="E32" s="287" t="n"/>
+      <c r="F32" s="287" t="n"/>
+      <c r="G32" s="287" t="n"/>
+      <c r="H32" s="287" t="n"/>
+      <c r="I32" s="287" t="n"/>
+      <c r="J32" s="287" t="n"/>
+      <c r="K32" s="287" t="n"/>
+      <c r="L32" s="274" t="n"/>
     </row>
     <row r="33" ht="24" customHeight="1">
       <c r="A33" s="253" t="inlineStr">
@@ -2973,27 +3031,25 @@
           <t>확인자</t>
         </is>
       </c>
-      <c r="B33" s="248" t="n"/>
+      <c r="B33" s="271" t="n"/>
       <c r="C33" s="261" t="inlineStr">
         <is>
-          <t>품질 김OO</t>
-        </is>
-      </c>
-      <c r="D33" s="250" t="n"/>
-      <c r="E33" s="250" t="n"/>
-      <c r="F33" s="250" t="n"/>
+          <t>확인 대기</t>
+        </is>
+      </c>
+      <c r="D33" s="277" t="n"/>
+      <c r="E33" s="277" t="n"/>
+      <c r="F33" s="276" t="n"/>
       <c r="G33" s="253" t="inlineStr">
         <is>
           <t>종결일</t>
         </is>
       </c>
-      <c r="H33" s="248" t="n"/>
-      <c r="I33" s="269" t="n">
-        <v>46280</v>
-      </c>
-      <c r="J33" s="250" t="n"/>
-      <c r="K33" s="250" t="n"/>
-      <c r="L33" s="250" t="n"/>
+      <c r="H33" s="271" t="n"/>
+      <c r="I33" s="288" t="n"/>
+      <c r="J33" s="277" t="n"/>
+      <c r="K33" s="277" t="n"/>
+      <c r="L33" s="276" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="253" t="inlineStr">
@@ -3001,54 +3057,43 @@
           <t>종결 판정</t>
         </is>
       </c>
-      <c r="B34" s="248" t="n"/>
+      <c r="B34" s="280" t="n"/>
       <c r="C34" s="263" t="inlineStr">
         <is>
-          <t>09-10 공정 재개·09-14 출하 보류 해제 승인 완료. 격리품 처분: DISP-01.
-효과 확인 후 종결 / 보드 설계 변경 시 지지 조건 재확인.</t>
-        </is>
-      </c>
-      <c r="D34" s="250" t="n"/>
-      <c r="E34" s="250" t="n"/>
-      <c r="F34" s="250" t="n"/>
-      <c r="G34" s="250" t="n"/>
-      <c r="H34" s="250" t="n"/>
-      <c r="I34" s="250" t="n"/>
-      <c r="J34" s="250" t="n"/>
-      <c r="K34" s="250" t="n"/>
-      <c r="L34" s="250" t="n"/>
+          <t>미종결. 확정 판정·원인·조치·효과 검증 후 종결 여부 결정.
+본 샘플은 재개·출하 승인 근거로 사용할 수 없음.</t>
+        </is>
+      </c>
+      <c r="D34" s="286" t="n"/>
+      <c r="E34" s="286" t="n"/>
+      <c r="F34" s="286" t="n"/>
+      <c r="G34" s="286" t="n"/>
+      <c r="H34" s="286" t="n"/>
+      <c r="I34" s="286" t="n"/>
+      <c r="J34" s="286" t="n"/>
+      <c r="K34" s="286" t="n"/>
+      <c r="L34" s="272" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="248" t="n"/>
-      <c r="B35" s="248" t="n"/>
-      <c r="C35" s="250" t="n"/>
-      <c r="D35" s="250" t="n"/>
-      <c r="E35" s="250" t="n"/>
-      <c r="F35" s="250" t="n"/>
-      <c r="G35" s="250" t="n"/>
-      <c r="H35" s="250" t="n"/>
-      <c r="I35" s="250" t="n"/>
-      <c r="J35" s="250" t="n"/>
-      <c r="K35" s="250" t="n"/>
-      <c r="L35" s="250" t="n"/>
+      <c r="A35" s="281" t="n"/>
+      <c r="B35" s="283" t="n"/>
+      <c r="C35" s="273" t="n"/>
+      <c r="D35" s="287" t="n"/>
+      <c r="E35" s="287" t="n"/>
+      <c r="F35" s="287" t="n"/>
+      <c r="G35" s="287" t="n"/>
+      <c r="H35" s="287" t="n"/>
+      <c r="I35" s="287" t="n"/>
+      <c r="J35" s="287" t="n"/>
+      <c r="K35" s="287" t="n"/>
+      <c r="L35" s="274" t="n"/>
     </row>
     <row r="36" ht="16" customHeight="1">
       <c r="A36" s="270" t="inlineStr">
         <is>
-          <t>노란 칸: 담당자 작성 · 원인·조치·효과는 확인 후 기록 · 가상 예시</t>
-        </is>
-      </c>
-      <c r="B36" s="246" t="n"/>
-      <c r="C36" s="246" t="n"/>
-      <c r="D36" s="246" t="n"/>
-      <c r="E36" s="246" t="n"/>
-      <c r="F36" s="246" t="n"/>
-      <c r="G36" s="246" t="n"/>
-      <c r="H36" s="246" t="n"/>
-      <c r="I36" s="246" t="n"/>
-      <c r="J36" s="246" t="n"/>
-      <c r="K36" s="246" t="n"/>
-      <c r="L36" s="246" t="n"/>
+          <t>첨부 이미지 배치 예시 · 판정 미확정 · 자동 발행 / 종결 문서 아님</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
@@ -3065,8 +3110,8 @@
     <mergeCell ref="I10:L10"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="A17:B18"/>
+    <mergeCell ref="A1:H3"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A1:H3"/>
     <mergeCell ref="A15:F16"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="I9:L9"/>
@@ -3080,8 +3125,8 @@
     <mergeCell ref="A22:L22"/>
     <mergeCell ref="C33:F33"/>
     <mergeCell ref="C6:L6"/>
+    <mergeCell ref="C31:L32"/>
     <mergeCell ref="A27:B28"/>
-    <mergeCell ref="C31:L32"/>
     <mergeCell ref="A4:L4"/>
     <mergeCell ref="A34:B35"/>
     <mergeCell ref="C17:F18"/>
@@ -3124,11 +3169,224 @@
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.32" right="0.32" top="0.3" bottom="0.3" header="0.1" footer="0.1"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001F3864"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:L26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" s="295" t="inlineStr">
+        <is>
+          <t>검사 근거 · 원본 진단 화면</t>
+        </is>
+      </c>
+      <c r="B1" s="54" t="n"/>
+      <c r="C1" s="54" t="n"/>
+      <c r="D1" s="54" t="n"/>
+      <c r="E1" s="54" t="n"/>
+      <c r="F1" s="54" t="n"/>
+      <c r="G1" s="54" t="n"/>
+      <c r="H1" s="54" t="n"/>
+      <c r="I1" s="54" t="n"/>
+      <c r="J1" s="54" t="n"/>
+      <c r="K1" s="54" t="n"/>
+      <c r="L1" s="54" t="n"/>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="54" t="n"/>
+      <c r="B2" s="54" t="n"/>
+      <c r="C2" s="54" t="n"/>
+      <c r="D2" s="54" t="n"/>
+      <c r="E2" s="54" t="n"/>
+      <c r="F2" s="54" t="n"/>
+      <c r="G2" s="54" t="n"/>
+      <c r="H2" s="54" t="n"/>
+      <c r="I2" s="54" t="n"/>
+      <c r="J2" s="54" t="n"/>
+      <c r="K2" s="54" t="n"/>
+      <c r="L2" s="54" t="n"/>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="296" t="inlineStr">
+        <is>
+          <t>판정 미확정 | FINAL UNKNOWN · ADVISORY CANDIDATES 1 · UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="B3" s="87" t="n"/>
+      <c r="C3" s="87" t="n"/>
+      <c r="D3" s="87" t="n"/>
+      <c r="E3" s="87" t="n"/>
+      <c r="F3" s="87" t="n"/>
+      <c r="G3" s="87" t="n"/>
+      <c r="H3" s="87" t="n"/>
+      <c r="I3" s="87" t="n"/>
+      <c r="J3" s="87" t="n"/>
+      <c r="K3" s="87" t="n"/>
+      <c r="L3" s="87" t="n"/>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="297" t="inlineStr">
+        <is>
+          <t>표시 위치: smd_capacitor_01 (POSITION?) · 의심 후보이며 확정 불량이 아닙니다.</t>
+        </is>
+      </c>
+      <c r="B4" s="246" t="n"/>
+      <c r="C4" s="246" t="n"/>
+      <c r="D4" s="246" t="n"/>
+      <c r="E4" s="246" t="n"/>
+      <c r="F4" s="246" t="n"/>
+      <c r="G4" s="246" t="n"/>
+      <c r="H4" s="246" t="n"/>
+      <c r="I4" s="246" t="n"/>
+      <c r="J4" s="246" t="n"/>
+      <c r="K4" s="246" t="n"/>
+      <c r="L4" s="246" t="n"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="298" t="inlineStr">
+        <is>
+          <t>전체 원본 · 원본 / 후보 히트맵 / 오버레이 · 비율 유지</t>
+        </is>
+      </c>
+      <c r="B5" s="299" t="n"/>
+      <c r="C5" s="299" t="n"/>
+      <c r="D5" s="299" t="n"/>
+      <c r="E5" s="299" t="n"/>
+      <c r="F5" s="299" t="n"/>
+      <c r="G5" s="299" t="n"/>
+      <c r="H5" s="299" t="n"/>
+      <c r="I5" s="299" t="n"/>
+      <c r="J5" s="299" t="n"/>
+      <c r="K5" s="299" t="n"/>
+      <c r="L5" s="299" t="n"/>
+    </row>
+    <row r="6" ht="18" customHeight="1"/>
+    <row r="7" ht="18" customHeight="1"/>
+    <row r="8" ht="18" customHeight="1"/>
+    <row r="9" ht="18" customHeight="1"/>
+    <row r="10" ht="18" customHeight="1"/>
+    <row r="11" ht="18" customHeight="1"/>
+    <row r="12" ht="18" customHeight="1"/>
+    <row r="13" ht="18" customHeight="1"/>
+    <row r="14" ht="18" customHeight="1"/>
+    <row r="15" ht="18" customHeight="1"/>
+    <row r="16" ht="18" customHeight="1"/>
+    <row r="17" ht="18" customHeight="1"/>
+    <row r="18" ht="18" customHeight="1"/>
+    <row r="19" ht="18" customHeight="1"/>
+    <row r="20" ht="18" customHeight="1"/>
+    <row r="21" ht="18" customHeight="1"/>
+    <row r="22" ht="18" customHeight="1"/>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="300" t="inlineStr">
+        <is>
+          <t>미표시 보조 pose 플래그 4개 · 검사 불가 항목 13개 · 빈 히트맵이나 후보 없음은 PASS를 뜻하지 않습니다.</t>
+        </is>
+      </c>
+      <c r="B23" s="87" t="n"/>
+      <c r="C23" s="87" t="n"/>
+      <c r="D23" s="87" t="n"/>
+      <c r="E23" s="87" t="n"/>
+      <c r="F23" s="87" t="n"/>
+      <c r="G23" s="87" t="n"/>
+      <c r="H23" s="87" t="n"/>
+      <c r="I23" s="87" t="n"/>
+      <c r="J23" s="87" t="n"/>
+      <c r="K23" s="87" t="n"/>
+      <c r="L23" s="87" t="n"/>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="301" t="inlineStr">
+        <is>
+          <t>ALIGN 0.981은 정렬 지표입니다. 실제 판정과 원인 확인에는 상세 검사 결과·실물 확인이 필요합니다.</t>
+        </is>
+      </c>
+      <c r="B24" s="246" t="n"/>
+      <c r="C24" s="246" t="n"/>
+      <c r="D24" s="246" t="n"/>
+      <c r="E24" s="246" t="n"/>
+      <c r="F24" s="246" t="n"/>
+      <c r="G24" s="246" t="n"/>
+      <c r="H24" s="246" t="n"/>
+      <c r="I24" s="246" t="n"/>
+      <c r="J24" s="246" t="n"/>
+      <c r="K24" s="246" t="n"/>
+      <c r="L24" s="246" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="302" t="inlineStr">
+        <is>
+          <t>원본: inspection_1e2f3eab-3d28-4e4b-859b-2ff37b5676f7_02_annotated_report.png
+SHA-256: db24b2e4f61367ef5e4ac5397bff03b3e9559d329a346f57db6834360f42f0df</t>
+        </is>
+      </c>
+      <c r="B25" s="246" t="n"/>
+      <c r="C25" s="246" t="n"/>
+      <c r="D25" s="246" t="n"/>
+      <c r="E25" s="246" t="n"/>
+      <c r="F25" s="246" t="n"/>
+      <c r="G25" s="246" t="n"/>
+      <c r="H25" s="246" t="n"/>
+      <c r="I25" s="246" t="n"/>
+      <c r="J25" s="246" t="n"/>
+      <c r="K25" s="246" t="n"/>
+      <c r="L25" s="246" t="n"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="246" t="n"/>
+      <c r="B26" s="246" t="n"/>
+      <c r="C26" s="246" t="n"/>
+      <c r="D26" s="246" t="n"/>
+      <c r="E26" s="246" t="n"/>
+      <c r="F26" s="246" t="n"/>
+      <c r="G26" s="246" t="n"/>
+      <c r="H26" s="246" t="n"/>
+      <c r="I26" s="246" t="n"/>
+      <c r="J26" s="246" t="n"/>
+      <c r="K26" s="246" t="n"/>
+      <c r="L26" s="246" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A24:L24"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A23:L23"/>
+    <mergeCell ref="A1:L2"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A25:L26"/>
+    <mergeCell ref="A4:L4"/>
+  </mergeCells>
+  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3148,14 +3406,14 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>현재 부품과 대체품 후보 · 가상 부품 검토 예시</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
+          <t>대체품 후보 · 기존 가상 MLCC 비교 예시</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" s="289" t="inlineStr">
         <is>
-          <t>현재 부품: CAP / Contoso CX-0603X7R104K100 / MLCC · 데이터시트 대조: 일치</t>
+          <t>아래 목록은 기존 가상 부품 예시입니다. 첨부 이미지의 smd_capacitor_01과 모델명·정격 대응은 미확인입니다.</t>
         </is>
       </c>
     </row>
@@ -3223,7 +3481,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="290" t="inlineStr">
         <is>
@@ -3320,7 +3577,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="293" t="inlineStr">
         <is>

</xml_diff>